<commit_message>
move snapshot timestamp to footer
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-06-30 12:41:19</t>
+          <t>Timestamp: 2026-06-30 12:58:07</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>725</v>
+        <v>775</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>596</v>
+        <v>646</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>598</v>
+        <v>638</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>533</v>
+        <v>558</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>494</v>
+        <v>519</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>686</v>
+        <v>736</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>632</v>
+        <v>682</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>574</v>
+        <v>609</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>508</v>
+        <v>533</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>460</v>
+        <v>510</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>459</v>
+        <v>509</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>321</v>
+        <v>361</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>360</v>
+        <v>385</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>275</v>
+        <v>300</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>419</v>
+        <v>444</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>287</v>
+        <v>337</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>281</v>
+        <v>331</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
rename tab title to [Reps]
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-06-30 12:58:07</t>
+          <t>Timestamp: 2026-06-30 13:32:30</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>138</v>
+        <v>213</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>210</v>
+        <v>285</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>775</v>
+        <v>800</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>646</v>
+        <v>671</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>638</v>
+        <v>663</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>558</v>
+        <v>583</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>519</v>
+        <v>544</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>736</v>
+        <v>761</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>682</v>
+        <v>707</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>609</v>
+        <v>634</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>533</v>
+        <v>558</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -888,7 +888,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>510</v>
+        <v>535</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>509</v>
+        <v>534</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>361</v>
+        <v>386</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>385</v>
+        <v>410</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>300</v>
+        <v>325</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>444</v>
+        <v>469</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>86</v>
+        <v>161</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>86</v>
+        <v>157</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>261</v>
+        <v>336</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
deploy: daily snapshot 2026-07-01 13:08
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-06-30" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-07-01" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1233,4 +1234,868 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-01 13:08:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mery</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GON</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>263</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>338</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>919</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+448</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Eucresia X</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>285</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2245</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1295</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2103</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1282</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1978</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1165</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1805</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1699</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>2216</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1305</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>2120</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1263</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1939</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1155</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1785</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1077</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1965</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1280</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1943</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1259</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1697</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1161</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1589</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1035</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1447</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>466</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+15</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1649</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1030</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>666</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+425</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>716</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+405</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+903</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Meteorx</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>704</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+397</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>950</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+464</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>890</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+528</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>971</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+615</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-01 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -1260,7 +1260,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-01 13:13:52</t>
+          <t>Timestamp: 2026-07-01 13:31:00</t>
         </is>
       </c>
     </row>
@@ -1453,11 +1453,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>2245</v>
+        <v>2270</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1295</t>
+          <t>+1320</t>
         </is>
       </c>
     </row>
@@ -1543,11 +1543,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>2103</v>
+        <v>2128</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1282</t>
+          <t>+1307</t>
         </is>
       </c>
     </row>
@@ -1558,11 +1558,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1978</v>
+        <v>2003</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1165</t>
+          <t>+1190</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1805</v>
+        <v>1830</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1699</v>
+        <v>1724</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
@@ -1603,11 +1603,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>2216</v>
+        <v>2241</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1305</t>
+          <t>+1330</t>
         </is>
       </c>
     </row>
@@ -1618,11 +1618,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2120</v>
+        <v>2145</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1263</t>
+          <t>+1288</t>
         </is>
       </c>
     </row>
@@ -1633,11 +1633,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1939</v>
+        <v>1964</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1155</t>
+          <t>+1180</t>
         </is>
       </c>
     </row>
@@ -1648,11 +1648,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1785</v>
+        <v>1810</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1077</t>
+          <t>+1102</t>
         </is>
       </c>
     </row>
@@ -1678,11 +1678,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1965</v>
+        <v>1990</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1305</t>
         </is>
       </c>
     </row>
@@ -1693,11 +1693,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1943</v>
+        <v>1968</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1259</t>
+          <t>+1284</t>
         </is>
       </c>
     </row>
@@ -1708,11 +1708,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1697</v>
+        <v>1722</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1161</t>
+          <t>+1186</t>
         </is>
       </c>
     </row>
@@ -1723,11 +1723,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1589</v>
+        <v>1614</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1035</t>
+          <t>+1060</t>
         </is>
       </c>
     </row>
@@ -1738,11 +1738,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>1447</v>
+        <v>1472</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+1005</t>
         </is>
       </c>
     </row>
@@ -1828,11 +1828,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>1649</v>
+        <v>1674</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1030</t>
+          <t>+1055</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: embed server hourly cache as __hourlyCache, use as JS fallback for accurate live diffs
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -1260,7 +1260,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-01 13:13:52</t>
+          <t>Timestamp: 2026-07-01 13:51:02</t>
         </is>
       </c>
     </row>
@@ -1453,11 +1453,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>2245</v>
+        <v>2295</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1295</t>
+          <t>+1345</t>
         </is>
       </c>
     </row>
@@ -1543,11 +1543,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>2103</v>
+        <v>2153</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1282</t>
+          <t>+1332</t>
         </is>
       </c>
     </row>
@@ -1558,11 +1558,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1978</v>
+        <v>2023</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1165</t>
+          <t>+1210</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1805</v>
+        <v>1830</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1699</v>
+        <v>1724</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
@@ -1603,11 +1603,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>2216</v>
+        <v>2266</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1305</t>
+          <t>+1355</t>
         </is>
       </c>
     </row>
@@ -1618,11 +1618,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2120</v>
+        <v>2170</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1263</t>
+          <t>+1313</t>
         </is>
       </c>
     </row>
@@ -1633,11 +1633,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1939</v>
+        <v>1984</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1155</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -1648,11 +1648,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1785</v>
+        <v>1810</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1077</t>
+          <t>+1102</t>
         </is>
       </c>
     </row>
@@ -1678,11 +1678,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1965</v>
+        <v>2015</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1280</t>
+          <t>+1330</t>
         </is>
       </c>
     </row>
@@ -1693,11 +1693,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1943</v>
+        <v>1993</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1259</t>
+          <t>+1309</t>
         </is>
       </c>
     </row>
@@ -1708,11 +1708,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1697</v>
+        <v>1732</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1161</t>
+          <t>+1196</t>
         </is>
       </c>
     </row>
@@ -1723,11 +1723,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1589</v>
+        <v>1614</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1035</t>
+          <t>+1060</t>
         </is>
       </c>
     </row>
@@ -1738,11 +1738,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>1447</v>
+        <v>1472</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+1005</t>
         </is>
       </c>
     </row>
@@ -1828,11 +1828,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>1649</v>
+        <v>1674</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1030</t>
+          <t>+1055</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-02 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-06-30" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-01" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-07-02" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2098,4 +2099,868 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-02 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mery</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GON</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>263</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>338</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1069</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Eucresia X</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>285</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>3145</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>3003</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2878</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2705</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2599</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3116</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3020</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2839</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>2685</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>2865</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2843</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2597</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2489</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2347</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>466</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2549</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>666</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>716</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1053</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1053</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Meteorx</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>704</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>1121</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+1121</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>1225</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>997</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+972</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>1025</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>1125</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>1125</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>1540</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>1601</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-02 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -2107,7 +2107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2125,7 +2125,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-02 13:01:00</t>
+          <t>Timestamp: 2026-07-02 13:31:00</t>
         </is>
       </c>
     </row>
@@ -2243,11 +2243,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1069</v>
+        <v>1094</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+175</t>
         </is>
       </c>
     </row>
@@ -2303,11 +2303,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>500</v>
+        <v>521</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+500</t>
+          <t>+521</t>
         </is>
       </c>
     </row>
@@ -2734,26 +2734,26 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Player</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>666</v>
+        <v>1078</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+1078</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Meteorx</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>716</v>
+        <v>0</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
@@ -2768,33 +2768,33 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>1053</v>
+        <v>0</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1053</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Meteorx</t>
+          <t>yatoro</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>0</v>
+        <v>1161</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+1161</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>Ryugai</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
@@ -2809,150 +2809,105 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>PuNch</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>704</v>
+        <v>1250</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>yatoro</t>
+          <t>§hitnobi</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>1121</v>
+        <v>1057</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+1121</t>
+          <t>+1032</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Ryugai</t>
+          <t>§hitnobi</t>
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>0</v>
+        <v>1071</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+1046</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>PuNch</t>
+          <t>KOPZ2</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>1225</v>
+        <v>1129</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+275</t>
+          <t>+1129</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>§hitnobi</t>
+          <t>COPZ1</t>
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>997</v>
+        <v>1235</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+972</t>
+          <t>+1235</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>§hitnobi</t>
+          <t>Ryzeee</t>
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>1025</v>
+        <v>1590</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>KOPZ2</t>
+          <t>Aluphiee</t>
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>1125</v>
+        <v>1651</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1125</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>COPZ1</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="n">
-        <v>1125</v>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>+1125</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>Ryzeee</t>
-        </is>
-      </c>
-      <c r="B56" s="5" t="n">
-        <v>1540</v>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>+650</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Aluphiee</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="n">
-        <v>1601</v>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>+630</t>
+          <t>+680</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-03 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -10,6 +10,7 @@
     <sheet name="2026-06-30" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-07-01" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-02" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-07-03" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2918,4 +2919,868 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-03 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>gokito</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Mery</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>225</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>GON</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>263</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>439</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+389</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>385</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+47</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2322</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1228</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>396</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+96</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Eucresia X</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>285</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1581</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>4025</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3883</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3750</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+872</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3585</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3504</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+905</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>4166</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>3811</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+972</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>3615</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+55</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>3790</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>3773</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>3477</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3339</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>3172</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>466</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>288</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+88</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>3479</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2319</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+2319</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>2292</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1131</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2474</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1224</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>395</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-676</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-721</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>350</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>-721</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2132</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1061</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2146</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>2234</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1105</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>2275</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1040</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>2456</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+866</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>2581</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-03 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -2945,7 +2945,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-03 13:01:00</t>
+          <t>Timestamp: 2026-07-03 13:31:00</t>
         </is>
       </c>
     </row>
@@ -3003,11 +3003,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>225</v>
+        <v>300</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+75</t>
         </is>
       </c>
     </row>
@@ -3018,11 +3018,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>550</v>
+        <v>575</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -3138,11 +3138,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1581</v>
+        <v>1681</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1060</t>
+          <t>+1160</t>
         </is>
       </c>
     </row>
@@ -3153,11 +3153,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>4025</v>
+        <v>4050</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -3243,11 +3243,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>3883</v>
+        <v>3908</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -3258,11 +3258,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3750</v>
+        <v>3775</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+872</t>
+          <t>+897</t>
         </is>
       </c>
     </row>
@@ -3273,11 +3273,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>3585</v>
+        <v>3610</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -3288,11 +3288,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>3504</v>
+        <v>3529</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+905</t>
+          <t>+930</t>
         </is>
       </c>
     </row>
@@ -3303,11 +3303,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>4166</v>
+        <v>4191</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1075</t>
         </is>
       </c>
     </row>
@@ -3318,11 +3318,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>4000</v>
+        <v>4025</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+1005</t>
         </is>
       </c>
     </row>
@@ -3333,11 +3333,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>3811</v>
+        <v>3836</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+972</t>
+          <t>+997</t>
         </is>
       </c>
     </row>
@@ -3348,11 +3348,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>3615</v>
+        <v>3640</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+955</t>
         </is>
       </c>
     </row>
@@ -3378,11 +3378,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>3790</v>
+        <v>3815</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -3393,11 +3393,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>3773</v>
+        <v>3798</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+955</t>
         </is>
       </c>
     </row>
@@ -3408,11 +3408,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>3477</v>
+        <v>3502</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+905</t>
         </is>
       </c>
     </row>
@@ -3423,11 +3423,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3339</v>
+        <v>3364</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -3438,11 +3438,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>3172</v>
+        <v>3197</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+850</t>
         </is>
       </c>
     </row>
@@ -3528,11 +3528,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3479</v>
+        <v>3504</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+955</t>
         </is>
       </c>
     </row>
@@ -3543,11 +3543,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+75</t>
         </is>
       </c>
     </row>
@@ -3558,11 +3558,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+75</t>
         </is>
       </c>
     </row>
@@ -3573,11 +3573,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>2319</v>
+        <v>2339</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+2319</t>
+          <t>+2339</t>
         </is>
       </c>
     </row>
@@ -3603,11 +3603,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>2292</v>
+        <v>2367</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+1131</t>
+          <t>+1206</t>
         </is>
       </c>
     </row>
@@ -3633,11 +3633,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>2474</v>
+        <v>2499</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+1224</t>
+          <t>+1249</t>
         </is>
       </c>
     </row>
@@ -3723,11 +3723,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>2234</v>
+        <v>2309</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1105</t>
+          <t>+1180</t>
         </is>
       </c>
     </row>
@@ -3738,11 +3738,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>2275</v>
+        <v>2350</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+1040</t>
+          <t>+1115</t>
         </is>
       </c>
     </row>
@@ -3753,11 +3753,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>2456</v>
+        <v>2481</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+866</t>
+          <t>+891</t>
         </is>
       </c>
     </row>
@@ -3768,11 +3768,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>2581</v>
+        <v>2602</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+951</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-04 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -11,6 +11,7 @@
     <sheet name="2026-07-01" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-07-02" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-03" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-07-04" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -3783,4 +3784,868 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-04 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>gokito</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>779</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>705</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+130</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>GON</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>284</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+21</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>573</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+134</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>492</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+96</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Eucresia X</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>306</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2175</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+494</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>5143</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1093</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>4981</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1073</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>4810</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1035</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>4621</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1011</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>4470</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+941</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5164</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+973</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>4992</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+967</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>4769</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+933</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>4516</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+876</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>479</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+424</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>4956</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1141</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>4919</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1121</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>4599</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1097</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>4421</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1057</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>4172</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+975</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>519</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+53</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>288</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>4310</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+806</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>461</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+386</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>386</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+311</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+2815</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>2948</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+581</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>3294</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+795</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>982</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1164</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>937</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1209</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>901</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>-1245</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2670</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+524</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2683</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+537</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>2877</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>2954</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+604</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>2893</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+412</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3024</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+422</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-04 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -3810,7 +3810,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-04 13:01:00</t>
+          <t>Timestamp: 2026-07-04 13:31:00</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>779</v>
+        <v>813</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -3928,11 +3928,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>805</v>
+        <v>875</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+420</t>
+          <t>+490</t>
         </is>
       </c>
     </row>
@@ -4018,11 +4018,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>5143</v>
+        <v>5181</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1093</t>
+          <t>+1131</t>
         </is>
       </c>
     </row>
@@ -4108,11 +4108,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>4981</v>
+        <v>5011</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1073</t>
+          <t>+1103</t>
         </is>
       </c>
     </row>
@@ -4123,11 +4123,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>4810</v>
+        <v>4840</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1035</t>
+          <t>+1065</t>
         </is>
       </c>
     </row>
@@ -4138,11 +4138,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>4621</v>
+        <v>4651</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1011</t>
+          <t>+1041</t>
         </is>
       </c>
     </row>
@@ -4153,11 +4153,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>4470</v>
+        <v>4500</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+941</t>
+          <t>+971</t>
         </is>
       </c>
     </row>
@@ -4168,11 +4168,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>5164</v>
+        <v>5198</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+973</t>
+          <t>+1007</t>
         </is>
       </c>
     </row>
@@ -4183,11 +4183,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>4992</v>
+        <v>5022</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+967</t>
+          <t>+997</t>
         </is>
       </c>
     </row>
@@ -4198,11 +4198,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>4769</v>
+        <v>4799</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+933</t>
+          <t>+963</t>
         </is>
       </c>
     </row>
@@ -4213,11 +4213,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>4516</v>
+        <v>4546</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+876</t>
+          <t>+906</t>
         </is>
       </c>
     </row>
@@ -4243,11 +4243,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>4956</v>
+        <v>4990</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1141</t>
+          <t>+1175</t>
         </is>
       </c>
     </row>
@@ -4258,11 +4258,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>4919</v>
+        <v>4949</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1121</t>
+          <t>+1151</t>
         </is>
       </c>
     </row>
@@ -4273,11 +4273,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>4599</v>
+        <v>4629</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1097</t>
+          <t>+1127</t>
         </is>
       </c>
     </row>
@@ -4288,11 +4288,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>4421</v>
+        <v>4451</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1057</t>
+          <t>+1087</t>
         </is>
       </c>
     </row>
@@ -4303,11 +4303,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>4172</v>
+        <v>4202</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+975</t>
+          <t>+1005</t>
         </is>
       </c>
     </row>
@@ -4393,11 +4393,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>4310</v>
+        <v>4340</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+806</t>
+          <t>+836</t>
         </is>
       </c>
     </row>
@@ -4468,11 +4468,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>2948</v>
+        <v>3002</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+581</t>
+          <t>+635</t>
         </is>
       </c>
     </row>
@@ -4513,11 +4513,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>982</v>
+        <v>1024</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>-1164</t>
+          <t>-1122</t>
         </is>
       </c>
     </row>
@@ -4528,11 +4528,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>937</v>
+        <v>979</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>-1209</t>
+          <t>-1167</t>
         </is>
       </c>
     </row>
@@ -4543,11 +4543,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>901</v>
+        <v>943</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>-1245</t>
+          <t>-1203</t>
         </is>
       </c>
     </row>
@@ -4558,11 +4558,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>2670</v>
+        <v>2712</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+524</t>
+          <t>+566</t>
         </is>
       </c>
     </row>
@@ -4573,11 +4573,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>2683</v>
+        <v>2725</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+537</t>
+          <t>+579</t>
         </is>
       </c>
     </row>
@@ -4588,11 +4588,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>2877</v>
+        <v>2923</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+568</t>
+          <t>+614</t>
         </is>
       </c>
     </row>
@@ -4603,11 +4603,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>2954</v>
+        <v>3020</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+604</t>
+          <t>+670</t>
         </is>
       </c>
     </row>
@@ -4618,11 +4618,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>2893</v>
+        <v>2923</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+412</t>
+          <t>+442</t>
         </is>
       </c>
     </row>
@@ -4633,11 +4633,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>3024</v>
+        <v>3074</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+422</t>
+          <t>+472</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-05 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -12,6 +12,7 @@
     <sheet name="2026-07-02" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-07-03" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-04" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-07-05" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -4648,4 +4649,868 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-05 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>gokito</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2292</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1479</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>705</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>453</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>573</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2565</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1690</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>574</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+82</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>405</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2820</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+645</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7391</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+2210</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>7083</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2072</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>6648</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1808</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>6195</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1544</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>5878</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1378</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7496</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2298</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>7196</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+2174</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>6733</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1934</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>6208</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1662</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>479</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7280</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+2290</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>7025</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+2076</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>6433</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1804</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>6011</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1560</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>5638</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1436</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1095</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+576</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>288</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>5830</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1490</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>461</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>386</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+2798</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>544</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+527</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>4123</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1121</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>4073</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+779</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>1530</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1195</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>1503</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>1467</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>-1258</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>3260</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+535</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>3272</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+547</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>4081</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1158</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>3987</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+967</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>3702</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+779</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>3904</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+830</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-05 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -4675,7 +4675,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-05 13:01:00</t>
+          <t>Timestamp: 2026-07-05 13:31:00</t>
         </is>
       </c>
     </row>
@@ -4868,11 +4868,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>2820</v>
+        <v>2850</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+645</t>
+          <t>+675</t>
         </is>
       </c>
     </row>
@@ -4883,11 +4883,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>7391</v>
+        <v>7429</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2210</t>
+          <t>+2248</t>
         </is>
       </c>
     </row>
@@ -4973,11 +4973,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>7083</v>
+        <v>7113</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2072</t>
+          <t>+2102</t>
         </is>
       </c>
     </row>
@@ -4988,11 +4988,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>6648</v>
+        <v>6678</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1808</t>
+          <t>+1838</t>
         </is>
       </c>
     </row>
@@ -5003,11 +5003,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>6195</v>
+        <v>6225</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1544</t>
+          <t>+1574</t>
         </is>
       </c>
     </row>
@@ -5018,11 +5018,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>5878</v>
+        <v>5908</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1378</t>
+          <t>+1408</t>
         </is>
       </c>
     </row>
@@ -5033,11 +5033,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>7496</v>
+        <v>7530</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2298</t>
+          <t>+2332</t>
         </is>
       </c>
     </row>
@@ -5048,11 +5048,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>7196</v>
+        <v>7226</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2174</t>
+          <t>+2204</t>
         </is>
       </c>
     </row>
@@ -5063,11 +5063,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>6733</v>
+        <v>6763</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1934</t>
+          <t>+1964</t>
         </is>
       </c>
     </row>
@@ -5078,11 +5078,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>6208</v>
+        <v>6238</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+1662</t>
+          <t>+1692</t>
         </is>
       </c>
     </row>
@@ -5258,11 +5258,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>5830</v>
+        <v>5860</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1490</t>
+          <t>+1520</t>
         </is>
       </c>
     </row>
@@ -5333,11 +5333,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>4123</v>
+        <v>4165</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+1121</t>
+          <t>+1163</t>
         </is>
       </c>
     </row>
@@ -5453,11 +5453,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>4081</v>
+        <v>4165</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1158</t>
+          <t>+1242</t>
         </is>
       </c>
     </row>
@@ -5468,11 +5468,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>3987</v>
+        <v>4059</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+967</t>
+          <t>+1039</t>
         </is>
       </c>
     </row>
@@ -5483,11 +5483,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>3702</v>
+        <v>3762</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+779</t>
+          <t>+839</t>
         </is>
       </c>
     </row>
@@ -5498,11 +5498,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>3904</v>
+        <v>3959</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+830</t>
+          <t>+885</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-06 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -13,6 +13,7 @@
     <sheet name="2026-07-03" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-07-04" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-05" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-07-06" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -5513,4 +5514,853 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-06 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>2550</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+258</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>855</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>526</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+73</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>623</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>3459</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+894</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>574</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>482</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+77</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3624</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+774</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>9565</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+2136</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>9072</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1959</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8492</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1814</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>7829</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1604</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>7430</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1522</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>9460</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1930</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>8970</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1744</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8339</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1576</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7680</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1442</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>479</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9099</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1819</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8739</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1714</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8029</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1596</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>7473</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1462</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>6965</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1327</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1422</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+327</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>393</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+105</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>7165</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1305</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>461</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>386</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+2271</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>886</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+342</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>5342</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1177</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>4298</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+225</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2352</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-920</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2305</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-967</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2304</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-968</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>4026</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+754</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>3983</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+711</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>5281</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1116</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>5225</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1166</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>4396</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+634</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4560</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+601</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-06 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -5540,7 +5540,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-06 13:01:00</t>
+          <t>Timestamp: 2026-07-06 13:31:00</t>
         </is>
       </c>
     </row>
@@ -5598,11 +5598,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+150</t>
+          <t>+155</t>
         </is>
       </c>
     </row>
@@ -5628,11 +5628,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>623</v>
+        <v>630</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+50</t>
+          <t>+57</t>
         </is>
       </c>
     </row>
@@ -5733,11 +5733,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>9565</v>
+        <v>9590</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2136</t>
+          <t>+2161</t>
         </is>
       </c>
     </row>
@@ -5823,11 +5823,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>9072</v>
+        <v>9095</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1959</t>
+          <t>+1982</t>
         </is>
       </c>
     </row>
@@ -5838,11 +5838,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>8492</v>
+        <v>8507</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1814</t>
+          <t>+1829</t>
         </is>
       </c>
     </row>
@@ -5853,11 +5853,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>7829</v>
+        <v>7844</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1604</t>
+          <t>+1619</t>
         </is>
       </c>
     </row>
@@ -5868,11 +5868,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>7430</v>
+        <v>7445</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1522</t>
+          <t>+1537</t>
         </is>
       </c>
     </row>
@@ -5883,11 +5883,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>9460</v>
+        <v>9485</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1930</t>
+          <t>+1955</t>
         </is>
       </c>
     </row>
@@ -5898,11 +5898,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>8970</v>
+        <v>8995</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1744</t>
+          <t>+1769</t>
         </is>
       </c>
     </row>
@@ -5913,11 +5913,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>8339</v>
+        <v>8356</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1576</t>
+          <t>+1593</t>
         </is>
       </c>
     </row>
@@ -5928,11 +5928,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>7680</v>
+        <v>7695</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1442</t>
+          <t>+1457</t>
         </is>
       </c>
     </row>
@@ -5958,11 +5958,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>9099</v>
+        <v>9124</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1819</t>
+          <t>+1844</t>
         </is>
       </c>
     </row>
@@ -5973,11 +5973,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>8739</v>
+        <v>8762</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1714</t>
+          <t>+1737</t>
         </is>
       </c>
     </row>
@@ -5988,11 +5988,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>8029</v>
+        <v>8046</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1596</t>
+          <t>+1613</t>
         </is>
       </c>
     </row>
@@ -6003,11 +6003,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>7473</v>
+        <v>7488</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1462</t>
+          <t>+1477</t>
         </is>
       </c>
     </row>
@@ -6018,11 +6018,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>6965</v>
+        <v>6980</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1327</t>
+          <t>+1342</t>
         </is>
       </c>
     </row>
@@ -6108,11 +6108,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>7165</v>
+        <v>7180</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1305</t>
+          <t>+1320</t>
         </is>
       </c>
     </row>
@@ -6183,11 +6183,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>5342</v>
+        <v>5343</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1177</t>
+          <t>+1178</t>
         </is>
       </c>
     </row>
@@ -6333,11 +6333,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>4396</v>
+        <v>4401</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+634</t>
+          <t>+639</t>
         </is>
       </c>
     </row>
@@ -6348,11 +6348,11 @@
         </is>
       </c>
       <c r="B56" s="5" t="n">
-        <v>4560</v>
+        <v>4565</v>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>+601</t>
+          <t>+606</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-07 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -14,6 +14,7 @@
     <sheet name="2026-07-04" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-07-05" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-07-06" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-07-07" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -6363,4 +6364,853 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-07 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>2863</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+313</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1653</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+793</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>861</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+335</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1427</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+797</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>3768</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+309</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>599</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>792</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+310</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4171</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+547</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>10739</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1149</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>10200</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1105</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9566</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1059</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8799</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+955</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8284</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+839</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>10630</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1145</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>10102</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1107</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>9423</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1067</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8648</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+953</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>695</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+216</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>10254</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1130</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>9811</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1049</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9084</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1038</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8433</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+945</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>7797</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+817</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1528</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+106</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>393</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>8041</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+861</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>663</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+202</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>525</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+139</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1929</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>972</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+86</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>5901</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+558</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>4551</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+253</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2769</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-1214</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>2724</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1259</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2713</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1270</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>4439</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+456</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>4419</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+436</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>5837</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+556</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>5863</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+638</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>4818</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+417</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4980</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+415</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
auto: snapshot 2026-07-07 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -6390,7 +6390,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-07 13:01:00</t>
+          <t>Timestamp: 2026-07-07 13:31:00</t>
         </is>
       </c>
     </row>
@@ -6433,11 +6433,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2863</v>
+        <v>2888</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+313</t>
+          <t>+338</t>
         </is>
       </c>
     </row>
@@ -6448,11 +6448,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1653</v>
+        <v>1678</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+793</t>
+          <t>+818</t>
         </is>
       </c>
     </row>
@@ -6463,11 +6463,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>861</v>
+        <v>886</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+335</t>
+          <t>+360</t>
         </is>
       </c>
     </row>
@@ -6478,11 +6478,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1427</v>
+        <v>1452</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+797</t>
+          <t>+822</t>
         </is>
       </c>
     </row>
@@ -6493,11 +6493,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>3768</v>
+        <v>3818</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+309</t>
+          <t>+359</t>
         </is>
       </c>
     </row>
@@ -6538,11 +6538,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>792</v>
+        <v>812</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+310</t>
+          <t>+330</t>
         </is>
       </c>
     </row>
@@ -6583,11 +6583,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>10739</v>
+        <v>10764</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1149</t>
+          <t>+1174</t>
         </is>
       </c>
     </row>
@@ -6673,11 +6673,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>10200</v>
+        <v>10225</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1105</t>
+          <t>+1130</t>
         </is>
       </c>
     </row>
@@ -6688,11 +6688,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>9566</v>
+        <v>9587</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1059</t>
+          <t>+1080</t>
         </is>
       </c>
     </row>
@@ -6703,11 +6703,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>8799</v>
+        <v>8814</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+955</t>
+          <t>+970</t>
         </is>
       </c>
     </row>
@@ -6718,11 +6718,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>8284</v>
+        <v>8299</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+839</t>
+          <t>+854</t>
         </is>
       </c>
     </row>
@@ -6733,11 +6733,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>10630</v>
+        <v>10655</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1145</t>
+          <t>+1170</t>
         </is>
       </c>
     </row>
@@ -6748,11 +6748,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>10102</v>
+        <v>10127</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1107</t>
+          <t>+1132</t>
         </is>
       </c>
     </row>
@@ -6763,11 +6763,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>9423</v>
+        <v>9446</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1067</t>
+          <t>+1090</t>
         </is>
       </c>
     </row>
@@ -6778,11 +6778,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>8648</v>
+        <v>8663</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+953</t>
+          <t>+968</t>
         </is>
       </c>
     </row>
@@ -6793,11 +6793,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>695</v>
+        <v>745</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+216</t>
+          <t>+266</t>
         </is>
       </c>
     </row>
@@ -6808,11 +6808,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>10254</v>
+        <v>10279</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1130</t>
+          <t>+1155</t>
         </is>
       </c>
     </row>
@@ -6823,11 +6823,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>9811</v>
+        <v>9836</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1049</t>
+          <t>+1074</t>
         </is>
       </c>
     </row>
@@ -6838,11 +6838,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>9084</v>
+        <v>9107</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1038</t>
+          <t>+1061</t>
         </is>
       </c>
     </row>
@@ -6853,11 +6853,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>8433</v>
+        <v>8448</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+945</t>
+          <t>+960</t>
         </is>
       </c>
     </row>
@@ -6868,11 +6868,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>7797</v>
+        <v>7812</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+817</t>
+          <t>+832</t>
         </is>
       </c>
     </row>
@@ -6958,11 +6958,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>8041</v>
+        <v>8056</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+861</t>
+          <t>+876</t>
         </is>
       </c>
     </row>
@@ -6973,11 +6973,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>663</v>
+        <v>713</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+202</t>
+          <t>+252</t>
         </is>
       </c>
     </row>
@@ -6988,11 +6988,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>525</v>
+        <v>560</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+139</t>
+          <t>+174</t>
         </is>
       </c>
     </row>
@@ -7033,11 +7033,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>5901</v>
+        <v>5957</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+558</t>
+          <t>+614</t>
         </is>
       </c>
     </row>
@@ -7153,11 +7153,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>5837</v>
+        <v>5897</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+556</t>
+          <t>+616</t>
         </is>
       </c>
     </row>
@@ -7168,11 +7168,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>5863</v>
+        <v>5884</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+638</t>
+          <t>+659</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-09 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -15,6 +15,7 @@
     <sheet name="2026-07-05" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-07-06" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-07-07" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-07-09" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -453,6 +454,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-09 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4453</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1565</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1853</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+175</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2150</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1264</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+124</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>5137</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1319</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>2110</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1298</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4892</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+721</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>13061</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+2297</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+370</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+370</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+360</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+366</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+362</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>12506</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+2281</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>11828</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2241</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10995</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2181</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>10409</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2110</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>12776</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2121</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>12252</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2125</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>11521</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+2075</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10662</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1999</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+393</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>12550</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+2271</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>12067</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+2231</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>11269</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+2162</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>10553</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+2105</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9823</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1811</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+283</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>393</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>9947</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1891</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+385</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+385</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1843</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1265</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+293</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>7450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1493</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5376</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>3970</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-449</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>3907</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-512</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>3926</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-493</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>5755</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1336</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>5673</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1254</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>7349</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1452</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>7444</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1560</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>6022</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1204</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>6216</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+1236</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-09 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-09 13:01:00</t>
+          <t>Timestamp: 2026-07-09 13:31:00</t>
         </is>
       </c>
     </row>
@@ -551,11 +551,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2150</v>
+        <v>2175</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1264</t>
+          <t>+1289</t>
         </is>
       </c>
     </row>
@@ -626,11 +626,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>2110</v>
+        <v>2135</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1298</t>
+          <t>+1323</t>
         </is>
       </c>
     </row>
@@ -656,11 +656,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>4892</v>
+        <v>4992</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+721</t>
+          <t>+821</t>
         </is>
       </c>
     </row>
@@ -671,11 +671,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>13061</v>
+        <v>13086</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2297</t>
+          <t>+2322</t>
         </is>
       </c>
     </row>
@@ -761,11 +761,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>12506</v>
+        <v>12531</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2281</t>
+          <t>+2306</t>
         </is>
       </c>
     </row>
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>11828</v>
+        <v>11853</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2241</t>
+          <t>+2266</t>
         </is>
       </c>
     </row>
@@ -791,11 +791,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>10995</v>
+        <v>11020</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2181</t>
+          <t>+2206</t>
         </is>
       </c>
     </row>
@@ -806,11 +806,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>10409</v>
+        <v>10434</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2110</t>
+          <t>+2135</t>
         </is>
       </c>
     </row>
@@ -821,11 +821,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>12776</v>
+        <v>12801</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2121</t>
+          <t>+2146</t>
         </is>
       </c>
     </row>
@@ -836,11 +836,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>12252</v>
+        <v>12277</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2125</t>
+          <t>+2150</t>
         </is>
       </c>
     </row>
@@ -851,11 +851,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>11521</v>
+        <v>11546</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2075</t>
+          <t>+2100</t>
         </is>
       </c>
     </row>
@@ -866,11 +866,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>10662</v>
+        <v>10687</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1999</t>
+          <t>+2024</t>
         </is>
       </c>
     </row>
@@ -896,11 +896,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>12550</v>
+        <v>12575</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+2271</t>
+          <t>+2296</t>
         </is>
       </c>
     </row>
@@ -911,11 +911,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>12067</v>
+        <v>12102</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2231</t>
+          <t>+2266</t>
         </is>
       </c>
     </row>
@@ -926,11 +926,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>11269</v>
+        <v>11319</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2162</t>
+          <t>+2212</t>
         </is>
       </c>
     </row>
@@ -941,11 +941,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>10553</v>
+        <v>10603</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2105</t>
+          <t>+2155</t>
         </is>
       </c>
     </row>
@@ -956,11 +956,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9823</v>
+        <v>9873</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2011</t>
+          <t>+2061</t>
         </is>
       </c>
     </row>
@@ -1046,11 +1046,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>9947</v>
+        <v>9972</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1891</t>
+          <t>+1916</t>
         </is>
       </c>
     </row>
@@ -1151,11 +1151,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>5376</v>
+        <v>5401</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+850</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-10 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -16,6 +16,7 @@
     <sheet name="2026-07-06" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-07-07" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-07-09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-07-10" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1303,6 +1304,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-10 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4753</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1853</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2996</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+821</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>5462</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+325</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>2928</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+793</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>5367</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>14086</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>13531</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>12853</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>12045</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>11444</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1010</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>13826</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>13302</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>12571</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>11712</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>13750</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>13241</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1139</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>12494</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>11778</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>11048</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1886</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>443</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>10997</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1550</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1340</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>8470</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1020</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>5927</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+526</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>4620</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-1053</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4557</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1116</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4576</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1097</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6405</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+732</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6348</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>8359</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1010</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>8465</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1021</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>6822</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7004</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+788</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-11 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -17,6 +17,7 @@
     <sheet name="2026-07-07" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-07-09" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-07-10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026-07-11" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2153,6 +2154,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-11 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>5003</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1853</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3196</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>5637</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+175</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3128</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+200</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>5692</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+325</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>15016</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>14436</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+905</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>13733</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+880</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>12945</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>12344</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>14776</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>14247</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+945</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>13496</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>12637</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>14650</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>14166</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>13419</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>12703</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>11948</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1961</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>443</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>11897</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1475</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1415</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+75</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>9070</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>6452</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+525</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>4870</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-1478</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4807</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1541</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4826</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1522</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6655</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+307</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6598</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+250</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>8959</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>9065</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>7472</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>7654</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-11 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -2178,7 +2178,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-11 13:01:00</t>
+          <t>Timestamp: 2026-07-11 13:31:00</t>
         </is>
       </c>
     </row>
@@ -2221,11 +2221,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>5003</v>
+        <v>5053</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+250</t>
+          <t>+300</t>
         </is>
       </c>
     </row>
@@ -2371,11 +2371,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>15016</v>
+        <v>15066</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+930</t>
+          <t>+980</t>
         </is>
       </c>
     </row>
@@ -2461,11 +2461,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>14436</v>
+        <v>14486</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+905</t>
+          <t>+955</t>
         </is>
       </c>
     </row>
@@ -2476,11 +2476,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>13733</v>
+        <v>13783</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+880</t>
+          <t>+930</t>
         </is>
       </c>
     </row>
@@ -2491,11 +2491,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>12945</v>
+        <v>12995</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -2506,11 +2506,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>12344</v>
+        <v>12394</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -2521,11 +2521,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>14776</v>
+        <v>14826</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+1000</t>
         </is>
       </c>
     </row>
@@ -2536,11 +2536,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>14247</v>
+        <v>14297</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+945</t>
+          <t>+995</t>
         </is>
       </c>
     </row>
@@ -2551,11 +2551,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>13496</v>
+        <v>13546</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -2566,11 +2566,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>12637</v>
+        <v>12687</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -2596,11 +2596,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>14650</v>
+        <v>14700</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -2611,11 +2611,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>14166</v>
+        <v>14216</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -2626,11 +2626,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>13419</v>
+        <v>13469</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -2641,11 +2641,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>12703</v>
+        <v>12753</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -2656,11 +2656,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>11948</v>
+        <v>11998</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -2746,11 +2746,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>11897</v>
+        <v>11947</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+950</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-12 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -18,6 +18,7 @@
     <sheet name="2026-07-09" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-07-10" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-07-11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-07-12" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -3003,6 +3004,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-12 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>6458</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1405</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1853</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3937</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+741</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>6587</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3878</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>6443</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+751</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>16866</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>16306</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1820</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>15583</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>14795</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1800</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>14114</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1720</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>17076</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2250</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>16537</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2240</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>15746</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+2200</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>14887</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+2200</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>17050</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>16566</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>15819</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>15103</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>14348</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2361</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>443</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>14147</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+2200</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>11020</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1950</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>7752</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1300</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>4870</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-1728</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4807</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1791</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4826</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1772</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6655</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+57</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6598</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10909</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1950</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>11015</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1950</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>9132</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1660</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>9354</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+1700</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-12 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -3028,7 +3028,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-12 13:01:00</t>
+          <t>Timestamp: 2026-07-12 13:31:00</t>
         </is>
       </c>
     </row>
@@ -3071,11 +3071,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>6458</v>
+        <v>6608</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1405</t>
+          <t>+1555</t>
         </is>
       </c>
     </row>
@@ -3101,11 +3101,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3937</v>
+        <v>4087</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+741</t>
+          <t>+891</t>
         </is>
       </c>
     </row>
@@ -3131,11 +3131,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>6587</v>
+        <v>6737</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -3176,11 +3176,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>3878</v>
+        <v>4028</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+750</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -3221,11 +3221,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>16866</v>
+        <v>16916</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1800</t>
+          <t>+1850</t>
         </is>
       </c>
     </row>
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>16306</v>
+        <v>16356</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1820</t>
+          <t>+1870</t>
         </is>
       </c>
     </row>
@@ -3326,11 +3326,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>15583</v>
+        <v>15633</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1800</t>
+          <t>+1850</t>
         </is>
       </c>
     </row>
@@ -3341,11 +3341,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>14795</v>
+        <v>14845</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1800</t>
+          <t>+1850</t>
         </is>
       </c>
     </row>
@@ -3356,11 +3356,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>14114</v>
+        <v>14164</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1720</t>
+          <t>+1770</t>
         </is>
       </c>
     </row>
@@ -3371,11 +3371,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>17076</v>
+        <v>17126</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -3386,11 +3386,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>16537</v>
+        <v>16587</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2240</t>
+          <t>+2290</t>
         </is>
       </c>
     </row>
@@ -3401,11 +3401,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>15746</v>
+        <v>15796</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2200</t>
+          <t>+2250</t>
         </is>
       </c>
     </row>
@@ -3416,11 +3416,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>14887</v>
+        <v>14937</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+2200</t>
+          <t>+2250</t>
         </is>
       </c>
     </row>
@@ -3446,11 +3446,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>17050</v>
+        <v>17100</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -3461,11 +3461,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>16566</v>
+        <v>16616</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -3476,11 +3476,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>15819</v>
+        <v>15869</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -3491,11 +3491,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>15103</v>
+        <v>15153</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -3506,11 +3506,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>14348</v>
+        <v>14398</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -3536,11 +3536,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>2361</v>
+        <v>2511</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+550</t>
         </is>
       </c>
     </row>
@@ -3596,11 +3596,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>14147</v>
+        <v>14197</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+2200</t>
+          <t>+2250</t>
         </is>
       </c>
     </row>
@@ -3656,11 +3656,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>1815</v>
+        <v>1965</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+400</t>
+          <t>+550</t>
         </is>
       </c>
     </row>
@@ -3671,11 +3671,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>11020</v>
+        <v>11120</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1950</t>
+          <t>+2050</t>
         </is>
       </c>
     </row>
@@ -3701,11 +3701,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>7752</v>
+        <v>7802</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1350</t>
         </is>
       </c>
     </row>
@@ -3791,11 +3791,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>10909</v>
+        <v>11009</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+1950</t>
+          <t>+2050</t>
         </is>
       </c>
     </row>
@@ -3806,11 +3806,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>11015</v>
+        <v>11115</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1950</t>
+          <t>+2050</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-13 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -19,6 +19,7 @@
     <sheet name="2026-07-10" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-07-11" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-07-12" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-07-13" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -3853,6 +3854,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-13 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>7608</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1853</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>5337</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7433</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+696</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>5179</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1151</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>7443</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>19266</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>18706</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>17983</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>17195</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>16514</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>19476</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>18937</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>18146</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>17287</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>19400</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+2300</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>18916</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+2300</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>18159</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+2290</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>17403</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+2250</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>16648</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+2250</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3116</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>443</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>16547</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+2350</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2597</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+632</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>13070</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1950</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>8962</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1160</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5020</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-1578</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4957</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1641</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4976</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1622</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6805</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+207</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6748</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>12959</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1950</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>13065</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1950</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>10732</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1600</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>10904</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+1550</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-13 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -3878,7 +3878,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-13 13:01:00</t>
+          <t>Timestamp: 2026-07-13 13:31:00</t>
         </is>
       </c>
     </row>
@@ -4071,11 +4071,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>19266</v>
+        <v>19291</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4161,11 +4161,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>18706</v>
+        <v>18731</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4176,11 +4176,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>17983</v>
+        <v>18008</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4191,11 +4191,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>17195</v>
+        <v>17220</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4206,11 +4206,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>16514</v>
+        <v>16539</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4221,11 +4221,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>19476</v>
+        <v>19501</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4236,11 +4236,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>18937</v>
+        <v>18962</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4251,11 +4251,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>18146</v>
+        <v>18171</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4266,11 +4266,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>17287</v>
+        <v>17312</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>
@@ -4296,11 +4296,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>19400</v>
+        <v>19425</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2325</t>
         </is>
       </c>
     </row>
@@ -4311,11 +4311,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>18916</v>
+        <v>18941</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2325</t>
         </is>
       </c>
     </row>
@@ -4326,11 +4326,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>18159</v>
+        <v>18184</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2290</t>
+          <t>+2315</t>
         </is>
       </c>
     </row>
@@ -4341,11 +4341,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>17403</v>
+        <v>17428</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -4356,11 +4356,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>16648</v>
+        <v>16673</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -4446,11 +4446,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>16547</v>
+        <v>16572</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-14 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -20,6 +20,7 @@
     <sheet name="2026-07-11" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-07-12" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-07-13" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2026-07-14" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -4703,6 +4704,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-14 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>7608</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1853</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>5337</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1576</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7433</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>699</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>5179</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>7453</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>20291</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>19696</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>18968</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+960</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>18205</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+985</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>17484</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+945</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>20676</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>20137</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>19346</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>18487</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>20525</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>20046</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1105</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>19284</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>18528</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1100</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>17748</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3116</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>443</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>17747</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+218</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2597</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>14120</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>8962</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5020</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-1728</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4957</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1791</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4976</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1772</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6805</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+57</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6748</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>13953</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+994</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>14115</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>11332</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>11504</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-14 13:31:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -4728,7 +4728,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-14 13:01:00</t>
+          <t>Timestamp: 2026-07-14 13:31:00</t>
         </is>
       </c>
     </row>
@@ -4921,11 +4921,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>20291</v>
+        <v>20316</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1025</t>
         </is>
       </c>
     </row>
@@ -5011,11 +5011,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>19696</v>
+        <v>19721</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+965</t>
+          <t>+990</t>
         </is>
       </c>
     </row>
@@ -5026,11 +5026,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>18968</v>
+        <v>18993</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+960</t>
+          <t>+985</t>
         </is>
       </c>
     </row>
@@ -5041,11 +5041,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>18205</v>
+        <v>18230</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+985</t>
+          <t>+1010</t>
         </is>
       </c>
     </row>
@@ -5056,11 +5056,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>17484</v>
+        <v>17509</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+945</t>
+          <t>+970</t>
         </is>
       </c>
     </row>
@@ -5071,11 +5071,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>20676</v>
+        <v>20701</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -5086,11 +5086,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>20137</v>
+        <v>20162</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -5101,11 +5101,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>19346</v>
+        <v>19371</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -5116,11 +5116,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>18487</v>
+        <v>18512</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -5146,11 +5146,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>20525</v>
+        <v>20550</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1125</t>
         </is>
       </c>
     </row>
@@ -5161,11 +5161,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>20046</v>
+        <v>20071</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1105</t>
+          <t>+1130</t>
         </is>
       </c>
     </row>
@@ -5176,11 +5176,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>19284</v>
+        <v>19309</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1125</t>
         </is>
       </c>
     </row>
@@ -5191,11 +5191,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>18528</v>
+        <v>18553</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1125</t>
         </is>
       </c>
     </row>
@@ -5206,11 +5206,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>17748</v>
+        <v>17773</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -5296,11 +5296,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>17747</v>
+        <v>17772</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -5371,11 +5371,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>14120</v>
+        <v>14145</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1075</t>
         </is>
       </c>
     </row>
@@ -5476,11 +5476,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>6748</v>
+        <v>6798</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+50</t>
         </is>
       </c>
     </row>
@@ -5491,11 +5491,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>13953</v>
+        <v>13978</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+994</t>
+          <t>+1019</t>
         </is>
       </c>
     </row>
@@ -5506,11 +5506,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>14115</v>
+        <v>14140</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1075</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-15 13:01:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -21,6 +21,7 @@
     <sheet name="2026-07-12" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-07-13" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-07-14" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026-07-15" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -5553,6 +5554,855 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-15 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>MY | Kosuke Ueki X</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>7608</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2253</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>5337</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1968</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+392</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>7433</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2802</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>849</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>5179</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nasi Goreng Kampung</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>7453</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>21191</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 007</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>370</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 008</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 009</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>366</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 010</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>362</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>20586</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+865</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>19843</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>19080</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>18359</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>21876</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>21337</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>20546</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>19682</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1170</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1138</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>21725</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>21246</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>20484</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>19728</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>18923</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MY | Naruke</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3116</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>443</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>18922</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1098</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MY | Player 003</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+218</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2597</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>15195</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ryugai</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>9087</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+125</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5020</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-1778</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>4957</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-1841</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>4976</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-1822</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6805</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+7</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>6798</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>14976</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+998</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>15190</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1050</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>11932</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>12104</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
backfill zeroed history sheets from detail_clan_history.php
save_daily_history: when a sheet's total rep drops >95% vs previous
(new season rollover), fetch the old season's final reps from the
history API and update both the XLSX cells and A1 metadata in place,
so the daily page shows correct end-of-season gains instead of zeros.
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -9640,7 +9640,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527)</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
     </row>
@@ -9671,11 +9671,11 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>MY | Kosuke Ueki X</t>
+          <t>Deucedrag</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0</v>
+        <v>35080</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -9686,11 +9686,11 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Tears</t>
+          <t>Elavoth</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0</v>
+        <v>28182</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -9701,11 +9701,11 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>MY | iMuiz</t>
+          <t>Shadow</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0</v>
+        <v>28025</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -9716,11 +9716,11 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Sugar Talking</t>
+          <t>Mahsuri</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>0</v>
+        <v>27136</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -9731,11 +9731,11 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>MY | iMuiz X</t>
+          <t>Dracoth</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>0</v>
+        <v>27048</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -9746,11 +9746,11 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Assassin</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0</v>
+        <v>26880</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
@@ -9761,11 +9761,11 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>warrior</t>
+          <t>Parameswara</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>0</v>
+        <v>25831</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
@@ -9776,11 +9776,11 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>CatDile</t>
+          <t>Summoth</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>0</v>
+        <v>25797</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -9791,11 +9791,11 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>My Man on Willpower</t>
+          <t>Zenith</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>0</v>
+        <v>25472</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -9806,11 +9806,11 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Nasi Goreng Kampung</t>
+          <t>Maximoth</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>0</v>
+        <v>24843</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -9821,11 +9821,11 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>OROCHIMARU</t>
+          <t>Hang Tuah</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0</v>
+        <v>24703</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -9836,11 +9836,11 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Mahsuri</t>
+          <t>Astraphel</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>0</v>
+        <v>24498</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -9851,11 +9851,11 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 006</t>
+          <t>Heracoth</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>0</v>
+        <v>24043</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -9866,11 +9866,11 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 007</t>
+          <t>Mahawangsa</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>0</v>
+        <v>23820</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
@@ -9881,11 +9881,11 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 008</t>
+          <t>Noir</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>0</v>
+        <v>23634</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
@@ -9896,11 +9896,11 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 009</t>
+          <t>Tun Teja</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>0</v>
+        <v>22921</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
@@ -9911,11 +9911,11 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 010</t>
+          <t>COPZ1</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>0</v>
+        <v>22049</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
@@ -9926,11 +9926,11 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Parameswara</t>
+          <t>yatoro</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>0</v>
+        <v>22004</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -9941,11 +9941,11 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Hang Tuah</t>
+          <t>KOPZ2</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>0</v>
+        <v>21080</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
@@ -9956,11 +9956,11 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Mahawangsa</t>
+          <t>Ripley</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>0</v>
+        <v>18090</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
@@ -9971,11 +9971,11 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Tun Teja</t>
+          <t>Aluphiee</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>0</v>
+        <v>17335</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
@@ -9986,11 +9986,11 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Elavoth</t>
+          <t>Ryzeee</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>0</v>
+        <v>17258</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
@@ -10001,11 +10001,11 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Dracoth</t>
+          <t>CatDile</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>0</v>
+        <v>15779</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
@@ -10016,11 +10016,11 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Summoth</t>
+          <t>RÄ“Ï‡ â€¢ Â¢â„“Î±Î·Â¢Ñƒ</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>0</v>
+        <v>14271</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -10031,11 +10031,11 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Maximoth</t>
+          <t>PuNch</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>0</v>
+        <v>12060</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -10046,11 +10046,11 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 001</t>
+          <t>§hitnobi</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>0</v>
+        <v>8043</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
@@ -10061,11 +10061,11 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Shadow</t>
+          <t>OROCHIMARU</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>0</v>
+        <v>7998</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -10076,11 +10076,11 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Assassin</t>
+          <t>Tears</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>0</v>
+        <v>7924</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -10091,11 +10091,11 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Zenith</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>0</v>
+        <v>7508</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -10106,11 +10106,11 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Astraphel</t>
+          <t>Sugar Talking</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>0</v>
+        <v>6912</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
@@ -10121,11 +10121,11 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Noir</t>
+          <t>My Man on Willpower</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>0</v>
+        <v>6754</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
@@ -10136,11 +10136,11 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>MY | Naruke</t>
+          <t>Jork</t>
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>0</v>
+        <v>4991</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
@@ -10151,11 +10151,11 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Jork</t>
+          <t>Player</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>0</v>
+        <v>4496</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
@@ -10166,11 +10166,11 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Lotus</t>
+          <t>§hitnobi</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>0</v>
+        <v>4436</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
@@ -10181,11 +10181,11 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Deucedrag</t>
+          <t>MY | iMuiz</t>
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>0</v>
+        <v>2853</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
@@ -10196,11 +10196,11 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Ripley</t>
+          <t>Player</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>0</v>
+        <v>2815</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
@@ -10211,11 +10211,11 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>iZengotsou</t>
+          <t>warrior</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>0</v>
+        <v>2802</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
@@ -10226,11 +10226,11 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Heracoth</t>
+          <t>MY | iMuiz X</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>0</v>
+        <v>2551</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
@@ -10241,11 +10241,11 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 002</t>
+          <t>§hitnobi</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>0</v>
+        <v>1520</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
@@ -10256,11 +10256,11 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>MY | Player 003</t>
+          <t>§hitnobi</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>0</v>
+        <v>1277</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
@@ -10271,11 +10271,11 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>MY | Player 001</t>
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>0</v>
+        <v>1138</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
@@ -10286,11 +10286,11 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>RÄ“Ï‡ â€¢ Â¢â„“Î±Î·Â¢Ñƒ</t>
+          <t>MY | Player 002</t>
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>0</v>
+        <v>1098</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
@@ -10301,11 +10301,11 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Player</t>
+          <t>§hitnobi</t>
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
@@ -10316,11 +10316,11 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>yatoro</t>
+          <t>MY | Player 003</t>
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>0</v>
+        <v>945</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
@@ -10331,11 +10331,11 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Ryugai</t>
+          <t>Nasi Goreng Kampung</t>
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>0</v>
+        <v>475</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
@@ -10346,11 +10346,11 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>PuNch</t>
+          <t>MY | Kosuke Ueki X</t>
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>0</v>
+        <v>462</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
@@ -10361,11 +10361,11 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>§hitnobi</t>
+          <t>MY | Player 006</t>
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>0</v>
+        <v>420</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
@@ -10376,11 +10376,11 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>§hitnobi</t>
+          <t>MY | Player 007</t>
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>0</v>
+        <v>420</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
@@ -10391,11 +10391,11 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>§hitnobi</t>
+          <t>MY | Player 009</t>
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>0</v>
+        <v>416</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
@@ -10406,11 +10406,11 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>§hitnobi</t>
+          <t>MY | Player 010</t>
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>0</v>
+        <v>412</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
@@ -10421,11 +10421,11 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>§hitnobi</t>
+          <t>MY | Player 008</t>
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
@@ -10436,11 +10436,11 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>KOPZ2</t>
+          <t>Lotus</t>
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
@@ -10451,7 +10451,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>COPZ1</t>
+          <t>Ryugai</t>
         </is>
       </c>
       <c r="B56" s="5" t="n">
@@ -10466,7 +10466,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Ryzeee</t>
+          <t>iZengotsou</t>
         </is>
       </c>
       <c r="B57" s="5" t="n">
@@ -10481,7 +10481,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Aluphiee</t>
+          <t>MY | Naruke</t>
         </is>
       </c>
       <c r="B58" s="5" t="n">

</xml_diff>

<commit_message>
un-backfill July 19 XLSX; cross-season guard for index daily diffs
- Rewrite July 19 sheet with live S62 data (17 members, total 10,144)
  instead of backfilled S61 history API data
- Add guard in save_snapshot: discard prev_data if its total rep
  exceeds current total by >20x (cross-season mismatch), so index
  shows N/A daily diffs on season transition day instead of negatives
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -9632,15 +9632,15 @@
   <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S61</t>
+          <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
     </row>
@@ -9671,11 +9671,11 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Deucedrag</t>
+          <t>Astraphel</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>35080</v>
+        <v>940</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -9686,11 +9686,11 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Elavoth</t>
+          <t>Summoth</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>28182</v>
+        <v>900</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -9701,11 +9701,11 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Shadow</t>
+          <t>Mahsuri</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>28025</v>
+        <v>897</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -9716,11 +9716,11 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Mahsuri</t>
+          <t>Noir</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>27136</v>
+        <v>864</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -9731,11 +9731,11 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Dracoth</t>
+          <t>Tun Teja</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>27048</v>
+        <v>795</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -9746,11 +9746,11 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Assassin</t>
+          <t>Shadow</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>26880</v>
+        <v>786</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
@@ -9765,7 +9765,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>25831</v>
+        <v>775</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
@@ -9776,11 +9776,11 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Summoth</t>
+          <t>Assassin</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>25797</v>
+        <v>692</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -9795,7 +9795,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>25472</v>
+        <v>652</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -9806,11 +9806,11 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Maximoth</t>
+          <t>Elavoth</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>24843</v>
+        <v>540</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -9821,11 +9821,11 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Hang Tuah</t>
+          <t>Dracoth</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>24703</v>
+        <v>500</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
@@ -9836,11 +9836,11 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Astraphel</t>
+          <t>Maximoth</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>24498</v>
+        <v>490</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
@@ -9851,11 +9851,11 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Heracoth</t>
+          <t>Hang Tuah</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>24043</v>
+        <v>450</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -9870,7 +9870,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>23820</v>
+        <v>450</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
@@ -9881,11 +9881,11 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Noir</t>
+          <t>Heracoth</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>23634</v>
+        <v>413</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
@@ -9896,11 +9896,11 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Tun Teja</t>
+          <t>OROCHIMARU</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>22921</v>
+        <v>0</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
@@ -9911,11 +9911,11 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>COPZ1</t>
+          <t>Deucedrag</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>22049</v>
+        <v>0</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
restore history API backfill for transition day; show S62 rep-from-reset as gain on new-season days
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -9631,866 +9631,586 @@
   </sheetPr>
   <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Timestamp: 2026-07-19 13:31:00</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-19 13:00:01</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Total Reps</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Daily Reps (+1d)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>35080</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>28182</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>28025</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>27136</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>27048</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>26880</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>25831</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25797</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>25472</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>24843</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>24703</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Astraphel</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>940</v>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>-462</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Summoth</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>900</v>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>-7733</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Mahsuri</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>897</v>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>-2853</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="B15" t="n">
+        <v>24498</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>24043</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>23820</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Noir</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>864</v>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>-5462</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="B18" t="n">
+        <v>23634</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Tun Teja</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>795</v>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>-2551</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Shadow</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>786</v>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>-7508</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Parameswara</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>775</v>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>-2802</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Assassin</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>692</v>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>-1229</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Zenith</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>652</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>-5304</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Elavoth</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>540</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>-475</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Dracoth</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>500</v>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>-7998</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Maximoth</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>490</v>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>-25926</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Hang Tuah</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>450</v>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>-420</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Mahawangsa</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>450</v>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>-420</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Heracoth</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>413</v>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>-410</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="B19" t="n">
+        <v>22921</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>COPZ1</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>22049</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>yatoro</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>22004</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>KOPZ2</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21080</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ripley</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>18090</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Aluphiee</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>17335</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ryzeee</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>17258</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CatDile</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>15779</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RÄ“Ï‡ â€¢ Â¢â„“Î±Î·Â¢Ñƒ</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>14271</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PuNch</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>12060</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>§hitnobi</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>8043</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>OROCHIMARU</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>-416</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Deucedrag</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>-412</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>yatoro</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>22004</v>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>-24631</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>KOPZ2</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="n">
-        <v>21080</v>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>-23303</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Ripley</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>18090</v>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>-22420</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Aluphiee</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>17335</v>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>-21701</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Ryzeee</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>17258</v>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>-26862</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>CatDile</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>15779</v>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>-25737</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>RÄ“Ï‡ â€¢ Â¢â„“Î±Î·Â¢Ñƒ</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>14271</v>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>-24486</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>PuNch</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>12060</v>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>-23402</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="B30" t="n">
+        <v>7998</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tears</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>7924</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>7508</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Sugar Talking</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>6912</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>My Man on Willpower</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>6754</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Jork</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4991</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4496</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>§hitnobi</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
-        <v>8043</v>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>-1138</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>OROCHIMARU</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>7998</v>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>-26825</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Tears</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>7924</v>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>-25689</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>7508</v>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>-24299</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Sugar Talking</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>6912</v>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>-23298</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>My Man on Willpower</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>6754</v>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>-22414</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Jork</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>4991</v>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="B37" t="n">
+        <v>4436</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>MY | iMuiz</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2853</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
-        <v>4496</v>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>-3241</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="B39" t="n">
+        <v>2815</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>warrior</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2802</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>MY | iMuiz X</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2551</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>§hitnobi</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
-        <v>4436</v>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>-70</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>MY | iMuiz</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>2853</v>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>-688</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Player</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>2815</v>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>-5160</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>warrior</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="n">
-        <v>2802</v>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>MY | iMuiz X</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>2551</v>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>-22593</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="B42" t="n">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>§hitnobi</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n">
-        <v>1520</v>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>-1098</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="B43" t="n">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>MY | Player 001</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>MY | Player 002</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>§hitnobi</t>
         </is>
       </c>
-      <c r="B43" s="5" t="n">
-        <v>1277</v>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>-945</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>MY | Player 001</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>1138</v>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>-2682</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>MY | Player 002</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>1098</v>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>-7678</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>§hitnobi</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="n">
+      <c r="B46" t="n">
         <v>1050</v>
       </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>-2682</t>
-        </is>
-      </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>MY | Player 003</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n">
+      <c r="B47" t="n">
         <v>945</v>
       </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>-19241</t>
-        </is>
-      </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Nasi Goreng Kampung</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n">
+      <c r="B48" t="n">
         <v>475</v>
       </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>MY | Kosuke Ueki X</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
+      <c r="B49" t="n">
         <v>462</v>
       </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>-11210</t>
-        </is>
-      </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>MY | Player 006</t>
         </is>
       </c>
-      <c r="B50" s="5" t="n">
+      <c r="B50" t="n">
         <v>420</v>
       </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>MY | Player 007</t>
         </is>
       </c>
-      <c r="B51" s="5" t="n">
+      <c r="B51" t="n">
         <v>420</v>
       </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>MY | Player 009</t>
         </is>
       </c>
-      <c r="B52" s="5" t="n">
+      <c r="B52" t="n">
         <v>416</v>
       </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>MY | Player 010</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n">
+      <c r="B53" t="n">
         <v>412</v>
       </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>MY | Player 008</t>
         </is>
       </c>
-      <c r="B54" s="5" t="n">
+      <c r="B54" t="n">
         <v>410</v>
       </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Lotus</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n">
+      <c r="B55" t="n">
         <v>70</v>
       </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>-18618</t>
-        </is>
-      </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>Ryugai</t>
         </is>
       </c>
-      <c r="B56" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>-19356</t>
-        </is>
+      <c r="B56" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>iZengotsou</t>
         </is>
       </c>
-      <c r="B57" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>-14437</t>
-        </is>
+      <c r="B57" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>MY | Naruke</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>-14531</t>
-        </is>
+      <c r="B58" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
backfill clan_day_points in all historical sheets + lower threshold to >=1
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -495,12 +495,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-09 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>51893</v>
       </c>
     </row>
     <row r="3">
@@ -1330,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1344,12 +1352,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-10 13:01:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>24653</v>
       </c>
     </row>
     <row r="3">
@@ -2179,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2193,12 +2209,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-11 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>19710</v>
       </c>
     </row>
     <row r="3">
@@ -3028,7 +3052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3042,12 +3066,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-12 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>49687</v>
       </c>
     </row>
     <row r="3">
@@ -3877,7 +3909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3891,12 +3923,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-13 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>51909</v>
       </c>
     </row>
     <row r="3">
@@ -4726,7 +4766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4740,12 +4780,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-14 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>21014</v>
       </c>
     </row>
     <row r="3">
@@ -5575,7 +5623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5589,12 +5637,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-15 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>21730</v>
       </c>
     </row>
     <row r="3">
@@ -6349,7 +6405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6363,12 +6419,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-16 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>25818</v>
       </c>
     </row>
     <row r="3">
@@ -7123,7 +7187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7137,12 +7201,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-17 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>28615</v>
       </c>
     </row>
     <row r="3">
@@ -7972,7 +8044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7986,12 +8058,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-18 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>28354</v>
       </c>
     </row>
     <row r="3">
@@ -9640,7 +9720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9649,12 +9729,20 @@
           <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-19 13:00:01</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>108129</v>
       </c>
     </row>
     <row r="3">
@@ -10239,7 +10327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10253,12 +10341,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-20 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -10548,7 +10644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10562,12 +10658,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-21 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>18375</v>
       </c>
     </row>
     <row r="3">
@@ -10857,7 +10961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10871,12 +10975,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-22 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>24979</v>
       </c>
     </row>
     <row r="3">
@@ -11166,7 +11278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11180,12 +11292,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-01 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>19284</v>
       </c>
     </row>
     <row r="3">
@@ -12030,7 +12150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12044,12 +12164,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-02 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>20222</v>
       </c>
     </row>
     <row r="3">
@@ -12849,7 +12977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12863,12 +12991,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-03 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>25494</v>
       </c>
     </row>
     <row r="3">
@@ -13713,7 +13849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13727,12 +13863,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-04 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>22829</v>
       </c>
     </row>
     <row r="3">
@@ -14577,7 +14721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14591,12 +14735,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-05 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>39571</v>
       </c>
     </row>
     <row r="3">
@@ -15441,7 +15593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -15455,12 +15607,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-06 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>33938</v>
       </c>
     </row>
     <row r="3">
@@ -16290,7 +16450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -16304,12 +16464,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-07 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>23419</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
re-backfill clan_day_points after merging remote snapshot
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -496,12 +496,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-09 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>51893</v>
       </c>
     </row>
     <row r="3">
@@ -1331,7 +1339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1345,12 +1353,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-10 13:01:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>24653</v>
       </c>
     </row>
     <row r="3">
@@ -2180,7 +2196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2194,12 +2210,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-11 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>19710</v>
       </c>
     </row>
     <row r="3">
@@ -3029,7 +3053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3043,12 +3067,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-12 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>49687</v>
       </c>
     </row>
     <row r="3">
@@ -3878,7 +3910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3892,12 +3924,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-13 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>51909</v>
       </c>
     </row>
     <row r="3">
@@ -4727,7 +4767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4741,12 +4781,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-14 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>21014</v>
       </c>
     </row>
     <row r="3">
@@ -5576,7 +5624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5590,12 +5638,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-15 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>21730</v>
       </c>
     </row>
     <row r="3">
@@ -6350,7 +6406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6364,12 +6420,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-16 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>25818</v>
       </c>
     </row>
     <row r="3">
@@ -7124,7 +7188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7138,12 +7202,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-17 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>28615</v>
       </c>
     </row>
     <row r="3">
@@ -7973,7 +8045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7987,12 +8059,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-18 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>28354</v>
       </c>
     </row>
     <row r="3">
@@ -9641,7 +9721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9650,12 +9730,20 @@
           <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-19 13:00:01</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>108129</v>
       </c>
     </row>
     <row r="3">
@@ -10240,7 +10328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10254,12 +10342,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-20 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -10549,7 +10645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10563,12 +10659,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-21 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>18375</v>
       </c>
     </row>
     <row r="3">
@@ -10858,7 +10962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10872,12 +10976,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-22 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>24979</v>
       </c>
     </row>
     <row r="3">
@@ -11485,7 +11597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11499,12 +11611,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-01 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>19284</v>
       </c>
     </row>
     <row r="3">
@@ -12349,7 +12469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12363,12 +12483,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-02 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>20222</v>
       </c>
     </row>
     <row r="3">
@@ -13168,7 +13296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -13182,12 +13310,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-03 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>25494</v>
       </c>
     </row>
     <row r="3">
@@ -14032,7 +14168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14046,12 +14182,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-04 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>22829</v>
       </c>
     </row>
     <row r="3">
@@ -14896,7 +15040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14910,12 +15054,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-05 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>39571</v>
       </c>
     </row>
     <row r="3">
@@ -15760,7 +15912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -15774,12 +15926,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-06 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>33938</v>
       </c>
     </row>
     <row r="3">
@@ -16609,7 +16769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -16623,12 +16783,20 @@
           <t>Clan: Clairvoyant (2527) | S62</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Timestamp: 2026-07-07 13:31:00</t>
         </is>
+      </c>
+      <c r="D2" t="n">
+        <v>23419</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
fix season tags, fix season transition bug, regenerate history pages
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -493,7 +493,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -1350,7 +1350,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -3064,7 +3064,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -3921,7 +3921,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -4778,7 +4778,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5635,7 +5635,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -6417,7 +6417,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -7199,7 +7199,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -8056,7 +8056,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -8943,7 +8943,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
     </row>
@@ -11608,7 +11608,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -12480,7 +12480,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -13307,7 +13307,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -14179,7 +14179,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -15051,7 +15051,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -15923,7 +15923,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -16780,7 +16780,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Clan: Clairvoyant (2527) | S62</t>
+          <t>Clan: Clairvoyant (2527) | S61</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>

<commit_message>
auto: snapshot 2026-07-25 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -30,6 +30,7 @@
     <sheet name="2026-07-21" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-07-22" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-07-23" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026-07-25" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -11591,6 +11592,399 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-25 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>18668</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>13397</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+3802</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>11845</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+3160</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>10038</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>9170</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+2305</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>9445</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+2367</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>13211</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+3913</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>11855</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+3425</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>10583</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+2720</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>9320</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+2315</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>13159</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+3858</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>11782</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+3255</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>10235</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+2535</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>9642</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+2317</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>9343</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+2297</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>9074</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+2325</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>1621</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1585</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1415</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1330</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1304</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-25 05:30:23
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -11622,11 +11622,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-25 13:00:10</t>
+          <t>Timestamp: 2026-07-25 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>18668</v>
+        <v>750</v>
       </c>
     </row>
     <row r="3">
@@ -11668,11 +11668,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>13397</v>
+        <v>13447</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+3802</t>
+          <t>+3852</t>
         </is>
       </c>
     </row>
@@ -11683,11 +11683,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>11845</v>
+        <v>11895</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+3160</t>
+          <t>+3210</t>
         </is>
       </c>
     </row>
@@ -11698,11 +11698,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>10038</v>
+        <v>10088</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -11713,11 +11713,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>9170</v>
+        <v>9220</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+2305</t>
+          <t>+2355</t>
         </is>
       </c>
     </row>
@@ -11728,11 +11728,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>9445</v>
+        <v>9495</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+2367</t>
+          <t>+2417</t>
         </is>
       </c>
     </row>
@@ -11743,11 +11743,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>13211</v>
+        <v>13261</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+3913</t>
+          <t>+3963</t>
         </is>
       </c>
     </row>
@@ -11758,11 +11758,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>11855</v>
+        <v>11905</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+3425</t>
+          <t>+3475</t>
         </is>
       </c>
     </row>
@@ -11773,11 +11773,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>10583</v>
+        <v>10633</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+2720</t>
+          <t>+2770</t>
         </is>
       </c>
     </row>
@@ -11788,11 +11788,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>9320</v>
+        <v>9370</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+2315</t>
+          <t>+2365</t>
         </is>
       </c>
     </row>
@@ -11803,11 +11803,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>13159</v>
+        <v>13209</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+3858</t>
+          <t>+3908</t>
         </is>
       </c>
     </row>
@@ -11818,11 +11818,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>11782</v>
+        <v>11832</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+3255</t>
+          <t>+3305</t>
         </is>
       </c>
     </row>
@@ -11833,11 +11833,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>10235</v>
+        <v>10285</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2535</t>
+          <t>+2585</t>
         </is>
       </c>
     </row>
@@ -11848,11 +11848,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>9642</v>
+        <v>9692</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+2317</t>
+          <t>+2367</t>
         </is>
       </c>
     </row>
@@ -11863,11 +11863,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>9343</v>
+        <v>9393</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+2297</t>
+          <t>+2347</t>
         </is>
       </c>
     </row>
@@ -11893,11 +11893,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>9074</v>
+        <v>9124</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+2325</t>
+          <t>+2375</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -31,6 +31,7 @@
     <sheet name="2026-07-22" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-07-23" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-07-25" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2026-07-26" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -11985,6 +11986,399 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-26 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>63934</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>17847</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+4400</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>15895</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+4000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>13408</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+3320</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>12160</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+2940</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>12165</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+2670</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>17631</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+4370</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>15805</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+3900</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>13943</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+3310</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>12340</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+2970</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>17609</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+4400</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>15792</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+3960</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>13585</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+3300</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>12652</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+2960</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>12053</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+2660</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Deucedrag</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11794</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+2670</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>4141</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+2520</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3985</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3845</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2430</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3500</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2170</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3138</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1834</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:30:21
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -12016,11 +12016,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-26 13:00:09</t>
+          <t>Timestamp: 2026-07-26 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>63934</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -12197,11 +12197,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>17609</v>
+        <v>17619</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+4400</t>
+          <t>+4410</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-26 05:44:32
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -12016,11 +12016,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-26 13:30:20</t>
+          <t>Timestamp: 2026-07-26 13:44:31</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>10</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3">
@@ -12302,11 +12302,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>4141</v>
+        <v>4241</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2520</t>
+          <t>+2620</t>
         </is>
       </c>
     </row>
@@ -12317,11 +12317,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>3985</v>
+        <v>4085</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -12332,11 +12332,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3845</v>
+        <v>3945</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2430</t>
+          <t>+2530</t>
         </is>
       </c>
     </row>
@@ -12347,11 +12347,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>3500</v>
+        <v>3600</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2170</t>
+          <t>+2270</t>
         </is>
       </c>
     </row>
@@ -12362,11 +12362,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>3138</v>
+        <v>3238</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1834</t>
+          <t>+1934</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -32,6 +32,7 @@
     <sheet name="2026-07-23" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-07-25" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-07-26" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2026-07-27" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -12379,6 +12380,414 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-27 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>51635</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>20347</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>18395</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>15908</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>14660</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>14665</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>20131</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>18305</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>16443</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>14840</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>19979</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+2360</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>18162</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+2370</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>15945</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+2360</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>15052</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>14433</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+2380</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>14294</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+2500</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>6596</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2355</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>6485</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>6345</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5638</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+2400</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:06:37
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -12410,11 +12410,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-27 13:00:10</t>
+          <t>Timestamp: 2026-07-27 13:06:37</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>51635</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-07-27 05:30:28
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -12410,11 +12410,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-27 13:06:37</t>
+          <t>Timestamp: 2026-07-27 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3">
@@ -12456,11 +12456,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>20347</v>
+        <v>20357</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2510</t>
         </is>
       </c>
     </row>
@@ -12531,11 +12531,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>20131</v>
+        <v>20151</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2520</t>
         </is>
       </c>
     </row>
@@ -12591,11 +12591,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>19979</v>
+        <v>20029</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+2360</t>
+          <t>+2410</t>
         </is>
       </c>
     </row>
@@ -12606,11 +12606,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>18162</v>
+        <v>18207</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2370</t>
+          <t>+2415</t>
         </is>
       </c>
     </row>
@@ -12621,11 +12621,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>15945</v>
+        <v>15970</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2360</t>
+          <t>+2385</t>
         </is>
       </c>
     </row>
@@ -12636,11 +12636,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>15052</v>
+        <v>15077</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2425</t>
         </is>
       </c>
     </row>
@@ -12651,11 +12651,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>14433</v>
+        <v>14458</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+2380</t>
+          <t>+2405</t>
         </is>
       </c>
     </row>
@@ -12666,7 +12666,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>1200</v>
+        <v>1250</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
@@ -12711,11 +12711,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>6596</v>
+        <v>6646</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2355</t>
+          <t>+2405</t>
         </is>
       </c>
     </row>
@@ -12726,11 +12726,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>6485</v>
+        <v>6535</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -12741,11 +12741,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>6345</v>
+        <v>6395</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -12756,11 +12756,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>6000</v>
+        <v>6050</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -12771,11 +12771,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>5638</v>
+        <v>5688</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-28 05:28:33
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -12819,11 +12819,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:00:09</t>
+          <t>Timestamp: 2026-07-28 13:28:32</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>975</v>
       </c>
     </row>
     <row r="3">
@@ -13075,11 +13075,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>1700</v>
+        <v>1750</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+500</t>
         </is>
       </c>
     </row>
@@ -13090,11 +13090,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1763</v>
+        <v>1813</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+663</t>
+          <t>+713</t>
         </is>
       </c>
     </row>
@@ -13120,11 +13120,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>7889</v>
+        <v>7964</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1243</t>
+          <t>+1318</t>
         </is>
       </c>
     </row>
@@ -13135,11 +13135,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>7940</v>
+        <v>8015</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1405</t>
+          <t>+1480</t>
         </is>
       </c>
     </row>
@@ -13150,11 +13150,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>7656</v>
+        <v>7731</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1261</t>
+          <t>+1336</t>
         </is>
       </c>
     </row>
@@ -13165,11 +13165,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>7304</v>
+        <v>7379</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1254</t>
+          <t>+1329</t>
         </is>
       </c>
     </row>
@@ -13180,11 +13180,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>6988</v>
+        <v>7063</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1300</t>
+          <t>+1375</t>
         </is>
       </c>
     </row>
@@ -13195,7 +13195,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
@@ -13210,7 +13210,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -13225,7 +13225,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
@@ -13240,7 +13240,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -13255,7 +13255,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -13270,7 +13270,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>575</v>
+        <v>625</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -13285,7 +13285,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>555</v>
+        <v>605</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
@@ -13300,7 +13300,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>550</v>
+        <v>600</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
@@ -13315,7 +13315,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>550</v>
+        <v>600</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
@@ -13330,7 +13330,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>550</v>
+        <v>600</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -34,6 +34,7 @@
     <sheet name="2026-07-26" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="2026-07-27" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-07-28" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="2026-07-29" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -13347,6 +13348,564 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-29 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>21627</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+595</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>19625</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>17118</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>15860</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>15865</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>21251</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>19405</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>17543</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>15920</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>21129</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>19307</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>17070</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>16132</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>15508</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2338</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+525</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>15344</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9195</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1231</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>9257</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1242</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8973</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1242</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>8587</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1208</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>8293</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1230</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+545</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1145</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+545</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>1056</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+456</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+450</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-29 05:30:22
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -13378,11 +13378,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-29 13:00:09</t>
+          <t>Timestamp: 2026-07-29 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -13499,11 +13499,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>21251</v>
+        <v>21266</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+450</t>
+          <t>+465</t>
         </is>
       </c>
     </row>
@@ -13649,11 +13649,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>2338</v>
+        <v>2363</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+525</t>
+          <t>+550</t>
         </is>
       </c>
     </row>
@@ -13829,11 +13829,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1200</v>
+        <v>1205</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+580</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:00:01
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -35,6 +35,7 @@
     <sheet name="2026-07-27" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="2026-07-28" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="2026-07-29" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="2026-07-30" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -14778,6 +14779,564 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-07-30 13:00:00</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>35213</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>22802</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>20800</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>18318</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>17060</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>17065</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>22451</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1185</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>20605</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>18743</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>17120</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>22329</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>20507</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>18270</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>17332</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>16708</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>2775</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>3513</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>16544</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>10179</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+984</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10232</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+975</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>9908</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+935</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>9519</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+932</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>9240</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+947</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1475</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+925</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+915</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+900</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2355</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2300</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2320</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>2256</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2220</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1170</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:15:48
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -14809,11 +14809,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:00:11</t>
+          <t>Timestamp: 2026-07-30 13:15:47</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>35213</v>
+        <v>35228</v>
       </c>
     </row>
     <row r="3">
@@ -15080,11 +15080,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>3513</v>
+        <v>3523</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1160</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:30:20
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -14809,11 +14809,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:15:47</t>
+          <t>Timestamp: 2026-07-30 13:30:19</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>35228</v>
+        <v>35888</v>
       </c>
     </row>
     <row r="3">
@@ -14855,11 +14855,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>22802</v>
+        <v>22827</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -14870,11 +14870,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>20800</v>
+        <v>20825</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -14885,11 +14885,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>18318</v>
+        <v>18343</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -14900,11 +14900,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>17060</v>
+        <v>17085</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -14915,11 +14915,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>17065</v>
+        <v>17090</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -14930,11 +14930,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>22451</v>
+        <v>22476</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1185</t>
+          <t>+1210</t>
         </is>
       </c>
     </row>
@@ -14945,11 +14945,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>20605</v>
+        <v>20630</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -14960,11 +14960,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>18743</v>
+        <v>18768</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -14975,11 +14975,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>17120</v>
+        <v>17145</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -14990,11 +14990,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>22329</v>
+        <v>22354</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -15005,11 +15005,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>20507</v>
+        <v>20532</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -15020,11 +15020,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>18270</v>
+        <v>18295</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -15035,11 +15035,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>17332</v>
+        <v>17357</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -15050,11 +15050,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>16708</v>
+        <v>16733</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -15065,11 +15065,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>2775</v>
+        <v>2800</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -15080,11 +15080,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>3523</v>
+        <v>3538</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1175</t>
         </is>
       </c>
     </row>
@@ -15095,11 +15095,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>16544</v>
+        <v>16569</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -15185,11 +15185,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>1475</v>
+        <v>1500</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+925</t>
+          <t>+950</t>
         </is>
       </c>
     </row>
@@ -15200,11 +15200,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1465</v>
+        <v>1490</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+915</t>
+          <t>+940</t>
         </is>
       </c>
     </row>
@@ -15215,11 +15215,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>1450</v>
+        <v>1475</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+925</t>
         </is>
       </c>
     </row>
@@ -15230,11 +15230,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1450</v>
+        <v>1475</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+925</t>
         </is>
       </c>
     </row>
@@ -15245,11 +15245,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1450</v>
+        <v>1475</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+900</t>
+          <t>+925</t>
         </is>
       </c>
     </row>
@@ -15260,11 +15260,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>2355</v>
+        <v>2380</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1175</t>
         </is>
       </c>
     </row>
@@ -15275,11 +15275,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>2300</v>
+        <v>2325</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1175</t>
         </is>
       </c>
     </row>
@@ -15290,11 +15290,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>2320</v>
+        <v>2345</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -15305,11 +15305,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>2256</v>
+        <v>2281</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1200</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>
@@ -15320,11 +15320,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>2220</v>
+        <v>2245</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+1170</t>
+          <t>+1195</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-30 05:46:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -14809,11 +14809,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-30 13:30:19</t>
+          <t>Timestamp: 2026-07-30 13:46:00</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>35888</v>
+        <v>35913</v>
       </c>
     </row>
     <row r="3">
@@ -15080,11 +15080,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>3538</v>
+        <v>3563</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1175</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-07-31 05:30:24
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -15368,11 +15368,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-31 13:00:10</t>
+          <t>Timestamp: 2026-07-31 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>675</v>
       </c>
     </row>
     <row r="3">
@@ -15414,11 +15414,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23848</v>
+        <v>23873</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1021</t>
+          <t>+1046</t>
         </is>
       </c>
     </row>
@@ -15429,11 +15429,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>21850</v>
+        <v>21875</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1025</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -15444,11 +15444,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>19368</v>
+        <v>19393</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1025</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -15459,11 +15459,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>18106</v>
+        <v>18131</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+1021</t>
+          <t>+1046</t>
         </is>
       </c>
     </row>
@@ -15474,11 +15474,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>18110</v>
+        <v>18135</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1020</t>
+          <t>+1045</t>
         </is>
       </c>
     </row>
@@ -15489,11 +15489,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>23498</v>
+        <v>23523</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1022</t>
+          <t>+1047</t>
         </is>
       </c>
     </row>
@@ -15504,11 +15504,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>21656</v>
+        <v>21681</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1026</t>
+          <t>+1051</t>
         </is>
       </c>
     </row>
@@ -15519,11 +15519,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>19798</v>
+        <v>19823</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1030</t>
+          <t>+1055</t>
         </is>
       </c>
     </row>
@@ -15534,11 +15534,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>18183</v>
+        <v>18208</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1038</t>
+          <t>+1063</t>
         </is>
       </c>
     </row>
@@ -15549,11 +15549,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>23380</v>
+        <v>23405</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1026</t>
+          <t>+1051</t>
         </is>
       </c>
     </row>
@@ -15564,11 +15564,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>21562</v>
+        <v>21587</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1030</t>
+          <t>+1055</t>
         </is>
       </c>
     </row>
@@ -15579,11 +15579,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>19325</v>
+        <v>19350</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1030</t>
+          <t>+1055</t>
         </is>
       </c>
     </row>
@@ -15594,11 +15594,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>18395</v>
+        <v>18420</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1038</t>
+          <t>+1063</t>
         </is>
       </c>
     </row>
@@ -15609,11 +15609,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>17783</v>
+        <v>17808</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1075</t>
         </is>
       </c>
     </row>
@@ -15624,11 +15624,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>3745</v>
+        <v>3770</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+945</t>
+          <t>+970</t>
         </is>
       </c>
     </row>
@@ -15639,11 +15639,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>4580</v>
+        <v>4605</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1017</t>
+          <t>+1042</t>
         </is>
       </c>
     </row>
@@ -15654,11 +15654,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>17615</v>
+        <v>17640</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1046</t>
+          <t>+1071</t>
         </is>
       </c>
     </row>
@@ -15744,11 +15744,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>2500</v>
+        <v>2525</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1000</t>
+          <t>+1025</t>
         </is>
       </c>
     </row>
@@ -15759,11 +15759,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>2481</v>
+        <v>2506</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+991</t>
+          <t>+1016</t>
         </is>
       </c>
     </row>
@@ -15774,11 +15774,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2455</v>
+        <v>2480</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+980</t>
+          <t>+1005</t>
         </is>
       </c>
     </row>
@@ -15789,11 +15789,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>2364</v>
+        <v>2389</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+889</t>
+          <t>+914</t>
         </is>
       </c>
     </row>
@@ -15804,11 +15804,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>2310</v>
+        <v>2335</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+835</t>
+          <t>+860</t>
         </is>
       </c>
     </row>
@@ -15819,11 +15819,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>3426</v>
+        <v>3451</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1046</t>
+          <t>+1071</t>
         </is>
       </c>
     </row>
@@ -15834,11 +15834,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>3346</v>
+        <v>3371</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1021</t>
+          <t>+1046</t>
         </is>
       </c>
     </row>
@@ -15849,11 +15849,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3395</v>
+        <v>3420</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1050</t>
+          <t>+1075</t>
         </is>
       </c>
     </row>
@@ -15864,11 +15864,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>3282</v>
+        <v>3307</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1001</t>
+          <t>+1026</t>
         </is>
       </c>
     </row>
@@ -15879,11 +15879,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>3255</v>
+        <v>3280</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+1010</t>
+          <t>+1035</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -37,6 +37,7 @@
     <sheet name="2026-07-29" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="2026-07-30" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-07-31" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="2026-08-01" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -15896,6 +15897,564 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-01 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>17920</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>24593</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>22620</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+745</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>20118</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>18821</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>18835</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>23918</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+395</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>22076</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+395</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>20223</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>18588</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+380</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>23780</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>21962</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>19725</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>18795</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>18183</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4445</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>5305</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>18015</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>10529</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10582</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+275</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>10278</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+295</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>9889</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+295</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>9615</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3250</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>3206</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>3145</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+665</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>3049</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2965</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>4226</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+775</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>4121</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>4120</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>4032</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+725</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3980</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-01 05:30:31
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -15927,11 +15927,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-01 13:00:11</t>
+          <t>Timestamp: 2026-08-01 13:30:30</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>17920</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:00:13
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -38,6 +38,7 @@
     <sheet name="2026-07-30" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="2026-07-31" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="2026-08-01" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="2026-08-02" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -16455,6 +16456,564 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-02 13:00:12</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>32770</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>26123</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1530</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24141</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1521</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>21668</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1550</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>20311</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1490</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>20335</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1500</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>23918</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>22076</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>20223</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>18588</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>23780</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>21962</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>19725</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>18795</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>18183</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>6106</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1661</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>6995</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1690</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>18015</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>11694</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1165</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>11822</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1240</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>11488</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1210</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>11069</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1180</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>10825</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1210</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>4840</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1590</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>4806</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1600</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>4745</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1600</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>4610</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1561</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>4445</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1480</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>5847</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1621</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>5752</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1631</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>5720</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1600</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>5582</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1550</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>5570</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1590</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-02 05:30:32
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -16486,11 +16486,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-02 13:00:12</t>
+          <t>Timestamp: 2026-08-02 13:30:31</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>32770</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-03 05:30:22
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -17045,11 +17045,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-03 13:00:10</t>
+          <t>Timestamp: 2026-08-03 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>27266</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:13:41
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -17604,11 +17604,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-04 13:00:09</t>
+          <t>Timestamp: 2026-08-04 13:13:40</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>16045</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-04 05:30:23
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -17604,11 +17604,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-04 13:13:40</t>
+          <t>Timestamp: 2026-08-04 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3">
@@ -17905,11 +17905,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>14190</v>
+        <v>14240</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1096</t>
+          <t>+1146</t>
         </is>
       </c>
     </row>
@@ -17920,11 +17920,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>14274</v>
+        <v>14324</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1150</t>
         </is>
       </c>
     </row>
@@ -17935,11 +17935,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>13846</v>
+        <v>13896</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1092</t>
+          <t>+1142</t>
         </is>
       </c>
     </row>
@@ -17950,11 +17950,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>13359</v>
+        <v>13409</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1064</t>
+          <t>+1114</t>
         </is>
       </c>
     </row>
@@ -17965,11 +17965,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>13283</v>
+        <v>13333</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1150</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -41,6 +41,7 @@
     <sheet name="2026-08-02" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="2026-08-03" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="2026-08-04" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="2026-08-05" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -18132,6 +18133,564 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-05 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>22311</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>28841</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>26846</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>24257</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+865</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>22922</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+865</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>22969</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>23918</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>22076</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>20223</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>18588</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>23780</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>21962</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>19725</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>18795</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>18183</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>9837</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1813</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>10420</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1527</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>18015</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>15411</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1171</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>15475</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1151</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>15043</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1147</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>14564</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1155</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>14508</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1175</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>7617</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>7494</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7434</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>7253</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+839</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7050</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8629</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8529</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>8473</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>8321</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+875</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>8208</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+838</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-05 05:12:36
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -18163,11 +18163,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-05 13:00:09</t>
+          <t>Timestamp: 2026-08-05 13:12:35</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>22311</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:22:44
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -18722,11 +18722,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:00:09</t>
+          <t>Timestamp: 2026-08-06 13:22:43</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>31821</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3">
@@ -19038,11 +19038,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>16660</v>
+        <v>16675</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1185</t>
+          <t>+1200</t>
         </is>
       </c>
     </row>
@@ -19053,11 +19053,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>16169</v>
+        <v>16244</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1126</t>
+          <t>+1201</t>
         </is>
       </c>
     </row>
@@ -19068,11 +19068,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>15710</v>
+        <v>15785</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1146</t>
+          <t>+1221</t>
         </is>
       </c>
     </row>
@@ -19083,11 +19083,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>15658</v>
+        <v>15733</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1225</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:30:29
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -18722,11 +18722,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:22:43</t>
+          <t>Timestamp: 2026-08-06 13:30:28</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>238</v>
+        <v>913</v>
       </c>
     </row>
     <row r="3">
@@ -18768,11 +18768,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>29916</v>
+        <v>29941</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -18783,11 +18783,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>27921</v>
+        <v>27946</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -18798,11 +18798,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>25332</v>
+        <v>25357</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -18813,11 +18813,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>23997</v>
+        <v>24022</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -18828,11 +18828,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>24007</v>
+        <v>24032</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1038</t>
+          <t>+1063</t>
         </is>
       </c>
     </row>
@@ -18843,11 +18843,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>24718</v>
+        <v>24743</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+825</t>
         </is>
       </c>
     </row>
@@ -18858,11 +18858,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>22868</v>
+        <v>22893</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+792</t>
+          <t>+817</t>
         </is>
       </c>
     </row>
@@ -18873,11 +18873,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>21003</v>
+        <v>21028</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+780</t>
+          <t>+805</t>
         </is>
       </c>
     </row>
@@ -18888,11 +18888,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>19388</v>
+        <v>19413</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+825</t>
         </is>
       </c>
     </row>
@@ -18903,11 +18903,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>24580</v>
+        <v>24605</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+825</t>
         </is>
       </c>
     </row>
@@ -18918,11 +18918,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>22721</v>
+        <v>22746</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+759</t>
+          <t>+784</t>
         </is>
       </c>
     </row>
@@ -18933,11 +18933,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>20464</v>
+        <v>20489</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+739</t>
+          <t>+764</t>
         </is>
       </c>
     </row>
@@ -18948,11 +18948,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>19570</v>
+        <v>19595</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+775</t>
+          <t>+800</t>
         </is>
       </c>
     </row>
@@ -18963,11 +18963,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>18958</v>
+        <v>18983</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+775</t>
+          <t>+800</t>
         </is>
       </c>
     </row>
@@ -18978,11 +18978,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>10942</v>
+        <v>10967</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1105</t>
+          <t>+1130</t>
         </is>
       </c>
     </row>
@@ -18993,11 +18993,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>11525</v>
+        <v>11550</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1105</t>
+          <t>+1130</t>
         </is>
       </c>
     </row>
@@ -19008,11 +19008,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>18815</v>
+        <v>18840</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+800</t>
+          <t>+825</t>
         </is>
       </c>
     </row>
@@ -19098,11 +19098,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>8673</v>
+        <v>8698</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1056</t>
+          <t>+1081</t>
         </is>
       </c>
     </row>
@@ -19113,11 +19113,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>8569</v>
+        <v>8594</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19128,11 +19128,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>8509</v>
+        <v>8534</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19143,11 +19143,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>8308</v>
+        <v>8333</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1055</t>
+          <t>+1080</t>
         </is>
       </c>
     </row>
@@ -19158,11 +19158,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>8105</v>
+        <v>8130</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1055</t>
+          <t>+1080</t>
         </is>
       </c>
     </row>
@@ -19173,11 +19173,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>9700</v>
+        <v>9725</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1071</t>
+          <t>+1096</t>
         </is>
       </c>
     </row>
@@ -19188,11 +19188,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>9604</v>
+        <v>9629</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19203,11 +19203,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9548</v>
+        <v>9573</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19218,11 +19218,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>9396</v>
+        <v>9421</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19233,11 +19233,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>9283</v>
+        <v>9308</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 05:52:58
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -18722,11 +18722,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:30:28</t>
+          <t>Timestamp: 2026-08-06 13:52:57</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>913</v>
+        <v>918</v>
       </c>
     </row>
     <row r="3">
@@ -18978,11 +18978,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>10967</v>
+        <v>10972</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1130</t>
+          <t>+1135</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:00:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -43,6 +43,7 @@
     <sheet name="2026-08-04" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="2026-08-05" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-06" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="2026-08-07" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -19250,6 +19251,654 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-07 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>42351</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>31031</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1090</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>29021</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>26432</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>25097</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>25102</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1070</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>25893</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>24043</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>22103</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>20488</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>25751</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1146</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>23856</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1110</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>21564</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>20670</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>20058</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>12092</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>12675</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1065</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>19905</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1065</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>17770</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1200</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>17796</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1121</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>17345</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1101</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>16894</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1109</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>16798</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1065</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>9799</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1101</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9669</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>9609</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>9408</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>9205</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>10845</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>10704</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>10648</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>10496</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>10383</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 05:30:26
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -19281,11 +19281,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-07 13:00:11</t>
+          <t>Timestamp: 2026-08-07 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>42351</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="3">
@@ -19327,11 +19327,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>31031</v>
+        <v>31056</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1090</t>
+          <t>+1115</t>
         </is>
       </c>
     </row>
@@ -19342,11 +19342,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>29021</v>
+        <v>29046</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19357,11 +19357,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>26432</v>
+        <v>26457</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19372,11 +19372,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>25097</v>
+        <v>25122</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19387,11 +19387,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>25102</v>
+        <v>25127</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1070</t>
+          <t>+1095</t>
         </is>
       </c>
     </row>
@@ -19402,11 +19402,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>25893</v>
+        <v>25918</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1175</t>
         </is>
       </c>
     </row>
@@ -19417,11 +19417,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>24043</v>
+        <v>24068</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1150</t>
+          <t>+1175</t>
         </is>
       </c>
     </row>
@@ -19432,11 +19432,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>22103</v>
+        <v>22128</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19447,11 +19447,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>20488</v>
+        <v>20513</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19462,11 +19462,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>25751</v>
+        <v>25776</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1146</t>
+          <t>+1171</t>
         </is>
       </c>
     </row>
@@ -19477,11 +19477,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>23856</v>
+        <v>23881</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1110</t>
+          <t>+1135</t>
         </is>
       </c>
     </row>
@@ -19492,11 +19492,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>21564</v>
+        <v>21589</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19507,11 +19507,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>20670</v>
+        <v>20695</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19522,11 +19522,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>20058</v>
+        <v>20083</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19537,7 +19537,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
@@ -19552,7 +19552,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
@@ -19567,11 +19567,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>12092</v>
+        <v>12117</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1145</t>
         </is>
       </c>
     </row>
@@ -19582,11 +19582,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>12675</v>
+        <v>12700</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1125</t>
+          <t>+1150</t>
         </is>
       </c>
     </row>
@@ -19597,7 +19597,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
@@ -19612,7 +19612,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1065</v>
+        <v>1090</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
@@ -19627,7 +19627,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1050</v>
+        <v>1075</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
@@ -19642,7 +19642,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1050</v>
+        <v>1075</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
@@ -19657,11 +19657,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>19905</v>
+        <v>19930</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1065</t>
+          <t>+1090</t>
         </is>
       </c>
     </row>
@@ -19687,11 +19687,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>17796</v>
+        <v>17859</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+1121</t>
+          <t>+1184</t>
         </is>
       </c>
     </row>
@@ -19702,11 +19702,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>17345</v>
+        <v>17420</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1101</t>
+          <t>+1176</t>
         </is>
       </c>
     </row>
@@ -19717,11 +19717,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>16894</v>
+        <v>16969</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1109</t>
+          <t>+1184</t>
         </is>
       </c>
     </row>
@@ -19732,11 +19732,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>16798</v>
+        <v>16873</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1065</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -19747,11 +19747,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>9799</v>
+        <v>9824</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1101</t>
+          <t>+1126</t>
         </is>
       </c>
     </row>
@@ -19762,11 +19762,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9669</v>
+        <v>9694</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19777,11 +19777,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>9609</v>
+        <v>9634</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19792,11 +19792,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>9408</v>
+        <v>9433</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19807,11 +19807,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>9205</v>
+        <v>9230</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19822,11 +19822,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>10845</v>
+        <v>10870</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1145</t>
         </is>
       </c>
     </row>
@@ -19837,11 +19837,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>10704</v>
+        <v>10729</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19852,11 +19852,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>10648</v>
+        <v>10673</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19867,11 +19867,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>10496</v>
+        <v>10521</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -19882,11 +19882,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>10383</v>
+        <v>10408</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:00:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -44,6 +44,7 @@
     <sheet name="2026-08-05" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="2026-08-06" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-07" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="2026-08-08" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -19899,6 +19900,654 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-08 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>34670</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>31947</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+891</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>29877</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+831</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>27264</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+807</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>25892</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>25888</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+761</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>27002</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1084</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>25092</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1024</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>23124</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+996</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>21427</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+914</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>26838</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1062</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>24889</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1008</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>22531</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+942</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>21571</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+876</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>20887</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+804</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>2212</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1112</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>2162</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1062</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>13168</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1051</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>13755</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1055</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2082</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+982</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1986</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+896</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1913</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+838</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1866</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+791</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>20776</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+846</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>18559</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+789</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>18629</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+770</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>18208</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+788</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>17761</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+792</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>17622</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+749</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>10747</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+923</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>10529</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+835</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10449</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+815</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>10238</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+805</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>10006</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+776</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>11793</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+923</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>11572</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+843</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>11484</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+811</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>11294</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+773</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>11170</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+762</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 05:30:36
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -19930,11 +19930,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:00:11</t>
+          <t>Timestamp: 2026-08-08 13:30:35</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>34670</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="3">
@@ -19976,11 +19976,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>31947</v>
+        <v>31997</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+891</t>
+          <t>+941</t>
         </is>
       </c>
     </row>
@@ -19991,11 +19991,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>29877</v>
+        <v>29927</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+831</t>
+          <t>+881</t>
         </is>
       </c>
     </row>
@@ -20006,11 +20006,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>27264</v>
+        <v>27310</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+807</t>
+          <t>+853</t>
         </is>
       </c>
     </row>
@@ -20021,11 +20021,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>25892</v>
+        <v>25922</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+770</t>
+          <t>+800</t>
         </is>
       </c>
     </row>
@@ -20036,11 +20036,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>25888</v>
+        <v>25918</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+761</t>
+          <t>+791</t>
         </is>
       </c>
     </row>
@@ -20051,11 +20051,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>27002</v>
+        <v>27052</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1084</t>
+          <t>+1134</t>
         </is>
       </c>
     </row>
@@ -20066,11 +20066,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>25092</v>
+        <v>25142</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1024</t>
+          <t>+1074</t>
         </is>
       </c>
     </row>
@@ -20081,11 +20081,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>23124</v>
+        <v>23174</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+996</t>
+          <t>+1046</t>
         </is>
       </c>
     </row>
@@ -20096,11 +20096,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>21427</v>
+        <v>21477</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+914</t>
+          <t>+964</t>
         </is>
       </c>
     </row>
@@ -20111,11 +20111,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>26838</v>
+        <v>26888</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1062</t>
+          <t>+1112</t>
         </is>
       </c>
     </row>
@@ -20126,11 +20126,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>24889</v>
+        <v>24939</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1008</t>
+          <t>+1058</t>
         </is>
       </c>
     </row>
@@ -20141,11 +20141,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>22531</v>
+        <v>22581</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+942</t>
+          <t>+992</t>
         </is>
       </c>
     </row>
@@ -20156,11 +20156,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>21571</v>
+        <v>21621</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+876</t>
+          <t>+926</t>
         </is>
       </c>
     </row>
@@ -20171,11 +20171,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>20887</v>
+        <v>20917</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+804</t>
+          <t>+834</t>
         </is>
       </c>
     </row>
@@ -20186,11 +20186,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>2212</v>
+        <v>2262</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1112</t>
+          <t>+1162</t>
         </is>
       </c>
     </row>
@@ -20201,11 +20201,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>2162</v>
+        <v>2212</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1062</t>
+          <t>+1112</t>
         </is>
       </c>
     </row>
@@ -20216,11 +20216,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>13168</v>
+        <v>13218</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1051</t>
+          <t>+1101</t>
         </is>
       </c>
     </row>
@@ -20231,11 +20231,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>13755</v>
+        <v>13805</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1055</t>
+          <t>+1105</t>
         </is>
       </c>
     </row>
@@ -20246,11 +20246,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>2082</v>
+        <v>2132</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+982</t>
+          <t>+1032</t>
         </is>
       </c>
     </row>
@@ -20261,11 +20261,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>1986</v>
+        <v>2036</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+896</t>
+          <t>+946</t>
         </is>
       </c>
     </row>
@@ -20276,11 +20276,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>1913</v>
+        <v>1963</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+838</t>
+          <t>+888</t>
         </is>
       </c>
     </row>
@@ -20291,11 +20291,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1866</v>
+        <v>1904</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+791</t>
+          <t>+829</t>
         </is>
       </c>
     </row>
@@ -20306,11 +20306,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>20776</v>
+        <v>20814</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+846</t>
+          <t>+884</t>
         </is>
       </c>
     </row>
@@ -20396,11 +20396,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>10747</v>
+        <v>10797</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+923</t>
+          <t>+973</t>
         </is>
       </c>
     </row>
@@ -20411,11 +20411,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>10529</v>
+        <v>10579</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+835</t>
+          <t>+885</t>
         </is>
       </c>
     </row>
@@ -20426,11 +20426,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>10449</v>
+        <v>10479</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+815</t>
+          <t>+845</t>
         </is>
       </c>
     </row>
@@ -20441,11 +20441,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>10238</v>
+        <v>10268</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+805</t>
+          <t>+835</t>
         </is>
       </c>
     </row>
@@ -20456,11 +20456,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>10006</v>
+        <v>10036</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+776</t>
+          <t>+806</t>
         </is>
       </c>
     </row>
@@ -20471,11 +20471,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>11793</v>
+        <v>11843</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+923</t>
+          <t>+973</t>
         </is>
       </c>
     </row>
@@ -20486,11 +20486,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>11572</v>
+        <v>11622</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+843</t>
+          <t>+893</t>
         </is>
       </c>
     </row>
@@ -20501,11 +20501,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>11484</v>
+        <v>11514</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+811</t>
+          <t>+841</t>
         </is>
       </c>
     </row>
@@ -20516,11 +20516,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>11294</v>
+        <v>11324</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+773</t>
+          <t>+803</t>
         </is>
       </c>
     </row>
@@ -20531,11 +20531,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>11170</v>
+        <v>11200</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+762</t>
+          <t>+792</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-09 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -45,6 +45,7 @@
     <sheet name="2026-08-06" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="2026-08-07" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-08-08" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="2026-08-09" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -21375,6 +21376,669 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S62</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-09 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>33347</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>31261</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1334</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>28590</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1280</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>27034</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1112</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>28368</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+2450</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>28402</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>26492</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1350</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>24476</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1302</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>22675</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1198</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>28268</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1380</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>26311</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1372</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>23905</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1324</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>22864</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1243</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>28218</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+7301</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>3662</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>3612</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1400</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45740</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>58752</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+45534</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>60364</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+46559</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3536</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1404</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3320</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1284</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3135</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1172</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3010</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1106</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>25054</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+4240</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>19945</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1386</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>20060</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1431</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>19627</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1419</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>19180</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1419</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>19099</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1477</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>12847</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+2050</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>12593</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>12311</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1832</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>11991</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1723</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>11586</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1550</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>13925</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+2082</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>13622</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>13397</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1883</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>13034</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1710</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>12808</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1608</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 05:00:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -46,6 +46,7 @@
     <sheet name="2026-08-07" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="2026-08-08" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-08-09" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="2026-08-10" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -22039,6 +22040,669 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-10 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>OROCHIMARU</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -47,6 +47,7 @@
     <sheet name="2026-08-08" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="2026-08-09" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-08-10" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="2026-08-11" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -22703,6 +22704,639 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-11 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>47685</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1030</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1030</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1018</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1018</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>740</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>740</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1922</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1922</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1625</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1625</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>1570</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1570</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>1528</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1528</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>2366</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+2366</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>2150</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+2150</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>2071</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+2071</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>2027</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2449</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+2449</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>2377</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+2377</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>1075</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2335</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+2335</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>2225</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+2225</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>2061</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2061</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>2040</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+2040</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1417</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1417</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1045</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1045</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1025</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>890</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>740</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>695</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+695</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1070</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1070</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1025</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1025</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>790</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>740</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>733</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+733</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:01:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -22734,11 +22734,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-11 13:00:09</t>
+          <t>Timestamp: 2026-08-11 13:01:10</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>47685</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 05:30:21
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -22734,11 +22734,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-11 13:01:10</t>
+          <t>Timestamp: 2026-08-11 13:30:20</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>790</v>
       </c>
     </row>
     <row r="3">
@@ -22765,11 +22765,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -22780,11 +22780,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1030</v>
+        <v>1055</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+1030</t>
+          <t>+1055</t>
         </is>
       </c>
     </row>
@@ -22795,11 +22795,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1018</v>
+        <v>1043</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+1018</t>
+          <t>+1043</t>
         </is>
       </c>
     </row>
@@ -22810,11 +22810,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>740</v>
+        <v>765</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+765</t>
         </is>
       </c>
     </row>
@@ -22825,11 +22825,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>740</v>
+        <v>765</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+765</t>
         </is>
       </c>
     </row>
@@ -22840,11 +22840,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1922</v>
+        <v>1947</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1922</t>
+          <t>+1947</t>
         </is>
       </c>
     </row>
@@ -22855,11 +22855,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>1625</v>
+        <v>1650</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1625</t>
+          <t>+1650</t>
         </is>
       </c>
     </row>
@@ -22870,11 +22870,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1570</v>
+        <v>1595</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1570</t>
+          <t>+1595</t>
         </is>
       </c>
     </row>
@@ -22885,11 +22885,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>1528</v>
+        <v>1553</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1528</t>
+          <t>+1553</t>
         </is>
       </c>
     </row>
@@ -22900,11 +22900,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>2366</v>
+        <v>2391</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+2366</t>
+          <t>+2391</t>
         </is>
       </c>
     </row>
@@ -22915,11 +22915,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>2150</v>
+        <v>2175</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+2150</t>
+          <t>+2175</t>
         </is>
       </c>
     </row>
@@ -22930,11 +22930,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>2071</v>
+        <v>2096</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2071</t>
+          <t>+2096</t>
         </is>
       </c>
     </row>
@@ -22945,11 +22945,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>2027</v>
+        <v>2042</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2027</t>
+          <t>+2042</t>
         </is>
       </c>
     </row>
@@ -22975,11 +22975,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>2449</v>
+        <v>2474</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+2449</t>
+          <t>+2474</t>
         </is>
       </c>
     </row>
@@ -22990,11 +22990,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>2377</v>
+        <v>2402</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+2377</t>
+          <t>+2402</t>
         </is>
       </c>
     </row>
@@ -23005,11 +23005,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -23020,11 +23020,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>1075</v>
+        <v>1100</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1100</t>
         </is>
       </c>
     </row>
@@ -23035,11 +23035,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>2335</v>
+        <v>2360</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2335</t>
+          <t>+2360</t>
         </is>
       </c>
     </row>
@@ -23050,11 +23050,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>2225</v>
+        <v>2250</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2225</t>
+          <t>+2250</t>
         </is>
       </c>
     </row>
@@ -23065,11 +23065,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>2061</v>
+        <v>2086</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2061</t>
+          <t>+2086</t>
         </is>
       </c>
     </row>
@@ -23080,11 +23080,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>2040</v>
+        <v>2065</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2040</t>
+          <t>+2065</t>
         </is>
       </c>
     </row>
@@ -23095,11 +23095,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1417</v>
+        <v>1442</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1417</t>
+          <t>+1442</t>
         </is>
       </c>
     </row>
@@ -23185,11 +23185,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1045</v>
+        <v>1070</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1045</t>
+          <t>+1070</t>
         </is>
       </c>
     </row>
@@ -23200,11 +23200,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1025</v>
+        <v>1050</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1025</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -23215,11 +23215,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>890</v>
+        <v>915</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+915</t>
         </is>
       </c>
     </row>
@@ -23230,11 +23230,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>740</v>
+        <v>765</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+765</t>
         </is>
       </c>
     </row>
@@ -23245,11 +23245,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>695</v>
+        <v>720</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+695</t>
+          <t>+720</t>
         </is>
       </c>
     </row>
@@ -23260,11 +23260,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>1070</v>
+        <v>1095</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+1070</t>
+          <t>+1095</t>
         </is>
       </c>
     </row>
@@ -23275,11 +23275,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>1025</v>
+        <v>1050</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1025</t>
+          <t>+1050</t>
         </is>
       </c>
     </row>
@@ -23290,11 +23290,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>790</v>
+        <v>815</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+790</t>
+          <t>+815</t>
         </is>
       </c>
     </row>
@@ -23305,11 +23305,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>740</v>
+        <v>765</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+765</t>
         </is>
       </c>
     </row>
@@ -23320,11 +23320,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>733</v>
+        <v>758</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+733</t>
+          <t>+758</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -48,6 +48,7 @@
     <sheet name="2026-08-09" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="2026-08-10" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-08-11" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -23337,6 +23338,744 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-12 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>31916</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1990</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1905</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1748</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+705</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1465</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1440</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>3117</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1170</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2625</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+975</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2366</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+771</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>2218</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+665</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>3606</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1215</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>3345</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1170</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>3226</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1130</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>3102</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1060</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>2971</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+955</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3724</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>3652</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>2050</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2050</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>3610</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1250</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3430</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1180</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>3236</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>3120</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1055</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2092</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+650</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Ñ‚Ñ”Ð¼ÏÑ”Ñ•Ñ‚</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>MercidaÎ¦</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Digipicâ„¢</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Î›Ñ”tÑ”rÐŸÂµÐ¼</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1935</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+885</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1740</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>1530</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+765</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1455</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+735</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2045</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1935</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+885</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>1640</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+825</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>1530</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+765</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>1473</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+715</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:26:27
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -23368,11 +23368,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:00:10</t>
+          <t>Timestamp: 2026-08-12 13:26:26</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>31916</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3">
@@ -23399,11 +23399,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1990</v>
+        <v>2015</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+915</t>
         </is>
       </c>
     </row>
@@ -23414,11 +23414,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1905</v>
+        <v>1915</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+860</t>
         </is>
       </c>
     </row>
@@ -23639,7 +23639,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
@@ -23654,11 +23654,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>2050</v>
+        <v>2075</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -23669,11 +23669,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>2050</v>
+        <v>2075</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -23759,7 +23759,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -23774,7 +23774,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
@@ -23789,7 +23789,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -23804,7 +23804,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -23819,7 +23819,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -23834,7 +23834,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
@@ -23924,11 +23924,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>2020</v>
+        <v>2045</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -23939,11 +23939,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>1935</v>
+        <v>1960</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+885</t>
+          <t>+910</t>
         </is>
       </c>
     </row>
@@ -23999,11 +23999,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>2045</v>
+        <v>2070</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+950</t>
+          <t>+975</t>
         </is>
       </c>
     </row>
@@ -24014,11 +24014,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>1935</v>
+        <v>1960</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+885</t>
+          <t>+910</t>
         </is>
       </c>
     </row>
@@ -24029,11 +24029,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>1640</v>
+        <v>1665</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+825</t>
+          <t>+850</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:30:24
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -23368,11 +23368,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:26:26</t>
+          <t>Timestamp: 2026-08-12 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>385</v>
+        <v>650</v>
       </c>
     </row>
     <row r="3">
@@ -23414,11 +23414,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1915</v>
+        <v>1930</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+875</t>
         </is>
       </c>
     </row>
@@ -23429,11 +23429,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1748</v>
+        <v>1798</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+705</t>
+          <t>+755</t>
         </is>
       </c>
     </row>
@@ -23444,11 +23444,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1465</v>
+        <v>1515</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -23459,11 +23459,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1440</v>
+        <v>1490</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+725</t>
         </is>
       </c>
     </row>
@@ -24044,11 +24044,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>1530</v>
+        <v>1580</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+765</t>
+          <t>+815</t>
         </is>
       </c>
     </row>
@@ -24059,11 +24059,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>1473</v>
+        <v>1523</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+715</t>
+          <t>+765</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 05:56:47
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -23368,11 +23368,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:30:23</t>
+          <t>Timestamp: 2026-08-12 13:56:46</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>650</v>
+        <v>825</v>
       </c>
     </row>
     <row r="3">
@@ -23639,7 +23639,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
@@ -23759,7 +23759,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
@@ -23774,7 +23774,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
@@ -23789,7 +23789,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
@@ -23804,7 +23804,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -23819,7 +23819,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -23834,7 +23834,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -49,6 +49,7 @@
     <sheet name="2026-08-10" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="2026-08-11" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="2026-08-13" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -24076,6 +24077,744 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-13 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>46286</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3140</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3055</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2923</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2635</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>2610</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1120</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4267</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>3766</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1141</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>3491</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3343</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>4756</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>4490</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1145</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>4371</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1145</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>4247</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1145</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>4116</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1145</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>4874</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4802</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1235</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1160</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>4760</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>4580</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>4386</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>4270</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1150</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3157</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1065</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1240</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1155</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1240</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1240</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1160</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1235</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1245</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1235</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Hika 2</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Hika 3</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Hika 4</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Hika 5</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Hika 6</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3170</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>3085</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>2865</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2655</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2580</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>3195</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3085</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>2705</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2648</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1125</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 05:29:49
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -24107,11 +24107,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-13 13:00:11</t>
+          <t>Timestamp: 2026-08-13 13:29:48</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>46286</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -24378,11 +24378,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1235</v>
+        <v>1245</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1170</t>
         </is>
       </c>
     </row>
@@ -24498,11 +24498,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1240</v>
+        <v>1250</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1155</t>
+          <t>+1165</t>
         </is>
       </c>
     </row>
@@ -24513,7 +24513,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>1240</v>
+        <v>1250</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
@@ -24528,11 +24528,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1240</v>
+        <v>1250</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1160</t>
+          <t>+1170</t>
         </is>
       </c>
     </row>
@@ -24543,7 +24543,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1235</v>
+        <v>1250</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
@@ -24558,7 +24558,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1245</v>
+        <v>1255</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
@@ -24573,7 +24573,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1235</v>
+        <v>1240</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -50,6 +50,7 @@
     <sheet name="2026-08-11" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="2026-08-13" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="2026-08-14" sheetId="45" state="visible" r:id="rId45"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -24815,6 +24816,669 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-14 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>21805</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3710</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+570</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3625</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+570</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3493</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+570</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3210</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>3160</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+550</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4867</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>4366</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>4091</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3943</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>5356</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>5090</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>4971</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>4847</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>4691</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>5474</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>5402</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1595</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>3775</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>3775</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>5360</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>5180</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>4986</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>4870</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>3732</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1605</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1590</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+350</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>3745</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>3660</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>3440</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>3230</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>3155</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3770</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>3660</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>3365</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>3280</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>3223</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+575</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:27:21
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -24846,11 +24846,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-14 13:00:09</t>
+          <t>Timestamp: 2026-08-14 13:27:20</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>21805</v>
+        <v>825</v>
       </c>
     </row>
     <row r="3">
@@ -24877,11 +24877,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>3710</v>
+        <v>3735</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+595</t>
         </is>
       </c>
     </row>
@@ -24892,11 +24892,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3625</v>
+        <v>3650</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+595</t>
         </is>
       </c>
     </row>
@@ -24907,11 +24907,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>3493</v>
+        <v>3518</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+570</t>
+          <t>+595</t>
         </is>
       </c>
     </row>
@@ -24922,11 +24922,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3210</v>
+        <v>3235</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -24937,11 +24937,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3160</v>
+        <v>3185</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+550</t>
+          <t>+575</t>
         </is>
       </c>
     </row>
@@ -24952,11 +24952,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>4867</v>
+        <v>4892</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -24967,11 +24967,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>4366</v>
+        <v>4391</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -24982,11 +24982,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>4091</v>
+        <v>4116</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -24997,11 +24997,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>3943</v>
+        <v>3968</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25012,11 +25012,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5356</v>
+        <v>5381</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25027,11 +25027,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>5090</v>
+        <v>5115</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25042,11 +25042,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>4971</v>
+        <v>4996</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25057,11 +25057,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>4847</v>
+        <v>4872</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25072,11 +25072,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>4691</v>
+        <v>4716</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25087,11 +25087,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>5474</v>
+        <v>5499</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25102,11 +25102,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>5402</v>
+        <v>5427</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25132,11 +25132,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>3775</v>
+        <v>3800</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25147,11 +25147,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>3775</v>
+        <v>3800</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25162,11 +25162,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>5360</v>
+        <v>5385</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25177,11 +25177,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>5180</v>
+        <v>5205</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25192,11 +25192,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>4986</v>
+        <v>5011</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25207,11 +25207,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>4870</v>
+        <v>4895</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25222,11 +25222,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>3732</v>
+        <v>3757</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25327,11 +25327,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3745</v>
+        <v>3770</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25342,11 +25342,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>3660</v>
+        <v>3685</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25357,11 +25357,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>3440</v>
+        <v>3465</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25372,11 +25372,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>3230</v>
+        <v>3255</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25387,11 +25387,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>3155</v>
+        <v>3180</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25402,11 +25402,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>3770</v>
+        <v>3795</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25417,11 +25417,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>3660</v>
+        <v>3685</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25432,11 +25432,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3365</v>
+        <v>3390</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25447,11 +25447,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>3280</v>
+        <v>3305</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -25462,11 +25462,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>3223</v>
+        <v>3248</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-14 05:57:36
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -24846,11 +24846,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-14 13:30:23</t>
+          <t>Timestamp: 2026-08-14 13:57:35</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>825</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="3">
@@ -24877,11 +24877,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>3735</v>
+        <v>3760</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+620</t>
         </is>
       </c>
     </row>
@@ -24892,11 +24892,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>3650</v>
+        <v>3675</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+620</t>
         </is>
       </c>
     </row>
@@ -24907,11 +24907,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>3518</v>
+        <v>3543</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+595</t>
+          <t>+620</t>
         </is>
       </c>
     </row>
@@ -24922,11 +24922,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3235</v>
+        <v>3260</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -24937,11 +24937,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>3185</v>
+        <v>3210</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+575</t>
+          <t>+600</t>
         </is>
       </c>
     </row>
@@ -24952,11 +24952,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>4892</v>
+        <v>4917</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -24967,11 +24967,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>4391</v>
+        <v>4416</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -24982,11 +24982,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>4116</v>
+        <v>4141</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -24997,11 +24997,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>3968</v>
+        <v>3993</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25012,11 +25012,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5381</v>
+        <v>5406</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25027,11 +25027,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>5115</v>
+        <v>5140</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25042,11 +25042,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>4996</v>
+        <v>5021</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25057,11 +25057,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>4872</v>
+        <v>4897</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25072,11 +25072,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>4716</v>
+        <v>4741</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25087,11 +25087,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>5499</v>
+        <v>5524</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25102,11 +25102,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>5427</v>
+        <v>5452</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25117,11 +25117,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>1595</v>
+        <v>1645</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -25132,11 +25132,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>3800</v>
+        <v>3825</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25147,11 +25147,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>3800</v>
+        <v>3825</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25162,11 +25162,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>5385</v>
+        <v>5410</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25177,11 +25177,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>5205</v>
+        <v>5230</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25192,11 +25192,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>5011</v>
+        <v>5036</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25207,11 +25207,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>4895</v>
+        <v>4920</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+625</t>
+          <t>+650</t>
         </is>
       </c>
     </row>
@@ -25222,11 +25222,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>3757</v>
+        <v>3782</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25237,11 +25237,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -25252,11 +25252,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -25267,11 +25267,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -25282,11 +25282,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1600</v>
+        <v>1650</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -25297,11 +25297,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>1605</v>
+        <v>1655</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -25312,11 +25312,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1590</v>
+        <v>1640</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+350</t>
+          <t>+400</t>
         </is>
       </c>
     </row>
@@ -25327,11 +25327,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3770</v>
+        <v>3795</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25342,11 +25342,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>3685</v>
+        <v>3710</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25357,11 +25357,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>3465</v>
+        <v>3490</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25372,11 +25372,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>3255</v>
+        <v>3280</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25387,11 +25387,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>3180</v>
+        <v>3205</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25402,11 +25402,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>3795</v>
+        <v>3820</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25417,11 +25417,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>3685</v>
+        <v>3710</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25432,11 +25432,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3390</v>
+        <v>3415</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25447,11 +25447,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>3305</v>
+        <v>3330</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>
@@ -25462,11 +25462,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>3248</v>
+        <v>3273</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+600</t>
+          <t>+625</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:19:46
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -25510,11 +25510,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-15 13:00:08</t>
+          <t>Timestamp: 2026-08-15 13:19:45</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>50316</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-15 05:30:28
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -25510,11 +25510,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-15 13:19:45</t>
+          <t>Timestamp: 2026-08-15 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3">
@@ -25541,11 +25541,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>4860</v>
+        <v>4870</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1110</t>
         </is>
       </c>
     </row>
@@ -25676,11 +25676,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>6506</v>
+        <v>6526</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -25751,11 +25751,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>6624</v>
+        <v>6674</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1150</t>
         </is>
       </c>
     </row>
@@ -25766,11 +25766,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>6552</v>
+        <v>6572</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -25796,11 +25796,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>4925</v>
+        <v>4975</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1150</t>
         </is>
       </c>
     </row>
@@ -25811,11 +25811,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>4925</v>
+        <v>4945</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -26111,11 +26111,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>4895</v>
+        <v>4905</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1100</t>
+          <t>+1110</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:29:05
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -26294,11 +26294,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:00:09</t>
+          <t>Timestamp: 2026-08-16 13:29:04</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>114972</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="3">
@@ -26325,11 +26325,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>7241</v>
+        <v>7291</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+2371</t>
+          <t>+2421</t>
         </is>
       </c>
     </row>
@@ -26340,11 +26340,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7071</v>
+        <v>7121</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -26355,11 +26355,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>6813</v>
+        <v>6863</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+2290</t>
+          <t>+2340</t>
         </is>
       </c>
     </row>
@@ -26370,11 +26370,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>6522</v>
+        <v>6572</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -26385,11 +26385,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6437</v>
+        <v>6487</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -26400,11 +26400,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8417</v>
+        <v>8467</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26415,11 +26415,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7862</v>
+        <v>7912</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26430,11 +26430,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>7465</v>
+        <v>7515</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26445,11 +26445,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7230</v>
+        <v>7280</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -26460,11 +26460,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>8926</v>
+        <v>8976</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26475,11 +26475,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>8621</v>
+        <v>8671</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+2391</t>
+          <t>+2441</t>
         </is>
       </c>
     </row>
@@ -26490,11 +26490,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>8429</v>
+        <v>8479</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26505,11 +26505,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>8207</v>
+        <v>8257</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26520,11 +26520,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>7997</v>
+        <v>8047</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+2330</t>
+          <t>+2380</t>
         </is>
       </c>
     </row>
@@ -26535,11 +26535,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>9074</v>
+        <v>9124</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26550,11 +26550,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>8972</v>
+        <v>9022</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26565,11 +26565,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>5260</v>
+        <v>5310</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -26580,11 +26580,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>7375</v>
+        <v>7425</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26595,11 +26595,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>7345</v>
+        <v>7395</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26610,11 +26610,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>8900</v>
+        <v>8950</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2390</t>
+          <t>+2440</t>
         </is>
       </c>
     </row>
@@ -26625,11 +26625,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>8666</v>
+        <v>8716</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26640,11 +26640,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>8394</v>
+        <v>8444</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26655,11 +26655,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>8180</v>
+        <v>8230</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -26670,11 +26670,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>6967</v>
+        <v>7017</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2300</t>
+          <t>+2350</t>
         </is>
       </c>
     </row>
@@ -26685,11 +26685,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>5265</v>
+        <v>5315</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -26700,11 +26700,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>5265</v>
+        <v>5315</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -26715,11 +26715,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>5265</v>
+        <v>5315</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -26730,11 +26730,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>5265</v>
+        <v>5315</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -26745,11 +26745,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>5270</v>
+        <v>5320</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -26760,11 +26760,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>3257</v>
+        <v>3307</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2432</t>
+          <t>+2482</t>
         </is>
       </c>
     </row>
@@ -26775,11 +26775,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>5255</v>
+        <v>5305</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2500</t>
+          <t>+2550</t>
         </is>
       </c>
     </row>
@@ -26790,7 +26790,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>3257</v>
+        <v>3307</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
@@ -26805,7 +26805,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>3266</v>
+        <v>3316</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
@@ -26820,11 +26820,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>3266</v>
+        <v>3316</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2441</t>
+          <t>+2491</t>
         </is>
       </c>
     </row>
@@ -26835,7 +26835,7 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>3266</v>
+        <v>3316</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
@@ -26850,11 +26850,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>3266</v>
+        <v>3316</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+2441</t>
+          <t>+2491</t>
         </is>
       </c>
     </row>
@@ -26865,7 +26865,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>3266</v>
+        <v>3316</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
@@ -26880,11 +26880,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3266</v>
+        <v>3316</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+2441</t>
+          <t>+2491</t>
         </is>
       </c>
     </row>
@@ -26895,11 +26895,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>7305</v>
+        <v>7355</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26910,11 +26910,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>7160</v>
+        <v>7210</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+2360</t>
+          <t>+2410</t>
         </is>
       </c>
     </row>
@@ -26925,11 +26925,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>6854</v>
+        <v>6904</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26940,11 +26940,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>6590</v>
+        <v>6640</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26955,11 +26955,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>6466</v>
+        <v>6516</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26970,11 +26970,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>7320</v>
+        <v>7370</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26985,11 +26985,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>7173</v>
+        <v>7223</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -27000,11 +27000,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>6846</v>
+        <v>6896</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -27015,11 +27015,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>6651</v>
+        <v>6701</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -27030,11 +27030,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>6549</v>
+        <v>6599</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:54:14
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -26294,11 +26294,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:30:20</t>
+          <t>Timestamp: 2026-08-16 13:54:13</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>2400</v>
+        <v>4660</v>
       </c>
     </row>
     <row r="3">
@@ -26325,11 +26325,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>7291</v>
+        <v>7341</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+2421</t>
+          <t>+2471</t>
         </is>
       </c>
     </row>
@@ -26340,11 +26340,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7121</v>
+        <v>7171</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26355,11 +26355,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>6863</v>
+        <v>6913</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+2340</t>
+          <t>+2390</t>
         </is>
       </c>
     </row>
@@ -26370,11 +26370,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>6572</v>
+        <v>6592</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2370</t>
         </is>
       </c>
     </row>
@@ -26400,11 +26400,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8467</v>
+        <v>8517</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26415,11 +26415,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>7912</v>
+        <v>7962</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26430,11 +26430,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>7515</v>
+        <v>7565</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26445,11 +26445,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7280</v>
+        <v>7330</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26460,11 +26460,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>8976</v>
+        <v>9026</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26475,11 +26475,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>8671</v>
+        <v>8721</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+2441</t>
+          <t>+2491</t>
         </is>
       </c>
     </row>
@@ -26490,11 +26490,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>8479</v>
+        <v>8529</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26505,11 +26505,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>8257</v>
+        <v>8307</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26520,11 +26520,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>8047</v>
+        <v>8097</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+2380</t>
+          <t>+2430</t>
         </is>
       </c>
     </row>
@@ -26535,11 +26535,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>9124</v>
+        <v>9174</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26550,11 +26550,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>9022</v>
+        <v>9072</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26565,11 +26565,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>5310</v>
+        <v>5360</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -26580,11 +26580,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>7425</v>
+        <v>7475</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26595,11 +26595,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>7395</v>
+        <v>7445</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26610,11 +26610,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>8950</v>
+        <v>9000</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2440</t>
+          <t>+2490</t>
         </is>
       </c>
     </row>
@@ -26625,11 +26625,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>8716</v>
+        <v>8766</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26640,11 +26640,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>8444</v>
+        <v>8494</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26655,11 +26655,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>8230</v>
+        <v>8270</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2390</t>
         </is>
       </c>
     </row>
@@ -26670,11 +26670,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>7017</v>
+        <v>7047</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2380</t>
         </is>
       </c>
     </row>
@@ -26685,11 +26685,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>5315</v>
+        <v>5365</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -26700,11 +26700,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>5315</v>
+        <v>5365</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -26715,11 +26715,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>5315</v>
+        <v>5365</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -26730,11 +26730,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>5315</v>
+        <v>5365</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -26745,11 +26745,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>5320</v>
+        <v>5370</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -26760,11 +26760,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>3307</v>
+        <v>3357</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2482</t>
+          <t>+2532</t>
         </is>
       </c>
     </row>
@@ -26775,11 +26775,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>5305</v>
+        <v>5355</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2550</t>
+          <t>+2600</t>
         </is>
       </c>
     </row>
@@ -26790,7 +26790,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>3307</v>
+        <v>3357</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
@@ -26805,7 +26805,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>3316</v>
+        <v>3366</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
@@ -26820,11 +26820,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>3316</v>
+        <v>3366</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2491</t>
+          <t>+2541</t>
         </is>
       </c>
     </row>
@@ -26835,7 +26835,7 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>3316</v>
+        <v>3366</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
@@ -26850,11 +26850,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>3316</v>
+        <v>3366</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+2491</t>
+          <t>+2541</t>
         </is>
       </c>
     </row>
@@ -26865,7 +26865,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>3316</v>
+        <v>3366</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
@@ -26880,11 +26880,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3316</v>
+        <v>3366</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+2491</t>
+          <t>+2541</t>
         </is>
       </c>
     </row>
@@ -26895,11 +26895,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>7355</v>
+        <v>7405</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26910,11 +26910,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>7210</v>
+        <v>7260</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+2410</t>
+          <t>+2460</t>
         </is>
       </c>
     </row>
@@ -26925,11 +26925,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>6904</v>
+        <v>6954</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26940,11 +26940,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>6640</v>
+        <v>6690</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -26955,11 +26955,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>6516</v>
+        <v>6536</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2420</t>
         </is>
       </c>
     </row>
@@ -26970,11 +26970,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>7370</v>
+        <v>7420</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -26985,11 +26985,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>7223</v>
+        <v>7273</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -27000,11 +27000,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>6896</v>
+        <v>6946</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+2450</t>
+          <t>+2500</t>
         </is>
       </c>
     </row>
@@ -27015,11 +27015,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>6701</v>
+        <v>6751</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -27030,11 +27030,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>6599</v>
+        <v>6649</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+2400</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 05:59:20
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -26294,11 +26294,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:54:13</t>
+          <t>Timestamp: 2026-08-16 13:59:19</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>4660</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="3">
@@ -26370,11 +26370,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>6592</v>
+        <v>6622</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+2370</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26385,11 +26385,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>6487</v>
+        <v>6537</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+2350</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26655,11 +26655,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>8270</v>
+        <v>8280</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+2390</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26670,11 +26670,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>7047</v>
+        <v>7067</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+2380</t>
+          <t>+2400</t>
         </is>
       </c>
     </row>
@@ -26955,11 +26955,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>6536</v>
+        <v>6566</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+2420</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:06:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -27078,11 +27078,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:00:10</t>
+          <t>Timestamp: 2026-08-17 13:06:11</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>105550</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:30:27
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -27078,11 +27078,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:06:11</t>
+          <t>Timestamp: 2026-08-17 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="3">
@@ -27109,7 +27109,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>2671</v>
+        <v>2706</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -27124,7 +27124,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2531</v>
+        <v>2566</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -27139,7 +27139,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>2521</v>
+        <v>2556</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -27154,11 +27154,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>9287</v>
+        <v>9312</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+1946</t>
+          <t>+1971</t>
         </is>
       </c>
     </row>
@@ -27169,11 +27169,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>8973</v>
+        <v>8998</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+1802</t>
+          <t>+1827</t>
         </is>
       </c>
     </row>
@@ -27184,11 +27184,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8653</v>
+        <v>8678</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1740</t>
+          <t>+1765</t>
         </is>
       </c>
     </row>
@@ -27199,11 +27199,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>8310</v>
+        <v>8335</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+1688</t>
+          <t>+1713</t>
         </is>
       </c>
     </row>
@@ -27214,11 +27214,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>8172</v>
+        <v>8202</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+1635</t>
+          <t>+1665</t>
         </is>
       </c>
     </row>
@@ -27229,11 +27229,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>10561</v>
+        <v>10586</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+2044</t>
+          <t>+2069</t>
         </is>
       </c>
     </row>
@@ -27244,11 +27244,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>9880</v>
+        <v>9905</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1918</t>
+          <t>+1943</t>
         </is>
       </c>
     </row>
@@ -27259,11 +27259,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>9367</v>
+        <v>9392</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1802</t>
+          <t>+1827</t>
         </is>
       </c>
     </row>
@@ -27274,11 +27274,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>9096</v>
+        <v>9121</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1766</t>
+          <t>+1791</t>
         </is>
       </c>
     </row>
@@ -27289,11 +27289,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>11054</v>
+        <v>11079</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+2028</t>
+          <t>+2053</t>
         </is>
       </c>
     </row>
@@ -27304,11 +27304,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>10655</v>
+        <v>10680</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+1934</t>
+          <t>+1959</t>
         </is>
       </c>
     </row>
@@ -27319,11 +27319,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>10343</v>
+        <v>10368</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+1814</t>
+          <t>+1839</t>
         </is>
       </c>
     </row>
@@ -27334,11 +27334,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>10007</v>
+        <v>10032</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+1700</t>
+          <t>+1725</t>
         </is>
       </c>
     </row>
@@ -27349,11 +27349,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>9777</v>
+        <v>9802</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+1680</t>
+          <t>+1705</t>
         </is>
       </c>
     </row>
@@ -27364,11 +27364,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>11246</v>
+        <v>11271</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+2072</t>
+          <t>+2097</t>
         </is>
       </c>
     </row>
@@ -27379,11 +27379,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>11036</v>
+        <v>11061</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1964</t>
+          <t>+1989</t>
         </is>
       </c>
     </row>
@@ -27394,11 +27394,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>7400</v>
+        <v>7425</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2040</t>
+          <t>+2065</t>
         </is>
       </c>
     </row>
@@ -27409,11 +27409,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>9551</v>
+        <v>9576</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+2076</t>
+          <t>+2101</t>
         </is>
       </c>
     </row>
@@ -27424,11 +27424,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>9545</v>
+        <v>9570</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+2100</t>
+          <t>+2125</t>
         </is>
       </c>
     </row>
@@ -27439,11 +27439,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>10754</v>
+        <v>10779</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1754</t>
+          <t>+1779</t>
         </is>
       </c>
     </row>
@@ -27454,11 +27454,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>10504</v>
+        <v>10529</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+1738</t>
+          <t>+1763</t>
         </is>
       </c>
     </row>
@@ -27469,11 +27469,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>10224</v>
+        <v>10249</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+1730</t>
+          <t>+1755</t>
         </is>
       </c>
     </row>
@@ -27484,11 +27484,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>10026</v>
+        <v>10051</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+1746</t>
+          <t>+1771</t>
         </is>
       </c>
     </row>
@@ -27499,11 +27499,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>8817</v>
+        <v>8842</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1750</t>
+          <t>+1775</t>
         </is>
       </c>
     </row>
@@ -27514,11 +27514,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>7405</v>
+        <v>7430</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2040</t>
+          <t>+2065</t>
         </is>
       </c>
     </row>
@@ -27529,11 +27529,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>7405</v>
+        <v>7430</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2040</t>
+          <t>+2065</t>
         </is>
       </c>
     </row>
@@ -27544,11 +27544,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>7415</v>
+        <v>7440</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2050</t>
+          <t>+2075</t>
         </is>
       </c>
     </row>
@@ -27559,11 +27559,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>7415</v>
+        <v>7440</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2050</t>
+          <t>+2075</t>
         </is>
       </c>
     </row>
@@ -27574,11 +27574,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>7420</v>
+        <v>7445</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+2050</t>
+          <t>+2075</t>
         </is>
       </c>
     </row>
@@ -27589,11 +27589,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>5607</v>
+        <v>5632</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27604,11 +27604,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>7405</v>
+        <v>7430</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2050</t>
+          <t>+2075</t>
         </is>
       </c>
     </row>
@@ -27619,11 +27619,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>5607</v>
+        <v>5632</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27634,11 +27634,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>5616</v>
+        <v>5641</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27649,11 +27649,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>5616</v>
+        <v>5641</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27664,11 +27664,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>5616</v>
+        <v>5641</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27679,11 +27679,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>5616</v>
+        <v>5641</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27694,11 +27694,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>5616</v>
+        <v>5641</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27709,11 +27709,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>5616</v>
+        <v>5641</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+2250</t>
+          <t>+2275</t>
         </is>
       </c>
     </row>
@@ -27724,11 +27724,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>9357</v>
+        <v>9382</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1952</t>
+          <t>+1977</t>
         </is>
       </c>
     </row>
@@ -27739,11 +27739,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>9038</v>
+        <v>9063</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+1778</t>
+          <t>+1803</t>
         </is>
       </c>
     </row>
@@ -27754,11 +27754,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>8704</v>
+        <v>8729</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+1750</t>
+          <t>+1775</t>
         </is>
       </c>
     </row>
@@ -27769,11 +27769,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>8424</v>
+        <v>8449</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+1734</t>
+          <t>+1759</t>
         </is>
       </c>
     </row>
@@ -27784,11 +27784,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>8256</v>
+        <v>8281</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+1690</t>
+          <t>+1715</t>
         </is>
       </c>
     </row>
@@ -27799,11 +27799,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>9476</v>
+        <v>9501</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+2056</t>
+          <t>+2081</t>
         </is>
       </c>
     </row>
@@ -27814,11 +27814,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>9223</v>
+        <v>9248</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+1950</t>
+          <t>+1975</t>
         </is>
       </c>
     </row>
@@ -27829,11 +27829,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>8788</v>
+        <v>8813</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+1842</t>
+          <t>+1867</t>
         </is>
       </c>
     </row>
@@ -27844,11 +27844,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>8529</v>
+        <v>8554</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+1778</t>
+          <t>+1803</t>
         </is>
       </c>
     </row>
@@ -27859,11 +27859,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>8399</v>
+        <v>8424</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+1750</t>
+          <t>+1775</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-17 05:59:00
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -27078,11 +27078,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-17 13:36:21</t>
+          <t>Timestamp: 2026-08-17 13:58:59</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>1310</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="3">
@@ -27109,7 +27109,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>2706</v>
+        <v>2731</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -27394,11 +27394,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>7425</v>
+        <v>7450</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+2065</t>
+          <t>+2090</t>
         </is>
       </c>
     </row>
@@ -27514,11 +27514,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>7430</v>
+        <v>7455</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+2065</t>
+          <t>+2090</t>
         </is>
       </c>
     </row>
@@ -27529,11 +27529,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>7430</v>
+        <v>7455</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2065</t>
+          <t>+2090</t>
         </is>
       </c>
     </row>
@@ -27544,11 +27544,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>7440</v>
+        <v>7465</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2075</t>
+          <t>+2100</t>
         </is>
       </c>
     </row>
@@ -27559,11 +27559,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>7440</v>
+        <v>7465</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+2075</t>
+          <t>+2100</t>
         </is>
       </c>
     </row>
@@ -27574,11 +27574,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>7445</v>
+        <v>7470</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+2075</t>
+          <t>+2100</t>
         </is>
       </c>
     </row>
@@ -27589,11 +27589,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>5632</v>
+        <v>5657</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -27604,11 +27604,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>7430</v>
+        <v>7455</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2075</t>
+          <t>+2100</t>
         </is>
       </c>
     </row>
@@ -27619,11 +27619,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>5632</v>
+        <v>5657</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -27634,11 +27634,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>5641</v>
+        <v>5666</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -27649,11 +27649,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>5641</v>
+        <v>5666</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -27664,11 +27664,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>5641</v>
+        <v>5666</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -27679,11 +27679,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>5641</v>
+        <v>5666</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -27694,11 +27694,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>5641</v>
+        <v>5666</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>
@@ -27709,11 +27709,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>5641</v>
+        <v>5666</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+2275</t>
+          <t>+2300</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:00:02
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -54,6 +54,7 @@
     <sheet name="2026-08-15" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="2026-08-16" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-08-17" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="2026-08-18" sheetId="49" state="visible" r:id="rId49"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -27876,6 +27877,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-18 13:00:01</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>41372</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3337</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+606</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3274</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+708</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3291</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+735</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>10151</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+839</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>9775</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+777</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>9385</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+707</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>8981</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+646</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>8784</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+582</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>11453</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+867</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>10686</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+781</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>10134</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+742</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>9829</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+708</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>11932</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+853</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>11434</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+754</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>11088</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+720</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>10718</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+686</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>10439</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+637</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>12241</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+970</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>11920</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+859</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>8380</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+930</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>10548</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+972</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>10556</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+986</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>11598</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+819</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>11290</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+761</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>10965</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+716</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>10706</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+655</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>9441</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>8390</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+935</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8383</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+928</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8385</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+920</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>8387</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+922</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>8396</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+926</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>6362</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+705</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>8390</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+935</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>6380</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+723</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>6379</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+713</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>6383</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+717</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>6387</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+721</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>6387</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+721</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>6385</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+719</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>6379</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+713</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>10252</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+870</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>9879</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+816</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>9465</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+736</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>9159</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+710</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>8967</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+686</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>10409</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+908</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10081</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+833</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>9571</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+758</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>9288</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+734</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>9122</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+698</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-18 05:00:48
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -27907,11 +27907,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-18 13:00:01</t>
+          <t>Timestamp: 2026-08-18 13:00:47</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>41372</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -55,6 +55,7 @@
     <sheet name="2026-08-16" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="2026-08-17" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-08-18" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="2026-08-19" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -29577,6 +29578,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-19 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>43216</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3911</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+574</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3826</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+552</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3833</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+542</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>11049</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+898</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>10529</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+754</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>10077</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+692</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>9671</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>9460</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+676</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>12385</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+932</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>11458</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+772</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>10846</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+712</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>10519</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>12778</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+846</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>12152</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+718</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>11778</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>11408</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11129</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>13235</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+994</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>12822</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+902</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>9476</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1096</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>11544</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+996</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>11544</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+988</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>12328</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>11984</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+694</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>11655</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>11396</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>10131</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>9472</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1082</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9469</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1086</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>9467</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1082</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>9461</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1074</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>9466</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1070</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7461</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1099</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>9446</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1056</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>7473</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1093</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>7474</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1095</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>7498</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1115</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>7502</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1115</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>7498</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1111</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>7496</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1111</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>7490</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1111</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>11100</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+848</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>10609</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+730</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>10163</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+698</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>9849</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>9657</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>11305</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+896</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>10797</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+716</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10261</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>9978</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>9802</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+680</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:00:37
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -29608,11 +29608,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:00:09</t>
+          <t>Timestamp: 2026-08-19 13:00:36</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>43216</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-19 05:30:23
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -29608,11 +29608,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-19 13:00:36</t>
+          <t>Timestamp: 2026-08-19 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>934</v>
       </c>
     </row>
     <row r="3">
@@ -29684,11 +29684,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>11049</v>
+        <v>11068</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+898</t>
+          <t>+917</t>
         </is>
       </c>
     </row>
@@ -29699,11 +29699,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>10529</v>
+        <v>10544</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+754</t>
+          <t>+769</t>
         </is>
       </c>
     </row>
@@ -29714,11 +29714,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>10077</v>
+        <v>10092</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+692</t>
+          <t>+707</t>
         </is>
       </c>
     </row>
@@ -29729,11 +29729,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>9671</v>
+        <v>9686</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -29744,11 +29744,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>9460</v>
+        <v>9475</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+676</t>
+          <t>+691</t>
         </is>
       </c>
     </row>
@@ -29759,11 +29759,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>12385</v>
+        <v>12408</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+932</t>
+          <t>+955</t>
         </is>
       </c>
     </row>
@@ -29774,11 +29774,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>11458</v>
+        <v>11473</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+772</t>
+          <t>+787</t>
         </is>
       </c>
     </row>
@@ -29789,11 +29789,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>10846</v>
+        <v>10861</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+712</t>
+          <t>+727</t>
         </is>
       </c>
     </row>
@@ -29804,11 +29804,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>10519</v>
+        <v>10534</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -29819,11 +29819,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>12778</v>
+        <v>12799</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+846</t>
+          <t>+867</t>
         </is>
       </c>
     </row>
@@ -29834,11 +29834,11 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>12152</v>
+        <v>12167</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>+718</t>
+          <t>+733</t>
         </is>
       </c>
     </row>
@@ -29849,11 +29849,11 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>11778</v>
+        <v>11793</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -29864,11 +29864,11 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>11408</v>
+        <v>11423</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -29879,11 +29879,11 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>11129</v>
+        <v>11144</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -29894,11 +29894,11 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>13235</v>
+        <v>13260</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>+994</t>
+          <t>+1019</t>
         </is>
       </c>
     </row>
@@ -29909,11 +29909,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>12822</v>
+        <v>12843</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+902</t>
+          <t>+923</t>
         </is>
       </c>
     </row>
@@ -29924,11 +29924,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>9476</v>
+        <v>9501</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1096</t>
+          <t>+1121</t>
         </is>
       </c>
     </row>
@@ -29939,11 +29939,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>11544</v>
+        <v>11569</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+996</t>
+          <t>+1021</t>
         </is>
       </c>
     </row>
@@ -29954,11 +29954,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>11544</v>
+        <v>11569</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+988</t>
+          <t>+1013</t>
         </is>
       </c>
     </row>
@@ -29969,11 +29969,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>12328</v>
+        <v>12343</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+745</t>
         </is>
       </c>
     </row>
@@ -29984,11 +29984,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>11984</v>
+        <v>11999</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+694</t>
+          <t>+709</t>
         </is>
       </c>
     </row>
@@ -29999,11 +29999,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>11655</v>
+        <v>11670</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30014,11 +30014,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>11396</v>
+        <v>11411</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30029,11 +30029,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>10131</v>
+        <v>10146</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30044,11 +30044,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>9472</v>
+        <v>9497</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1082</t>
+          <t>+1107</t>
         </is>
       </c>
     </row>
@@ -30059,11 +30059,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>9469</v>
+        <v>9494</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1086</t>
+          <t>+1111</t>
         </is>
       </c>
     </row>
@@ -30074,11 +30074,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>9467</v>
+        <v>9492</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1082</t>
+          <t>+1107</t>
         </is>
       </c>
     </row>
@@ -30089,11 +30089,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>9461</v>
+        <v>9486</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1074</t>
+          <t>+1099</t>
         </is>
       </c>
     </row>
@@ -30104,11 +30104,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>9466</v>
+        <v>9491</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1070</t>
+          <t>+1095</t>
         </is>
       </c>
     </row>
@@ -30119,11 +30119,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>7461</v>
+        <v>7486</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+1099</t>
+          <t>+1124</t>
         </is>
       </c>
     </row>
@@ -30134,11 +30134,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>9446</v>
+        <v>9471</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+1056</t>
+          <t>+1081</t>
         </is>
       </c>
     </row>
@@ -30149,11 +30149,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>7473</v>
+        <v>7498</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1093</t>
+          <t>+1118</t>
         </is>
       </c>
     </row>
@@ -30164,11 +30164,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>7474</v>
+        <v>7499</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+1095</t>
+          <t>+1120</t>
         </is>
       </c>
     </row>
@@ -30179,11 +30179,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>7498</v>
+        <v>7523</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1115</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -30194,11 +30194,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>7502</v>
+        <v>7527</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1115</t>
+          <t>+1140</t>
         </is>
       </c>
     </row>
@@ -30209,11 +30209,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>7498</v>
+        <v>7523</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1111</t>
+          <t>+1136</t>
         </is>
       </c>
     </row>
@@ -30224,11 +30224,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>7496</v>
+        <v>7521</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1111</t>
+          <t>+1136</t>
         </is>
       </c>
     </row>
@@ -30239,11 +30239,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>7490</v>
+        <v>7515</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1111</t>
+          <t>+1136</t>
         </is>
       </c>
     </row>
@@ -30254,11 +30254,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>11100</v>
+        <v>11115</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+848</t>
+          <t>+863</t>
         </is>
       </c>
     </row>
@@ -30269,11 +30269,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>10609</v>
+        <v>10624</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+730</t>
+          <t>+745</t>
         </is>
       </c>
     </row>
@@ -30284,11 +30284,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>10163</v>
+        <v>10178</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+698</t>
+          <t>+713</t>
         </is>
       </c>
     </row>
@@ -30299,11 +30299,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>9849</v>
+        <v>9864</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30314,11 +30314,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>9657</v>
+        <v>9672</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30329,11 +30329,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>11305</v>
+        <v>11330</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+896</t>
+          <t>+921</t>
         </is>
       </c>
     </row>
@@ -30344,11 +30344,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>10797</v>
+        <v>10812</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+716</t>
+          <t>+731</t>
         </is>
       </c>
     </row>
@@ -30359,11 +30359,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>10261</v>
+        <v>10276</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30374,11 +30374,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>9978</v>
+        <v>9993</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30389,11 +30389,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>9802</v>
+        <v>9817</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+680</t>
+          <t>+695</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:00:09
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -56,6 +56,7 @@
     <sheet name="2026-08-17" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="2026-08-18" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-08-19" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="2026-08-20" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -30406,6 +30407,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-20 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>29873</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>4399</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+488</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4254</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+428</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4265</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+432</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>11636</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>11044</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>10590</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+498</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10176</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>9965</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>12980</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+572</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>11999</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+526</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>11361</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>11034</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>13377</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+578</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>12723</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+556</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>12293</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>11919</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+496</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>11634</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>13794</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+534</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>13411</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+568</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10204</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+703</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>12103</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+534</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>12097</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+528</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>12845</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+502</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>12489</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>12160</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>11901</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>10636</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>10196</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+699</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>10189</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+695</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>10177</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+685</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>10181</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+695</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10180</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+689</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>8186</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>10156</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+685</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>8190</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+692</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>8239</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+740</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>8255</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+732</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8265</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+738</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>8259</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+736</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>8263</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+742</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>8189</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+674</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>11661</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+546</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>11124</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>10672</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+494</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>10354</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>10162</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>11902</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+572</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>11334</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+522</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>10776</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+500</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>10485</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+492</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10307</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+490</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:02:56
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -30437,11 +30437,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:00:08</t>
+          <t>Timestamp: 2026-08-20 13:02:55</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>29873</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:30:23
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -30437,11 +30437,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:02:55</t>
+          <t>Timestamp: 2026-08-20 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
@@ -30753,11 +30753,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>10204</v>
+        <v>10209</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+703</t>
+          <t>+708</t>
         </is>
       </c>
     </row>
@@ -30873,11 +30873,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>10196</v>
+        <v>10201</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+699</t>
+          <t>+704</t>
         </is>
       </c>
     </row>
@@ -30888,11 +30888,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>10189</v>
+        <v>10194</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+695</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
@@ -30903,11 +30903,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>10177</v>
+        <v>10182</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+685</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -30918,11 +30918,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>10181</v>
+        <v>10186</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+695</t>
+          <t>+700</t>
         </is>
       </c>
     </row>
@@ -30933,11 +30933,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>10180</v>
+        <v>10185</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+689</t>
+          <t>+694</t>
         </is>
       </c>
     </row>
@@ -30948,11 +30948,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>8186</v>
+        <v>8191</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30963,11 +30963,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>10156</v>
+        <v>10161</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+685</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -30978,11 +30978,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>8190</v>
+        <v>8195</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+692</t>
+          <t>+697</t>
         </is>
       </c>
     </row>
@@ -30993,11 +30993,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>8239</v>
+        <v>8244</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+740</t>
+          <t>+745</t>
         </is>
       </c>
     </row>
@@ -31008,11 +31008,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>8255</v>
+        <v>8260</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+732</t>
+          <t>+737</t>
         </is>
       </c>
     </row>
@@ -31023,11 +31023,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>8265</v>
+        <v>8270</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+738</t>
+          <t>+743</t>
         </is>
       </c>
     </row>
@@ -31038,11 +31038,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>8259</v>
+        <v>8264</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+736</t>
+          <t>+741</t>
         </is>
       </c>
     </row>
@@ -31053,11 +31053,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>8263</v>
+        <v>8268</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+742</t>
+          <t>+747</t>
         </is>
       </c>
     </row>
@@ -31068,11 +31068,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>8189</v>
+        <v>8194</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+674</t>
+          <t>+679</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 05:55:03
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -30437,11 +30437,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:33:10</t>
+          <t>Timestamp: 2026-08-20 13:55:02</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>75</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
@@ -30753,11 +30753,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>10209</v>
+        <v>10214</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+708</t>
+          <t>+713</t>
         </is>
       </c>
     </row>
@@ -30873,11 +30873,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>10201</v>
+        <v>10206</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+704</t>
+          <t>+709</t>
         </is>
       </c>
     </row>
@@ -30888,11 +30888,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>10194</v>
+        <v>10199</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30903,11 +30903,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>10182</v>
+        <v>10187</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+695</t>
         </is>
       </c>
     </row>
@@ -30918,11 +30918,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>10186</v>
+        <v>10191</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+700</t>
+          <t>+705</t>
         </is>
       </c>
     </row>
@@ -30933,11 +30933,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>10185</v>
+        <v>10190</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+694</t>
+          <t>+699</t>
         </is>
       </c>
     </row>
@@ -30948,11 +30948,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>8191</v>
+        <v>8196</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+705</t>
+          <t>+710</t>
         </is>
       </c>
     </row>
@@ -30963,11 +30963,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>10161</v>
+        <v>10166</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+695</t>
         </is>
       </c>
     </row>
@@ -30978,11 +30978,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>8195</v>
+        <v>8200</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+697</t>
+          <t>+702</t>
         </is>
       </c>
     </row>
@@ -30993,11 +30993,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>8244</v>
+        <v>8249</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+745</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -31008,11 +31008,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>8260</v>
+        <v>8265</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+737</t>
+          <t>+742</t>
         </is>
       </c>
     </row>
@@ -31023,11 +31023,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>8270</v>
+        <v>8275</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+743</t>
+          <t>+748</t>
         </is>
       </c>
     </row>
@@ -31038,11 +31038,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>8264</v>
+        <v>8269</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+741</t>
+          <t>+746</t>
         </is>
       </c>
     </row>
@@ -31053,11 +31053,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>8268</v>
+        <v>8273</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+747</t>
+          <t>+752</t>
         </is>
       </c>
     </row>
@@ -31068,11 +31068,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>8194</v>
+        <v>8199</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+679</t>
+          <t>+684</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -57,6 +57,7 @@
     <sheet name="2026-08-18" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="2026-08-19" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="2026-08-20" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="2026-08-21" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -31235,6 +31236,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-21 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>25944</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>4771</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+372</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4600</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+346</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4584</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+319</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>12235</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>11640</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+596</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>11178</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+588</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10756</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>10530</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+565</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>13585</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>12598</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>11941</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>11614</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>13980</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+603</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>13303</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>12858</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+565</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>12458</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+539</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>12105</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+471</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>14203</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+409</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>13980</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+569</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>10652</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+438</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>12518</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+415</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>12514</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+417</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>13446</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+601</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>13094</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>12750</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+590</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>12483</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+582</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>11191</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+555</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>10630</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+424</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>10623</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+424</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>10617</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+430</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>10617</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+426</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>10620</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+430</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>8584</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+388</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>10592</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+426</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>8582</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+382</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>8633</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>8647</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+382</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8651</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+376</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>8655</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+386</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>8649</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+376</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>8583</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+384</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>12260</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+599</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>11729</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>11268</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+596</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>10938</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+584</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>10742</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>12485</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+583</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>11939</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+605</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>11366</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+590</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>11071</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+586</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>10887</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+580</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:03:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -31266,11 +31266,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:00:10</t>
+          <t>Timestamp: 2026-08-21 13:03:08</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>25944</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:30:22
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -31266,11 +31266,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:03:08</t>
+          <t>Timestamp: 2026-08-21 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3">
@@ -31582,11 +31582,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>10652</v>
+        <v>10667</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+438</t>
+          <t>+453</t>
         </is>
       </c>
     </row>
@@ -31702,11 +31702,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>10630</v>
+        <v>10645</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+424</t>
+          <t>+439</t>
         </is>
       </c>
     </row>
@@ -31717,11 +31717,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>10623</v>
+        <v>10636</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+424</t>
+          <t>+437</t>
         </is>
       </c>
     </row>
@@ -31732,11 +31732,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>10617</v>
+        <v>10632</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+445</t>
         </is>
       </c>
     </row>
@@ -31747,11 +31747,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>10617</v>
+        <v>10632</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+426</t>
+          <t>+441</t>
         </is>
       </c>
     </row>
@@ -31762,11 +31762,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>10620</v>
+        <v>10635</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+430</t>
+          <t>+445</t>
         </is>
       </c>
     </row>
@@ -31777,11 +31777,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>8584</v>
+        <v>8599</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+388</t>
+          <t>+403</t>
         </is>
       </c>
     </row>
@@ -31792,11 +31792,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>10592</v>
+        <v>10607</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+426</t>
+          <t>+441</t>
         </is>
       </c>
     </row>
@@ -31807,11 +31807,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>8582</v>
+        <v>8597</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+382</t>
+          <t>+397</t>
         </is>
       </c>
     </row>
@@ -31822,11 +31822,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>8633</v>
+        <v>8648</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+384</t>
+          <t>+399</t>
         </is>
       </c>
     </row>
@@ -31837,11 +31837,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>8647</v>
+        <v>8662</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+382</t>
+          <t>+397</t>
         </is>
       </c>
     </row>
@@ -31852,11 +31852,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>8651</v>
+        <v>8666</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+376</t>
+          <t>+391</t>
         </is>
       </c>
     </row>
@@ -31867,11 +31867,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>8655</v>
+        <v>8670</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+386</t>
+          <t>+401</t>
         </is>
       </c>
     </row>
@@ -31882,11 +31882,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>8649</v>
+        <v>8664</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+376</t>
+          <t>+391</t>
         </is>
       </c>
     </row>
@@ -31897,11 +31897,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>8583</v>
+        <v>8598</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+384</t>
+          <t>+399</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-21 05:56:30
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -31266,11 +31266,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-21 13:33:22</t>
+          <t>Timestamp: 2026-08-21 13:56:29</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>223</v>
+        <v>505</v>
       </c>
     </row>
     <row r="3">
@@ -31297,11 +31297,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>4771</v>
+        <v>4792</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+372</t>
+          <t>+393</t>
         </is>
       </c>
     </row>
@@ -31312,11 +31312,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>4600</v>
+        <v>4621</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+346</t>
+          <t>+367</t>
         </is>
       </c>
     </row>
@@ -31327,11 +31327,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4584</v>
+        <v>4599</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+319</t>
+          <t>+334</t>
         </is>
       </c>
     </row>
@@ -31582,11 +31582,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>10667</v>
+        <v>10682</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+453</t>
+          <t>+468</t>
         </is>
       </c>
     </row>
@@ -31702,11 +31702,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>10645</v>
+        <v>10660</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+439</t>
+          <t>+454</t>
         </is>
       </c>
     </row>
@@ -31717,11 +31717,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>10636</v>
+        <v>10651</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+437</t>
+          <t>+452</t>
         </is>
       </c>
     </row>
@@ -31732,11 +31732,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>10632</v>
+        <v>10647</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+445</t>
+          <t>+460</t>
         </is>
       </c>
     </row>
@@ -31747,11 +31747,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>10632</v>
+        <v>10647</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+441</t>
+          <t>+456</t>
         </is>
       </c>
     </row>
@@ -31762,11 +31762,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>10635</v>
+        <v>10650</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+445</t>
+          <t>+460</t>
         </is>
       </c>
     </row>
@@ -31777,11 +31777,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>8599</v>
+        <v>8614</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+403</t>
+          <t>+418</t>
         </is>
       </c>
     </row>
@@ -31792,11 +31792,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>10607</v>
+        <v>10622</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+441</t>
+          <t>+456</t>
         </is>
       </c>
     </row>
@@ -31807,11 +31807,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>8597</v>
+        <v>8612</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+397</t>
+          <t>+412</t>
         </is>
       </c>
     </row>
@@ -31822,11 +31822,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>8648</v>
+        <v>8663</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+399</t>
+          <t>+414</t>
         </is>
       </c>
     </row>
@@ -31837,11 +31837,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>8662</v>
+        <v>8677</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+397</t>
+          <t>+412</t>
         </is>
       </c>
     </row>
@@ -31852,11 +31852,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>8666</v>
+        <v>8681</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+391</t>
+          <t>+406</t>
         </is>
       </c>
     </row>
@@ -31867,11 +31867,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>8670</v>
+        <v>8685</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+401</t>
+          <t>+416</t>
         </is>
       </c>
     </row>
@@ -31882,11 +31882,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>8664</v>
+        <v>8679</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+391</t>
+          <t>+406</t>
         </is>
       </c>
     </row>
@@ -31897,11 +31897,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>8598</v>
+        <v>8613</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+399</t>
+          <t>+414</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-22 05:26:31
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -32095,11 +32095,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-22 13:00:10</t>
+          <t>Timestamp: 2026-08-22 13:26:28</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>32158</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:00:09
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -59,6 +59,7 @@
     <sheet name="2026-08-20" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="2026-08-21" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-08-22" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="2026-08-23" sheetId="54" state="visible" r:id="rId54"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -32893,6 +32894,834 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-23 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>68982</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>6137</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1027</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>6011</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1104</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>5999</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1114</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>14090</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+1210</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>13467</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1182</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>12978</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1170</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>12556</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1170</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>12228</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>15495</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1265</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>14423</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1180</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>13730</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1144</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>13353</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1106</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>15935</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1310</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>15238</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1290</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>14749</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1246</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>14306</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1218</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>13883</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1148</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>16240</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1394</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>15935</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1310</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>12986</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1671</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>14447</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1284</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>14511</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1354</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>15333</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1242</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>14945</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1206</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>14585</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1190</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>14297</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1178</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>12891</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1070</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>12982</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1689</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>13006</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1712</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>12990</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1698</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>13009</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1717</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>12946</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1651</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>10935</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1676</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>12938</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+1673</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>10986</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1729</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>11002</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1694</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>10985</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1663</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>11040</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+1714</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>11043</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1713</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>11042</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1718</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>10974</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1716</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>14171</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1266</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>13596</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1222</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>13103</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1190</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>12758</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1190</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>12562</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+1190</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>14456</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+1326</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>13890</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1306</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>13281</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1270</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>12922</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1206</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>12710</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1190</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-23 05:30:20
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -32924,11 +32924,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-23 13:00:08</t>
+          <t>Timestamp: 2026-08-23 13:30:19</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>68982</v>
+        <v>980</v>
       </c>
     </row>
     <row r="3">
@@ -33075,11 +33075,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>15495</v>
+        <v>15545</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1265</t>
+          <t>+1315</t>
         </is>
       </c>
     </row>
@@ -33135,11 +33135,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>15935</v>
+        <v>15965</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1310</t>
+          <t>+1340</t>
         </is>
       </c>
     </row>
@@ -33240,11 +33240,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>12986</v>
+        <v>13036</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+1671</t>
+          <t>+1721</t>
         </is>
       </c>
     </row>
@@ -33270,11 +33270,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>14511</v>
+        <v>14561</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+1354</t>
+          <t>+1404</t>
         </is>
       </c>
     </row>
@@ -33360,11 +33360,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>12982</v>
+        <v>13032</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+1689</t>
+          <t>+1739</t>
         </is>
       </c>
     </row>
@@ -33375,11 +33375,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>13006</v>
+        <v>13056</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1712</t>
+          <t>+1762</t>
         </is>
       </c>
     </row>
@@ -33390,11 +33390,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>12990</v>
+        <v>13040</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1698</t>
+          <t>+1748</t>
         </is>
       </c>
     </row>
@@ -33405,11 +33405,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>13009</v>
+        <v>13059</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1717</t>
+          <t>+1767</t>
         </is>
       </c>
     </row>
@@ -33420,11 +33420,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>12946</v>
+        <v>12996</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1651</t>
+          <t>+1701</t>
         </is>
       </c>
     </row>
@@ -33435,11 +33435,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>10935</v>
+        <v>10985</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+1676</t>
+          <t>+1726</t>
         </is>
       </c>
     </row>
@@ -33450,11 +33450,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>12938</v>
+        <v>12988</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+1673</t>
+          <t>+1723</t>
         </is>
       </c>
     </row>
@@ -33465,11 +33465,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>10986</v>
+        <v>11036</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1729</t>
+          <t>+1779</t>
         </is>
       </c>
     </row>
@@ -33480,11 +33480,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>11002</v>
+        <v>11052</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+1694</t>
+          <t>+1744</t>
         </is>
       </c>
     </row>
@@ -33495,11 +33495,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>10985</v>
+        <v>11035</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1663</t>
+          <t>+1713</t>
         </is>
       </c>
     </row>
@@ -33510,11 +33510,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>11040</v>
+        <v>11090</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+1714</t>
+          <t>+1764</t>
         </is>
       </c>
     </row>
@@ -33525,11 +33525,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>11043</v>
+        <v>11093</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1713</t>
+          <t>+1763</t>
         </is>
       </c>
     </row>
@@ -33540,11 +33540,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>11042</v>
+        <v>11092</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1718</t>
+          <t>+1768</t>
         </is>
       </c>
     </row>
@@ -33555,11 +33555,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>10974</v>
+        <v>11024</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1716</t>
+          <t>+1766</t>
         </is>
       </c>
     </row>
@@ -33645,11 +33645,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>14456</v>
+        <v>14506</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+1326</t>
+          <t>+1376</t>
         </is>
       </c>
     </row>
@@ -33660,11 +33660,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>13890</v>
+        <v>13940</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+1306</t>
+          <t>+1356</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:00:09
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -60,6 +60,7 @@
     <sheet name="2026-08-21" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="2026-08-22" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-08-23" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="2026-08-24" sheetId="55" state="visible" r:id="rId55"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -33722,6 +33723,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-24 13:00:08</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>95087</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7270</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1133</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>7274</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1263</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>7271</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1272</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>220</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>15966</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+1876</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>15327</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+1860</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>14826</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+1848</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>14396</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>14068</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>17275</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+1730</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>16133</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+1710</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>15420</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1690</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>15043</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+1690</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>17875</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+1910</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>17148</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+1910</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>16643</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+1894</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>16196</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+1890</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>15773</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+1890</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>18084</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1844</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>17775</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>15013</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1977</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>16277</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+1830</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>16407</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+1846</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>17173</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>16785</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>16425</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>16137</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+1840</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>14581</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+1690</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>15037</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>15093</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+2037</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>15034</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+1994</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>15080</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>15030</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+2034</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>13023</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+2038</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>14987</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1999</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>13081</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+2045</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>13074</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>13082</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+2047</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>13057</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1967</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>13134</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+2041</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>13091</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1999</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>13061</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+2037</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>15981</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+1810</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>15406</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1810</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>14893</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+1790</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>14548</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+1790</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>14352</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+1790</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>16316</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+1810</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>15738</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+1798</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>15071</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+1790</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>14712</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+1790</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>14500</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1790</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:10:01
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -33753,11 +33753,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:00:08</t>
+          <t>Timestamp: 2026-08-24 13:10:00</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>95087</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -33829,7 +33829,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>220</v>
+        <v>251</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-24 05:30:23
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -33753,11 +33753,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-24 13:10:00</t>
+          <t>Timestamp: 2026-08-24 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>31</v>
+        <v>596</v>
       </c>
     </row>
     <row r="3">
@@ -33829,7 +33829,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>251</v>
+        <v>276</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -33919,11 +33919,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>17275</v>
+        <v>17300</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>+1730</t>
+          <t>+1755</t>
         </is>
       </c>
     </row>
@@ -33934,11 +33934,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>16133</v>
+        <v>16158</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>+1710</t>
+          <t>+1735</t>
         </is>
       </c>
     </row>
@@ -33949,11 +33949,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>15420</v>
+        <v>15445</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>+1690</t>
+          <t>+1715</t>
         </is>
       </c>
     </row>
@@ -33964,11 +33964,11 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>15043</v>
+        <v>15068</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>+1690</t>
+          <t>+1715</t>
         </is>
       </c>
     </row>
@@ -34054,11 +34054,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>18084</v>
+        <v>18109</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+1844</t>
+          <t>+1869</t>
         </is>
       </c>
     </row>
@@ -34084,11 +34084,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>15013</v>
+        <v>15038</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1977</t>
+          <t>+2002</t>
         </is>
       </c>
     </row>
@@ -34114,11 +34114,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>16407</v>
+        <v>16432</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+1846</t>
+          <t>+1871</t>
         </is>
       </c>
     </row>
@@ -34204,11 +34204,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>15037</v>
+        <v>15062</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+2005</t>
+          <t>+2030</t>
         </is>
       </c>
     </row>
@@ -34219,11 +34219,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>15093</v>
+        <v>15118</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+2037</t>
+          <t>+2062</t>
         </is>
       </c>
     </row>
@@ -34234,11 +34234,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>15034</v>
+        <v>15059</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1994</t>
+          <t>+2019</t>
         </is>
       </c>
     </row>
@@ -34249,11 +34249,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>15080</v>
+        <v>15105</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+2021</t>
+          <t>+2046</t>
         </is>
       </c>
     </row>
@@ -34264,11 +34264,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>15030</v>
+        <v>15055</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+2034</t>
+          <t>+2059</t>
         </is>
       </c>
     </row>
@@ -34279,11 +34279,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>13023</v>
+        <v>13048</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2038</t>
+          <t>+2063</t>
         </is>
       </c>
     </row>
@@ -34294,11 +34294,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>14987</v>
+        <v>15012</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1999</t>
+          <t>+2024</t>
         </is>
       </c>
     </row>
@@ -34309,11 +34309,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>13081</v>
+        <v>13106</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+2045</t>
+          <t>+2070</t>
         </is>
       </c>
     </row>
@@ -34324,11 +34324,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>13074</v>
+        <v>13099</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+2022</t>
+          <t>+2047</t>
         </is>
       </c>
     </row>
@@ -34339,11 +34339,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>13082</v>
+        <v>13107</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+2047</t>
+          <t>+2072</t>
         </is>
       </c>
     </row>
@@ -34354,11 +34354,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>13057</v>
+        <v>13082</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1967</t>
+          <t>+1992</t>
         </is>
       </c>
     </row>
@@ -34369,11 +34369,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>13134</v>
+        <v>13159</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+2041</t>
+          <t>+2066</t>
         </is>
       </c>
     </row>
@@ -34384,11 +34384,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>13091</v>
+        <v>13116</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1999</t>
+          <t>+2024</t>
         </is>
       </c>
     </row>
@@ -34399,11 +34399,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>13061</v>
+        <v>13086</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+2037</t>
+          <t>+2062</t>
         </is>
       </c>
     </row>
@@ -34489,11 +34489,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>16316</v>
+        <v>16331</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+1810</t>
+          <t>+1825</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:00:08
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -61,6 +61,7 @@
     <sheet name="2026-08-22" sheetId="53" state="visible" r:id="rId53"/>
     <sheet name="2026-08-23" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-08-24" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="2026-08-25" sheetId="56" state="visible" r:id="rId56"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -34566,6 +34567,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-25 13:00:07</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>47702</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7796</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+526</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>7796</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+522</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>7799</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+528</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1149</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+873</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>16956</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>16312</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+985</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>15791</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>15361</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>15033</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>18290</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>17148</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+990</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>16430</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+985</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>16033</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>18850</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+975</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>18113</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>17608</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>17136</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>16713</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>19109</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>18775</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>16071</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1033</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>17077</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+800</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>17226</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+794</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>18173</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>17772</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+987</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>17390</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>17077</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+940</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>15546</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+965</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>16093</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1031</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>16130</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+1012</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>15992</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+933</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>16042</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+937</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>16086</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+1031</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>13854</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+806</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>15962</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+950</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>14139</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1033</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>14132</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+1033</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>14087</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+980</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>14069</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+987</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>14188</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1029</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>14151</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1035</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>14090</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+1004</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>16773</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+792</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>16196</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>15683</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>15323</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+775</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>15117</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+765</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>17121</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>16528</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+790</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>15836</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+765</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>15477</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+765</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>15265</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+765</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:06:28
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -34597,11 +34597,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:00:07</t>
+          <t>Timestamp: 2026-08-25 13:06:27</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>47702</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-25 05:56:33
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -34597,11 +34597,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-25 13:36:40</t>
+          <t>Timestamp: 2026-08-25 13:56:32</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>356</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3">
@@ -34628,11 +34628,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>7811</v>
+        <v>7826</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+541</t>
+          <t>+556</t>
         </is>
       </c>
     </row>
@@ -34643,11 +34643,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7811</v>
+        <v>7826</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+537</t>
+          <t>+552</t>
         </is>
       </c>
     </row>
@@ -34658,11 +34658,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7814</v>
+        <v>7829</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+558</t>
         </is>
       </c>
     </row>
@@ -34673,11 +34673,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1154</v>
+        <v>1159</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+878</t>
+          <t>+883</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -62,6 +62,7 @@
     <sheet name="2026-08-23" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="2026-08-24" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-08-25" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="2026-08-26" sheetId="57" state="visible" r:id="rId57"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -35410,6 +35411,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-26 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>24923</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>8164</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+338</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>8165</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+339</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>8158</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+329</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1463</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+304</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>17432</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+476</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>16782</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>16257</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+466</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>15821</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>15493</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>18745</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+455</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>17589</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+441</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>16865</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+435</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>16468</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+435</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>19345</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>18608</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>18088</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>17606</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>17173</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>19589</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>19255</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>16610</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+524</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>17572</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>17719</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+478</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>18653</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>18252</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>17860</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>17537</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>15981</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+435</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>16644</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+536</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>16669</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+524</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>16527</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+520</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>16585</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+528</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>16563</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+462</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>14395</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+526</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>16503</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+526</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>14656</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+502</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>14683</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+536</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>14566</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+464</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>14616</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+532</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>14733</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+530</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>14694</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+528</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>14639</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+534</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>17268</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>16679</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>16155</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+472</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>15793</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>15577</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>17604</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>17008</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+480</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>16308</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+472</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>15947</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+470</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>15725</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+460</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:28:37
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -35441,11 +35441,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-26 13:00:09</t>
+          <t>Timestamp: 2026-08-26 13:28:36</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>24923</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3">
@@ -35742,11 +35742,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>19589</v>
+        <v>19604</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>
@@ -35772,11 +35772,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>16610</v>
+        <v>16625</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+524</t>
+          <t>+539</t>
         </is>
       </c>
     </row>
@@ -35787,11 +35787,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>17572</v>
+        <v>17587</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>
@@ -35892,11 +35892,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>16644</v>
+        <v>16659</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+536</t>
+          <t>+551</t>
         </is>
       </c>
     </row>
@@ -35907,11 +35907,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>16669</v>
+        <v>16684</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+524</t>
+          <t>+539</t>
         </is>
       </c>
     </row>
@@ -35922,11 +35922,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>16527</v>
+        <v>16542</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+520</t>
+          <t>+535</t>
         </is>
       </c>
     </row>
@@ -35937,11 +35937,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>16585</v>
+        <v>16600</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+543</t>
         </is>
       </c>
     </row>
@@ -35952,11 +35952,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>16563</v>
+        <v>16578</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+462</t>
+          <t>+477</t>
         </is>
       </c>
     </row>
@@ -35967,11 +35967,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>14395</v>
+        <v>14410</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+541</t>
         </is>
       </c>
     </row>
@@ -35982,11 +35982,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>16503</v>
+        <v>16518</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+526</t>
+          <t>+541</t>
         </is>
       </c>
     </row>
@@ -35997,11 +35997,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>14656</v>
+        <v>14671</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+502</t>
+          <t>+517</t>
         </is>
       </c>
     </row>
@@ -36012,11 +36012,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>14683</v>
+        <v>14698</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+536</t>
+          <t>+551</t>
         </is>
       </c>
     </row>
@@ -36027,11 +36027,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>14566</v>
+        <v>14581</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+464</t>
+          <t>+479</t>
         </is>
       </c>
     </row>
@@ -36042,11 +36042,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>14616</v>
+        <v>14631</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+532</t>
+          <t>+547</t>
         </is>
       </c>
     </row>
@@ -36057,11 +36057,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>14733</v>
+        <v>14748</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+530</t>
+          <t>+545</t>
         </is>
       </c>
     </row>
@@ -36072,11 +36072,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>14694</v>
+        <v>14709</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+528</t>
+          <t>+543</t>
         </is>
       </c>
     </row>
@@ -36087,11 +36087,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>14639</v>
+        <v>14654</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+534</t>
+          <t>+549</t>
         </is>
       </c>
     </row>
@@ -36102,11 +36102,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>17268</v>
+        <v>17283</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>
@@ -36117,11 +36117,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>16679</v>
+        <v>16694</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:30:25
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -35441,11 +35441,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-26 13:28:36</t>
+          <t>Timestamp: 2026-08-26 13:30:24</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>285</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3">
@@ -35757,11 +35757,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>19255</v>
+        <v>19270</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>
@@ -35802,11 +35802,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>17719</v>
+        <v>17734</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+478</t>
+          <t>+493</t>
         </is>
       </c>
     </row>
@@ -35817,11 +35817,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>18653</v>
+        <v>18668</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>
@@ -35832,11 +35832,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>18252</v>
+        <v>18267</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>
@@ -36132,11 +36132,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>16155</v>
+        <v>16170</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+472</t>
+          <t>+487</t>
         </is>
       </c>
     </row>
@@ -36147,11 +36147,11 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>15793</v>
+        <v>15808</v>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+485</t>
         </is>
       </c>
     </row>
@@ -36162,11 +36162,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>15577</v>
+        <v>15592</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+460</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -36177,11 +36177,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>17604</v>
+        <v>17619</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+480</t>
+          <t>+495</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-26 05:58:53
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -35441,11 +35441,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-26 13:30:24</t>
+          <t>Timestamp: 2026-08-26 13:58:51</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>405</v>
+        <v>825</v>
       </c>
     </row>
     <row r="3">
@@ -35517,11 +35517,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1463</v>
+        <v>1583</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+304</t>
+          <t>+424</t>
         </is>
       </c>
     </row>
@@ -35532,11 +35532,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>17432</v>
+        <v>17447</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+476</t>
+          <t>+491</t>
         </is>
       </c>
     </row>
@@ -35547,11 +35547,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>16782</v>
+        <v>16797</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+470</t>
+          <t>+485</t>
         </is>
       </c>
     </row>
@@ -35562,11 +35562,11 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>16257</v>
+        <v>16272</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>+466</t>
+          <t>+481</t>
         </is>
       </c>
     </row>
@@ -35577,11 +35577,11 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>15821</v>
+        <v>15836</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>+460</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -35592,11 +35592,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>15493</v>
+        <v>15508</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+460</t>
+          <t>+475</t>
         </is>
       </c>
     </row>
@@ -35772,11 +35772,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>16625</v>
+        <v>16640</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+539</t>
+          <t>+554</t>
         </is>
       </c>
     </row>
@@ -35892,11 +35892,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>16659</v>
+        <v>16674</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+566</t>
         </is>
       </c>
     </row>
@@ -35907,11 +35907,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>16684</v>
+        <v>16699</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+539</t>
+          <t>+554</t>
         </is>
       </c>
     </row>
@@ -35922,11 +35922,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>16542</v>
+        <v>16557</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+535</t>
+          <t>+550</t>
         </is>
       </c>
     </row>
@@ -35937,11 +35937,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>16600</v>
+        <v>16615</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+558</t>
         </is>
       </c>
     </row>
@@ -35952,11 +35952,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>16578</v>
+        <v>16593</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+477</t>
+          <t>+492</t>
         </is>
       </c>
     </row>
@@ -35967,11 +35967,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>14410</v>
+        <v>14425</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+541</t>
+          <t>+556</t>
         </is>
       </c>
     </row>
@@ -35982,11 +35982,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>16518</v>
+        <v>16533</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+541</t>
+          <t>+556</t>
         </is>
       </c>
     </row>
@@ -35997,11 +35997,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>14671</v>
+        <v>14686</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+517</t>
+          <t>+532</t>
         </is>
       </c>
     </row>
@@ -36012,11 +36012,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>14698</v>
+        <v>14713</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+551</t>
+          <t>+566</t>
         </is>
       </c>
     </row>
@@ -36027,11 +36027,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>14581</v>
+        <v>14596</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+479</t>
+          <t>+494</t>
         </is>
       </c>
     </row>
@@ -36042,11 +36042,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>14631</v>
+        <v>14646</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+547</t>
+          <t>+562</t>
         </is>
       </c>
     </row>
@@ -36057,11 +36057,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>14748</v>
+        <v>14763</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+545</t>
+          <t>+560</t>
         </is>
       </c>
     </row>
@@ -36072,11 +36072,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>14709</v>
+        <v>14724</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+543</t>
+          <t>+558</t>
         </is>
       </c>
     </row>
@@ -36087,11 +36087,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>14654</v>
+        <v>14669</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+549</t>
+          <t>+564</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 05:00:14
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -63,6 +63,7 @@
     <sheet name="2026-08-24" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="2026-08-25" sheetId="56" state="visible" r:id="rId56"/>
     <sheet name="2026-08-26" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="2026-08-27" sheetId="58" state="visible" r:id="rId58"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -36254,6 +36255,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-27 13:00:13</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>37815</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>8910</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+746</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>8900</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+735</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>8904</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+746</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2119</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+536</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>18107</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>17457</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>16932</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>16496</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>16168</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+660</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>19420</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>18264</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>17540</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>17143</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>19975</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>19238</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+630</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>18703</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+615</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>18221</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+615</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>17788</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+615</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>20293</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+689</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>19945</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>17524</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+884</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>18260</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+673</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>18397</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+663</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>19343</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>18942</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>18535</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>18209</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+672</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>16644</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+663</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>17564</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+890</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>17465</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+766</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>17361</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+804</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>17481</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+866</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>17487</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+894</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>15179</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+754</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>17407</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+874</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>15546</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+860</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>15587</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+874</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>15398</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+802</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>15450</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+804</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>15453</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>15592</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+868</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>15351</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+682</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>17958</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>17369</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>16845</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>16483</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>16267</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>18294</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>17683</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>16983</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>16622</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>16400</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-27 05:30:30
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -36285,11 +36285,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-27 13:00:13</t>
+          <t>Timestamp: 2026-08-27 13:30:29</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>37815</v>
+        <v>487</v>
       </c>
     </row>
     <row r="3">
@@ -36586,11 +36586,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>20293</v>
+        <v>20308</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+689</t>
+          <t>+704</t>
         </is>
       </c>
     </row>
@@ -36601,11 +36601,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>19945</v>
+        <v>19960</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -36616,11 +36616,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>17524</v>
+        <v>17543</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+884</t>
+          <t>+903</t>
         </is>
       </c>
     </row>
@@ -36631,11 +36631,11 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>18260</v>
+        <v>18275</v>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>+673</t>
+          <t>+688</t>
         </is>
       </c>
     </row>
@@ -36646,11 +36646,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>18397</v>
+        <v>18412</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+663</t>
+          <t>+678</t>
         </is>
       </c>
     </row>
@@ -36661,11 +36661,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>19343</v>
+        <v>19358</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -36676,11 +36676,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>18942</v>
+        <v>18957</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -36691,11 +36691,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>18535</v>
+        <v>18550</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -36736,11 +36736,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>17564</v>
+        <v>17581</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+890</t>
+          <t>+907</t>
         </is>
       </c>
     </row>
@@ -36751,11 +36751,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>17465</v>
+        <v>17484</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+766</t>
+          <t>+785</t>
         </is>
       </c>
     </row>
@@ -36766,11 +36766,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>17361</v>
+        <v>17380</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+804</t>
+          <t>+823</t>
         </is>
       </c>
     </row>
@@ -36781,11 +36781,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>17481</v>
+        <v>17500</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+866</t>
+          <t>+885</t>
         </is>
       </c>
     </row>
@@ -36796,11 +36796,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>17487</v>
+        <v>17508</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+894</t>
+          <t>+915</t>
         </is>
       </c>
     </row>
@@ -36811,11 +36811,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>15179</v>
+        <v>15194</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+754</t>
+          <t>+769</t>
         </is>
       </c>
     </row>
@@ -36826,11 +36826,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>17407</v>
+        <v>17428</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+874</t>
+          <t>+895</t>
         </is>
       </c>
     </row>
@@ -36841,11 +36841,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>15546</v>
+        <v>15563</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+860</t>
+          <t>+877</t>
         </is>
       </c>
     </row>
@@ -36856,11 +36856,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>15587</v>
+        <v>15606</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+874</t>
+          <t>+893</t>
         </is>
       </c>
     </row>
@@ -36871,11 +36871,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>15398</v>
+        <v>15417</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+802</t>
+          <t>+821</t>
         </is>
       </c>
     </row>
@@ -36886,11 +36886,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>15450</v>
+        <v>15467</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+804</t>
+          <t>+821</t>
         </is>
       </c>
     </row>
@@ -36901,11 +36901,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>15453</v>
+        <v>15474</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+690</t>
+          <t>+711</t>
         </is>
       </c>
     </row>
@@ -36916,11 +36916,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>15592</v>
+        <v>15613</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+868</t>
+          <t>+889</t>
         </is>
       </c>
     </row>
@@ -36931,11 +36931,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>15351</v>
+        <v>15370</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+682</t>
+          <t>+701</t>
         </is>
       </c>
     </row>
@@ -36946,11 +36946,11 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>17958</v>
+        <v>17973</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -36961,11 +36961,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>17369</v>
+        <v>17384</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -36976,11 +36976,11 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>16845</v>
+        <v>16848</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+678</t>
         </is>
       </c>
     </row>
@@ -37021,11 +37021,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>18294</v>
+        <v>18309</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -37036,11 +37036,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>17683</v>
+        <v>17698</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -37051,11 +37051,11 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>16983</v>
+        <v>16998</v>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -37066,11 +37066,11 @@
         </is>
       </c>
       <c r="B54" s="5" t="n">
-        <v>16622</v>
+        <v>16637</v>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -37081,11 +37081,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>16400</v>
+        <v>16406</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+675</t>
+          <t>+681</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-28 05:30:24
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -37129,11 +37129,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-28 13:00:10</t>
+          <t>Timestamp: 2026-08-28 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>38958</v>
+        <v>420</v>
       </c>
     </row>
     <row r="3">
@@ -37460,11 +37460,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>18598</v>
+        <v>18623</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1055</t>
+          <t>+1080</t>
         </is>
       </c>
     </row>
@@ -37490,11 +37490,11 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>19104</v>
+        <v>19129</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>+692</t>
+          <t>+717</t>
         </is>
       </c>
     </row>
@@ -37580,11 +37580,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>18642</v>
+        <v>18667</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1061</t>
+          <t>+1086</t>
         </is>
       </c>
     </row>
@@ -37595,11 +37595,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>18443</v>
+        <v>18468</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+959</t>
+          <t>+984</t>
         </is>
       </c>
     </row>
@@ -37610,11 +37610,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>18293</v>
+        <v>18318</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+913</t>
+          <t>+938</t>
         </is>
       </c>
     </row>
@@ -37625,11 +37625,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>18573</v>
+        <v>18598</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1073</t>
+          <t>+1098</t>
         </is>
       </c>
     </row>
@@ -37640,11 +37640,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>18406</v>
+        <v>18431</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+898</t>
+          <t>+923</t>
         </is>
       </c>
     </row>
@@ -37655,11 +37655,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>16147</v>
+        <v>16172</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+953</t>
+          <t>+978</t>
         </is>
       </c>
     </row>
@@ -37670,11 +37670,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>18443</v>
+        <v>18468</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1015</t>
+          <t>+1040</t>
         </is>
       </c>
     </row>
@@ -37685,11 +37685,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>16540</v>
+        <v>16565</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+977</t>
+          <t>+1002</t>
         </is>
       </c>
     </row>
@@ -37700,11 +37700,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>16526</v>
+        <v>16551</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+920</t>
+          <t>+945</t>
         </is>
       </c>
     </row>
@@ -37715,11 +37715,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>16378</v>
+        <v>16403</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+961</t>
+          <t>+986</t>
         </is>
       </c>
     </row>
@@ -37730,11 +37730,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>16411</v>
+        <v>16436</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+944</t>
+          <t>+969</t>
         </is>
       </c>
     </row>
@@ -37745,11 +37745,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>16391</v>
+        <v>16416</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+917</t>
+          <t>+942</t>
         </is>
       </c>
     </row>
@@ -37760,11 +37760,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>16640</v>
+        <v>16665</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1027</t>
+          <t>+1052</t>
         </is>
       </c>
     </row>
@@ -37775,11 +37775,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>16363</v>
+        <v>16388</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+993</t>
+          <t>+1018</t>
         </is>
       </c>
     </row>
@@ -37865,11 +37865,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>18979</v>
+        <v>18999</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+670</t>
+          <t>+690</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:00:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -65,6 +65,7 @@
     <sheet name="2026-08-26" sheetId="57" state="visible" r:id="rId57"/>
     <sheet name="2026-08-27" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="2026-08-28" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="2026-08-29" sheetId="60" state="visible" r:id="rId60"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -38814,6 +38815,849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-29 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>39798</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>9891</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+475</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>9904</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+491</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>9908</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+491</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>3020</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+331</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>19432</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>18768</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>18237</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>17801</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>17473</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>20782</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+690</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>19603</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>18875</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>18478</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>21316</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>20573</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>20038</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>19556</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>19123</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>21828</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+760</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>21374</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+706</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>19732</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+1109</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>19670</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+732</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>19826</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+697</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>20750</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>20347</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>19940</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>19599</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>17979</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>19742</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>19459</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+991</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>19197</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+879</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>19673</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>+1075</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>19382</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+951</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>17022</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+850</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>19470</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+1002</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>17574</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+1009</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>17528</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+977</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>17272</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+869</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>17543</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+1107</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>17427</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+1011</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>17680</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+1015</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>17265</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+877</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>19296</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>18699</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>18163</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>17798</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+700</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>17578</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+696</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>19684</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+685</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>19037</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+677</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>18333</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>17972</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>17741</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:12:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -38845,11 +38845,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-29 13:00:11</t>
+          <t>Timestamp: 2026-08-29 13:12:11</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>39798</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:30:23
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -38845,11 +38845,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-29 13:12:11</t>
+          <t>Timestamp: 2026-08-29 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0</v>
+        <v>746</v>
       </c>
     </row>
     <row r="3">
@@ -39176,11 +39176,11 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>19732</v>
+        <v>19782</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>+1109</t>
+          <t>+1159</t>
         </is>
       </c>
     </row>
@@ -39296,11 +39296,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>19742</v>
+        <v>19792</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1125</t>
         </is>
       </c>
     </row>
@@ -39311,11 +39311,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>19459</v>
+        <v>19509</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+991</t>
+          <t>+1041</t>
         </is>
       </c>
     </row>
@@ -39326,11 +39326,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>19197</v>
+        <v>19247</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+879</t>
+          <t>+929</t>
         </is>
       </c>
     </row>
@@ -39341,11 +39341,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>19673</v>
+        <v>19723</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+1075</t>
+          <t>+1125</t>
         </is>
       </c>
     </row>
@@ -39356,11 +39356,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>19382</v>
+        <v>19432</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+951</t>
+          <t>+1001</t>
         </is>
       </c>
     </row>
@@ -39371,11 +39371,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>17022</v>
+        <v>17072</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+850</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -39386,11 +39386,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>19470</v>
+        <v>19520</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1002</t>
+          <t>+1052</t>
         </is>
       </c>
     </row>
@@ -39401,11 +39401,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>17574</v>
+        <v>17624</v>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>+1009</t>
+          <t>+1059</t>
         </is>
       </c>
     </row>
@@ -39416,11 +39416,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>17528</v>
+        <v>17574</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+977</t>
+          <t>+1023</t>
         </is>
       </c>
     </row>
@@ -39431,11 +39431,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>17272</v>
+        <v>17322</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+869</t>
+          <t>+919</t>
         </is>
       </c>
     </row>
@@ -39446,11 +39446,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>17543</v>
+        <v>17593</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+1107</t>
+          <t>+1157</t>
         </is>
       </c>
     </row>
@@ -39461,11 +39461,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>17427</v>
+        <v>17477</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1011</t>
+          <t>+1061</t>
         </is>
       </c>
     </row>
@@ -39476,11 +39476,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>17680</v>
+        <v>17730</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+1015</t>
+          <t>+1065</t>
         </is>
       </c>
     </row>
@@ -39491,11 +39491,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>17265</v>
+        <v>17315</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+877</t>
+          <t>+927</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 05:42:27
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -38845,11 +38845,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-29 13:30:22</t>
+          <t>Timestamp: 2026-08-29 13:42:26</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>746</v>
+        <v>1616</v>
       </c>
     </row>
     <row r="3">
@@ -38876,11 +38876,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>9891</v>
+        <v>9961</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+475</t>
+          <t>+545</t>
         </is>
       </c>
     </row>
@@ -38891,11 +38891,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>9904</v>
+        <v>9974</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+561</t>
         </is>
       </c>
     </row>
@@ -38906,11 +38906,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>9908</v>
+        <v>9978</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>+491</t>
+          <t>+561</t>
         </is>
       </c>
     </row>
@@ -38921,11 +38921,11 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>3020</v>
+        <v>3670</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>+331</t>
+          <t>+981</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-01 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -68,6 +68,7 @@
     <sheet name="2026-08-29" sheetId="60" state="visible" r:id="rId60"/>
     <sheet name="2026-08-30" sheetId="61" state="visible" r:id="rId61"/>
     <sheet name="2026-08-31" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="2026-09-01" sheetId="63" state="visible" r:id="rId63"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -41436,6 +41437,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S63</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-01 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>13754</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>13516</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>14031</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>7120</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>21042</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>20378</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>19839</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>19371</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>19043</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>22552</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>21353</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>20625</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>20232</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>23040</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>22293</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>21758</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>21256</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>20823</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>23540</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>23100</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>34988</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>33639</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>34373</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>22431</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>22037</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>21600</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>21279</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>19745</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>32506</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>32489</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>32779</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>33156</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>31737</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>29391</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>33199</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>33987</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>31731</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>31145</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>28805</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>31735</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>31852</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>29657</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>21146</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>20540</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>20013</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>19639</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>19408</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>21565</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>20898</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>20203</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>19814</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>19571</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>13839</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>13482</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>13481</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 05:00:13
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -69,6 +69,7 @@
     <sheet name="2026-08-30" sheetId="61" state="visible" r:id="rId61"/>
     <sheet name="2026-08-31" sheetId="62" state="visible" r:id="rId62"/>
     <sheet name="2026-09-01" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="2026-09-02" sheetId="64" state="visible" r:id="rId64"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -42325,6 +42326,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-02 13:00:11</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>274</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>214</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>186</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-02 05:30:27
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -42356,11 +42356,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-02 13:00:11</t>
+          <t>Timestamp: 2026-09-02 13:30:26</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>674</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-03 05:30:26
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -43245,11 +43245,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-03 13:00:10</t>
+          <t>Timestamp: 2026-09-03 13:30:25</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>34544</v>
+        <v>433</v>
       </c>
     </row>
     <row r="3">
@@ -43336,11 +43336,11 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>732</v>
+        <v>757</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>+732</t>
+          <t>+757</t>
         </is>
       </c>
     </row>
@@ -43351,11 +43351,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>722</v>
+        <v>747</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+722</t>
+          <t>+747</t>
         </is>
       </c>
     </row>
@@ -43546,11 +43546,11 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>655</v>
+        <v>680</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>+655</t>
+          <t>+680</t>
         </is>
       </c>
     </row>
@@ -43561,11 +43561,11 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>665</v>
+        <v>690</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>+665</t>
+          <t>+690</t>
         </is>
       </c>
     </row>
@@ -43621,11 +43621,11 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>663</v>
+        <v>688</v>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>+663</t>
+          <t>+688</t>
         </is>
       </c>
     </row>
@@ -43636,11 +43636,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>661</v>
+        <v>686</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+661</t>
+          <t>+686</t>
         </is>
       </c>
     </row>
@@ -43651,11 +43651,11 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>655</v>
+        <v>680</v>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>+655</t>
+          <t>+680</t>
         </is>
       </c>
     </row>
@@ -43696,11 +43696,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>976</v>
+        <v>995</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+976</t>
+          <t>+995</t>
         </is>
       </c>
     </row>
@@ -43711,11 +43711,11 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>1078</v>
+        <v>1101</v>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>+1078</t>
+          <t>+1101</t>
         </is>
       </c>
     </row>
@@ -43726,11 +43726,11 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>1088</v>
+        <v>1109</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>+1088</t>
+          <t>+1109</t>
         </is>
       </c>
     </row>
@@ -43756,11 +43756,11 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>936</v>
+        <v>953</v>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>+936</t>
+          <t>+953</t>
         </is>
       </c>
     </row>
@@ -43771,11 +43771,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>944</v>
+        <v>965</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+944</t>
+          <t>+965</t>
         </is>
       </c>
     </row>
@@ -43786,11 +43786,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>1078</v>
+        <v>1101</v>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>+1078</t>
+          <t>+1101</t>
         </is>
       </c>
     </row>
@@ -43816,11 +43816,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>1120</v>
+        <v>1143</v>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>+1120</t>
+          <t>+1143</t>
         </is>
       </c>
     </row>
@@ -43831,11 +43831,11 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>948</v>
+        <v>969</v>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>+948</t>
+          <t>+969</t>
         </is>
       </c>
     </row>
@@ -43846,11 +43846,11 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>873</v>
+        <v>896</v>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>+873</t>
+          <t>+896</t>
         </is>
       </c>
     </row>
@@ -43861,11 +43861,11 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>1110</v>
+        <v>1133</v>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>+1110</t>
+          <t>+1133</t>
         </is>
       </c>
     </row>
@@ -43876,11 +43876,11 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>972</v>
+        <v>991</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>+972</t>
+          <t>+991</t>
         </is>
       </c>
     </row>
@@ -43891,11 +43891,11 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>1128</v>
+        <v>1153</v>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>+1128</t>
+          <t>+1153</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 05:00:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -71,6 +71,7 @@
     <sheet name="2026-09-01" sheetId="63" state="visible" r:id="rId63"/>
     <sheet name="2026-09-02" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="2026-09-03" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="2026-09-04" sheetId="66" state="visible" r:id="rId66"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -44103,6 +44104,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-04 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>10206</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1605</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+772</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1597</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+836</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1623</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+843</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>+274</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>+266</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>+242</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+218</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+218</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>+226</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+198</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+188</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>+180</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>950</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>+270</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>954</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>+264</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>+25</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+246</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>935</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>+249</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>894</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>+214</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>857</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>+202</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+167</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>+313</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>+305</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>+307</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>+311</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>+307</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>+101</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>+305</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>+309</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>+38</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>+309</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>+42</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>+297</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>+115</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+115</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>+111</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+83</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+45</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>+15</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+15</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-04 05:30:24
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -44134,11 +44134,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-04 13:00:10</t>
+          <t>Timestamp: 2026-09-04 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>10206</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -72,6 +72,7 @@
     <sheet name="2026-09-02" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="2026-09-03" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="2026-09-04" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="2026-09-05" sheetId="67" state="visible" r:id="rId67"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -44992,6 +44993,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-05 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>6206</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>3646</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+2041</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>3708</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+2111</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>3677</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+2054</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>950</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>954</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>935</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>894</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>857</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-05 05:30:24
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -45023,11 +45023,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-05 13:00:09</t>
+          <t>Timestamp: 2026-09-05 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>6206</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -73,6 +73,7 @@
     <sheet name="2026-09-03" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="2026-09-04" sheetId="66" state="visible" r:id="rId66"/>
     <sheet name="2026-09-05" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="2026-09-06" sheetId="68" state="visible" r:id="rId68"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -45881,6 +45882,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-06 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>25941</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>10916</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+7270</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>10978</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+7270</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>10910</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+7233</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>4209</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+4168</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>950</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>954</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>935</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>894</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>857</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-06 05:30:22
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -45912,11 +45912,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-06 13:00:10</t>
+          <t>Timestamp: 2026-09-06 13:30:21</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>25941</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-07 05:30:24
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -46801,11 +46801,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-07 13:00:10</t>
+          <t>Timestamp: 2026-09-07 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>16855</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-08 05:32:19
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -75,6 +75,7 @@
     <sheet name="2026-09-05" sheetId="67" state="visible" r:id="rId67"/>
     <sheet name="2026-09-06" sheetId="68" state="visible" r:id="rId68"/>
     <sheet name="2026-09-07" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="2026-09-08" sheetId="70" state="visible" r:id="rId70"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -48531,6 +48532,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-08 13:32:18</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>17239</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+1249</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>16911</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+1181</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>16868</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1171</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>950</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>954</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>935</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>894</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>857</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-09 05:30:29
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -49451,11 +49451,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-09 13:00:10</t>
+          <t>Timestamp: 2026-09-09 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>8466</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -77,6 +77,7 @@
     <sheet name="2026-09-07" sheetId="69" state="visible" r:id="rId69"/>
     <sheet name="2026-09-08" sheetId="70" state="visible" r:id="rId70"/>
     <sheet name="2026-09-09" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="2026-09-10" sheetId="72" state="visible" r:id="rId72"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -50309,6 +50310,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-10 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>19989</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>19661</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>19595</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-10 05:30:29
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -50340,11 +50340,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-10 13:00:09</t>
+          <t>Timestamp: 2026-09-10 13:30:27</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>1125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-11 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -78,6 +78,7 @@
     <sheet name="2026-09-08" sheetId="70" state="visible" r:id="rId70"/>
     <sheet name="2026-09-09" sheetId="71" state="visible" r:id="rId71"/>
     <sheet name="2026-09-10" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="2026-09-11" sheetId="73" state="visible" r:id="rId73"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -51198,6 +51199,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-11 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>20364</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+375</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>20336</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+675</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>20345</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-11 05:30:23
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -51229,11 +51229,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-11 13:00:10</t>
+          <t>Timestamp: 2026-09-11 13:30:22</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>1800</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -51260,11 +51260,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>20364</v>
+        <v>20414</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>+375</t>
+          <t>+425</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -79,6 +79,7 @@
     <sheet name="2026-09-09" sheetId="71" state="visible" r:id="rId71"/>
     <sheet name="2026-09-10" sheetId="72" state="visible" r:id="rId72"/>
     <sheet name="2026-09-11" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="2026-09-12" sheetId="74" state="visible" r:id="rId74"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -52087,6 +52088,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-12 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>20414</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>20336</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>20345</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 05:30:25
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -52118,11 +52118,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-12 13:00:10</t>
+          <t>Timestamp: 2026-09-12 13:30:23</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>50</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="3">
@@ -52149,11 +52149,11 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>20414</v>
+        <v>21164</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -52164,11 +52164,11 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>20336</v>
+        <v>21086</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>
@@ -52179,11 +52179,11 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>20345</v>
+        <v>21095</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+750</t>
         </is>
       </c>
     </row>

</xml_diff>